<commit_message>
Add Atlantic Shores (VA) feedback to Q&A: mapped column + dedicated tab
Atlantic Shores Christian (VA), a current K-5 DeepRoots customer, gave
per-grade follow-up feedback (9/29/26). Added an 'Atlantic Shores' column to
the Interview Q&A matrix (mapped where their feedback aligns with our
questions) and a dedicated 'Atlantic Shores (VA) Feedback' tab with per-grade
comments and observed themes. Applied to tracker workbook + standalone Q&A.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BUC7AKNsC5W1a963Yi5JKY
</commit_message>
<xml_diff>
--- a/outreach/DeepRoots_Interview_QA.xlsx
+++ b/outreach/DeepRoots_Interview_QA.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interview Q&amp;A" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atlantic Shores (VA) Feedback" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +18,17 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="000563C1"/>
     </font>
     <font>
       <b val="1"/>
@@ -36,8 +41,16 @@
       <b val="1"/>
       <i val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00555555"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -54,6 +67,11 @@
         <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -67,18 +85,24 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -446,906 +470,1327 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D49"/>
+  <dimension ref="A1:E50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="5" customWidth="1" min="2" max="2"/>
-    <col width="55" customWidth="1" min="3" max="3"/>
-    <col width="80" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="70" customWidth="1" min="4" max="4"/>
+    <col width="70" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Section</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Q#</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Question</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Meredith Arldt — Aliso Viejo Christian School (CA) — 2026-09-24</t>
+          <t>Interview Q&amp;A (team-editable Google Sheet): https://docs.google.com/spreadsheets/d/1l05g_q15y2aV9FaNr8ABGPQdbd-yyJ0NLf2xXKy8uc4/edit</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Q#</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Question</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Meredith Arldt — Aliso Viejo Christian School (CA) — 2026-09-24</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Atlantic Shores Christian School (VA) — 9/29/26 (current K-5 use)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
           <t>Marketing &amp; Sales</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n">
+      <c r="B3" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>How does your school categorize Middle School / Junior High (5-8, 6-8, 7-8)?</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>Middle school is 6th, 7th, and 8th grade (6-8).</t>
         </is>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Marketing &amp; Sales</t>
         </is>
       </c>
-      <c r="B3" s="2" t="n">
+      <c r="B4" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>What are the primary differences between a 6th, 7th, and 8th grade student (developmentally, spiritually, emotionally)?</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>Students begin actively questioning their own faith and searching for personal identity ('why do I believe what I believe?') amid outside influences like social media. 6th graders want independence but still want the safety net of mom and dad, going back and forth. 7th graders like to push and challenge ('their own little beast'). 8th graders can get 'a little too big for their own.' Spirituality is hard at this age because it is not always tangible.</t>
         </is>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Marketing &amp; Sales</t>
         </is>
       </c>
-      <c r="B4" s="2" t="n">
+      <c r="B5" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>How do you best reach both churched and unchurched students? Is this an issue for you? What works best?</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>About 60% of the school population identifies with a church home; 40% do not. They are intentional about corporate worship (for some students it is their only weekly worship) and adopted the Teaching for Transformation framework (from CASE) two years ago, with flex projects that put faith into action. They are also rebuilding the historically broken bridge with their associated church to connect unchurched families with pastoral staff.</t>
         </is>
       </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Many unchurched students make deeper concepts hard (5th/Miriam): some don't even know who Noah is, yet the lesson teaches substitutionary death.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>Marketing &amp; Sales</t>
         </is>
       </c>
-      <c r="B5" s="2" t="n">
+      <c r="B6" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>What do you like or dislike about your current Bible curriculum?</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Currently workbook-based: Purposeful Design (Daring Deliverers), and Positive Action (Character Counts for 6th, Wise Up for 8th). All workbook-based and 'pretty dry and boring.' The goal is to keep Bible from feeling like just another academic class and to focus on students' hearts, not grade their faith.</t>
         </is>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>LIKES: love the content (3rd); Teacher Editions/Teacher Notes very helpful across grades; 3rd likes 10 days of content to choose from with room to dive deep; kids using their Bibles more (2nd); parents like it (2nd). DISLIKES: too much content for youngest grades (1st, 2nd); 'Intro to Jesus' unit too high-level (2nd + lower grades) — e.g., explaining Jesus called a 'lunatic' went over their heads; scrolling format is too much (5th); content over students' heads in 5th.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Marketing &amp; Sales</t>
         </is>
       </c>
-      <c r="B6" s="2" t="n">
+      <c r="B7" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>What elements would you like to see in it each week?</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>More reflection and personal application ('how does this resonate with you today? what do we do with this?'). Historical and cultural context so students understand the significance of events. Treat biblical figures and events as real history, not 'stories' or fairy tales.</t>
         </is>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Marketing &amp; Sales</t>
         </is>
       </c>
-      <c r="B7" s="2" t="n">
+      <c r="B8" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>What core ideals do you wish each student left your class identifying with?</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>Moving from head knowledge to heart knowledge; a real identity in Christ; applying scripture to their own lives; striving to be the best version of who God created them to be.</t>
         </is>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="E8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Marketing &amp; Sales</t>
         </is>
       </c>
-      <c r="B8" s="2" t="n">
+      <c r="B9" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>What types of resources (videos, activities, etc.) are most helpful for you as a teacher?</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>Short videos (about 1.5-5 minutes), historical family trees, Bible timelines, primary documents, original-language (Greek/Hebrew) references, and cultural/archaeological references (e.g., an archaeological Bible). Note: curating and vetting these is the most time-consuming part for teachers, so ready-made, vetted resources would help most.</t>
         </is>
       </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Teacher Editions / Teacher Notes (TEs/TNs) are the most helpful resource (1st printed &amp; uses TNs; 4th teaches from TNs; 3rd: TE super helpful with so much content).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>Editorial</t>
         </is>
       </c>
-      <c r="B9" s="2" t="n">
+      <c r="B10" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>How many minutes can students pay attention to teaching, reading, discussion, activities?</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>Lecture/teaching is kept to 15-20 minutes max before moving into discussion. A typical rhythm is a ~5-minute intro/review, a 10-15 minute lesson, then discussion. Class is mostly discussion-based; some reading.</t>
         </is>
       </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="E10" s="3" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>Editorial</t>
         </is>
       </c>
-      <c r="B10" s="2" t="n">
+      <c r="B11" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>What kind of engagements do students enjoy most (by grade)?</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D11" s="3" t="inlineStr">
         <is>
           <t>Discussion-based work and things they can relate to (real-world video, relatable visuals), partner work, and interactive questions. Discussion is the biggest draw across middle school.</t>
         </is>
       </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="E11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>Editorial</t>
         </is>
       </c>
-      <c r="B11" s="2" t="n">
+      <c r="B12" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>How do you use screens and technology in your classroom?</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D12" s="3" t="inlineStr">
         <is>
           <t>Google Classroom is the platform; laptops are provided but screen time is intentionally limited (parents appreciate this). Currently projection-based; installing BenQ interactive smartboards by January (grant-funded), with teacher training.</t>
         </is>
       </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>K teachers project and teach from the Teacher site; rooms don't have 2 devices (one-device teaching). Some early tech issues, now mostly worked through (possibly local).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>Editorial</t>
         </is>
       </c>
-      <c r="B12" s="2" t="n">
+      <c r="B13" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>What questions/issues do you see students wrestling with (by grade)?</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D13" s="3" t="inlineStr">
         <is>
           <t>Reconciling 'what my parents taught me' with 'what do I actually believe'; identity in Christ versus societal pressure and peer acceptance; influence of social media; and nominal Christianity ('Christian in name only') where students know the Sunday-school answers but haven't moved it from head to heart.</t>
         </is>
       </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="E13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>Editorial</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n">
+      <c r="B14" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>Would you use an end-of-year project students prepare as a group? (Yes/No/Maybe)</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D14" s="3" t="inlineStr">
         <is>
           <t>Maybe / planning to: no big end-of-year project currently (some project element in the final exam), but she wants to add an 8th-grade capstone project tied to Teaching for Transformation as students move into high school.</t>
         </is>
       </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="E14" s="3" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>Editorial</t>
         </is>
       </c>
-      <c r="B14" s="2" t="n">
+      <c r="B15" s="3" t="n">
         <v>13</v>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
         <is>
           <t>What tools have helped with parent engagement?</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D15" s="3" t="inlineStr">
         <is>
           <t>A required number of service hours per semester draws families in (parents help get middle schoolers to service projects and often serve together around a shared passion). Also communicating the grading approach clearly at tours, and rebuilding the church connection.</t>
         </is>
       </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="E15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>Editorial</t>
         </is>
       </c>
-      <c r="B15" s="2" t="n">
+      <c r="B16" s="3" t="n">
         <v>14</v>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C16" s="3" t="inlineStr">
         <is>
           <t>What is your school's homework policy (by grade)?</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="D16" s="3" t="inlineStr">
         <is>
           <t>Not directly addressed in this interview.</t>
         </is>
       </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="E16" s="3" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>Production</t>
         </is>
       </c>
-      <c r="B16" s="2" t="n">
+      <c r="B17" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr">
         <is>
           <t>What videos do you currently show, and how do you use them?</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="D17" s="3" t="inlineStr">
         <is>
           <t>Right Now Media and YouTube clips; one recurring activity has students take a Christian song and build a Bible-study object lesson around it. All videos are vetted by the teacher/administrator before showing.</t>
         </is>
       </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="E17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>Production</t>
         </is>
       </c>
-      <c r="B17" s="2" t="n">
+      <c r="B18" s="3" t="n">
         <v>16</v>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
         <is>
           <t>What length of video is most engaging? (30s-1m / 1-2m / 2-3m / 3m+)</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="D18" s="3" t="inlineStr">
         <is>
           <t>Short: generally no more than ~5 minutes, with song-based clips around 1.5-2 minutes, to match attention spans.</t>
         </is>
       </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>Songs feel too juvenile for upper elementary (5th); students prefer known 'brand name' worship songs (e.g., Forrest Frank).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>Production</t>
         </is>
       </c>
-      <c r="B18" s="2" t="n">
+      <c r="B19" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="C19" s="3" t="inlineStr">
         <is>
           <t>What types of visuals are most effective for middle schoolers?</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="D19" s="3" t="inlineStr">
         <is>
           <t>Real-life, relatable people (not cartoons); charts and graphs, family trees, timelines, historical artwork/renderings, primary documents, archaeological images, and maps. She favors visuals students can see themselves in.</t>
         </is>
       </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Classical/fine-art images didn't land — kids didn't like or understand the classical art in the Intro to Jesus unit (2nd).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
         <is>
           <t>Production</t>
         </is>
       </c>
-      <c r="B19" s="2" t="n">
+      <c r="B20" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="C20" s="3" t="inlineStr">
         <is>
           <t>Do you prefer digital assessments or printables?</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="D20" s="3" t="inlineStr">
         <is>
           <t>Leaning digital: with the move to Google Classroom (year two), they are less tied to printables; students interact with lessons and submit work electronically.</t>
         </is>
       </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Tried the online tests; could work, but strongly dislike the auto-grader marking off for spelling (3rd, 5th) — fixing every grade defeats the time savings. 1st still prints/uses paper TNs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>Production</t>
         </is>
       </c>
-      <c r="B20" s="2" t="n">
+      <c r="B21" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="C21" s="3" t="inlineStr">
         <is>
           <t>What balance between text and visuals on a typical student page?</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="D21" s="3" t="inlineStr">
         <is>
           <t>A balanced mix of text and visuals (stated explicitly). As a former English teacher she values the written word and dissecting scripture, and also sees strong value in relatable visuals.</t>
         </is>
       </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="E21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>Production</t>
         </is>
       </c>
-      <c r="B21" s="2" t="n">
+      <c r="B22" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C22" s="3" t="inlineStr">
         <is>
           <t>What would make a middle schooler pick up the curriculum rather than see it as 'just another textbook'?</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="D22" s="3" t="inlineStr">
         <is>
           <t>Relatable, real-world visuals plus the teacher's presentation and enthusiasm. Avoiding dry, workbook-feeling material; keeping it discussion-driven and engaging. The teacher's delivery makes a big difference.</t>
         </is>
       </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
+      <c r="E22" s="3" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>Production</t>
         </is>
       </c>
-      <c r="B22" s="2" t="n">
+      <c r="B23" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="C22" s="2" t="inlineStr">
+      <c r="C23" s="3" t="inlineStr">
         <is>
           <t>Are you limited by the amount of material you can print?</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr">
+      <c r="D23" s="3" t="inlineStr">
         <is>
           <t>Not really limited. Teachers are asked to reduce paper where possible, but the school is well-resourced (budget, laptops, Google Classroom) and prints less in middle school than in elementary.</t>
         </is>
       </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+      <c r="E23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
         <is>
           <t>Production</t>
         </is>
       </c>
-      <c r="B23" s="2" t="n">
+      <c r="B24" s="3" t="n">
         <v>22</v>
       </c>
-      <c r="C23" s="2" t="inlineStr">
+      <c r="C24" s="3" t="inlineStr">
         <is>
           <t>If an activity required non-standard supplies (e.g., food), would the school provide funds or would the teacher?</t>
         </is>
       </c>
-      <c r="D23" s="2" t="inlineStr">
+      <c r="D24" s="3" t="inlineStr">
         <is>
           <t>The school provides funds. Teachers have money set aside each year for curriculum and supplies; she orders what they need and tracks spending. In nine years she has never told a teacher 'no' to a resource request.</t>
         </is>
       </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
+      <c r="E24" s="3" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>Additional (Extra Time)</t>
         </is>
       </c>
-      <c r="B24" s="2" t="n">
+      <c r="B25" s="3" t="n">
         <v>23</v>
       </c>
-      <c r="C24" s="2" t="inlineStr">
+      <c r="C25" s="3" t="inlineStr">
         <is>
           <t>After 20 minutes of essential material, how much additional time would you like optional material to fill?</t>
         </is>
       </c>
-      <c r="D24" s="2" t="inlineStr">
+      <c r="D25" s="3" t="inlineStr">
         <is>
           <t>Since class is mostly discussion-based, if the core lesson runs about 20 minutes, guided discussion can take the majority of the remaining class time.</t>
         </is>
       </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
+      <c r="E25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>Additional (Extra Time)</t>
         </is>
       </c>
-      <c r="B25" s="2" t="n">
+      <c r="B26" s="3" t="n">
         <v>24</v>
       </c>
-      <c r="C25" s="2" t="inlineStr">
+      <c r="C26" s="3" t="inlineStr">
         <is>
           <t>Would you be interested in a multi-subject Timeline centered on Bible events (with optional Empires, Literature, Music/Arts, People, Inventions, clickable summaries and media)?</t>
         </is>
       </c>
-      <c r="D25" s="2" t="inlineStr">
+      <c r="D26" s="3" t="inlineStr">
         <is>
           <t>Not asked verbatim, but very likely yes: she strongly values timelines (built family trees and displayed a Bible timeline so students could see how events were organized) and finds chronology a real challenge for students.</t>
         </is>
       </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="E26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>Additional (Extra Time)</t>
         </is>
       </c>
-      <c r="B26" s="2" t="n">
+      <c r="B27" s="3" t="n">
         <v>25</v>
       </c>
-      <c r="C26" s="2" t="inlineStr">
+      <c r="C27" s="3" t="inlineStr">
         <is>
           <t>Approximately how many minutes of screen time/technology would you permit in Bible class?</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="D27" s="3" t="inlineStr">
         <is>
           <t>No specific number given; screen time is intentionally limited and balanced across the day rather than used continuously.</t>
         </is>
       </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
+      <c r="E27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>Additional (Extra Time)</t>
         </is>
       </c>
-      <c r="B27" s="2" t="n">
+      <c r="B28" s="3" t="n">
         <v>26</v>
       </c>
-      <c r="C27" s="2" t="inlineStr">
+      <c r="C28" s="3" t="inlineStr">
         <is>
           <t>What tools have you found most effective for encouraging Bible reading at home?</t>
         </is>
       </c>
-      <c r="D27" s="2" t="inlineStr">
+      <c r="D28" s="3" t="inlineStr">
         <is>
           <t>Not directly addressed in this interview.</t>
         </is>
       </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>Ask: memory-verse SONGS with HAND MOTIONS (raised by 3rd &amp; 4th; 3rd finds her own now). Hand motions aid retention even MS/HS per admin Melissa (older grades without the song).</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>Additional (Extra Time)</t>
         </is>
       </c>
-      <c r="B28" s="2" t="n">
+      <c r="B29" s="3" t="n">
         <v>27</v>
       </c>
-      <c r="C28" s="2" t="inlineStr">
+      <c r="C29" s="3" t="inlineStr">
         <is>
           <t>If the curriculum offered an optional human sexuality unit, how would you use it?</t>
         </is>
       </c>
-      <c r="D28" s="2" t="inlineStr">
+      <c r="D29" s="3" t="inlineStr">
         <is>
           <t>They would not teach it at school; human sexuality is treated as a parent matter and left entirely to parents. They already skip such lessons (e.g., a unit 10 in the 8th-grade book) and coordinate with teachers to do so.</t>
         </is>
       </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
+      <c r="E29" s="3" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
         <is>
           <t>Additional (Extra Time)</t>
         </is>
       </c>
-      <c r="B29" s="2" t="n">
+      <c r="B30" s="3" t="n">
         <v>28</v>
       </c>
-      <c r="C29" s="2" t="inlineStr">
+      <c r="C30" s="3" t="inlineStr">
         <is>
           <t>Would you be interested in a separate Logic course, primarily taught through videos and reinforced with worksheets?</t>
         </is>
       </c>
-      <c r="D29" s="2" t="inlineStr">
+      <c r="D30" s="3" t="inlineStr">
         <is>
           <t>Yes / interested, but video-based delivery matters: teachers would likely need videos of someone presenting the material to feel comfortable, rather than lecture- or worksheet-only.</t>
         </is>
       </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
+      <c r="E30" s="3" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>Additional (Extra Time)</t>
         </is>
       </c>
-      <c r="B30" s="2" t="n">
+      <c r="B31" s="3" t="n">
         <v>29</v>
       </c>
-      <c r="C30" s="2" t="inlineStr">
+      <c r="C31" s="3" t="inlineStr">
         <is>
           <t>With 5 minutes of independent reading + 15 minutes of teaching/engagement, would you use optional deeper material? What engagements?</t>
         </is>
       </c>
-      <c r="D30" s="2" t="inlineStr">
+      <c r="D31" s="3" t="inlineStr">
         <is>
           <t>Yes. She likes a ~5-minute reflection/journaling opening, then a lesson (~20 minutes total), then discussion. Engagements: discussion, journaling/reflection, returning to scripture, and partner work.</t>
         </is>
       </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
+      <c r="E31" s="3" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
         <is>
           <t>Additional (Extra Time)</t>
         </is>
       </c>
-      <c r="B31" s="2" t="n">
+      <c r="B32" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="C31" s="2" t="inlineStr">
+      <c r="C32" s="3" t="inlineStr">
         <is>
           <t>How important is handling a printable reference book (Course Pack) vs. an online reference?</t>
         </is>
       </c>
-      <c r="D31" s="2" t="inlineStr">
+      <c r="D32" s="3" t="inlineStr">
         <is>
           <t>Mixed, leaning digital with the Google Classroom move, but she still values the written word and dissecting scripture, so there is real value in a text reference for some students.</t>
         </is>
       </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
+      <c r="E32" s="3" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
         <is>
           <t>Additional (Extra Time)</t>
         </is>
       </c>
-      <c r="B32" s="2" t="n">
+      <c r="B33" s="3" t="n">
         <v>31</v>
       </c>
-      <c r="C32" s="2" t="inlineStr">
+      <c r="C33" s="3" t="inlineStr">
         <is>
           <t>Individual quiet work vs. group activity: which do you prefer? Which do students prefer?</t>
         </is>
       </c>
-      <c r="D32" s="2" t="inlineStr">
+      <c r="D33" s="3" t="inlineStr">
         <is>
           <t>Group/discussion for both. Independent Bible study is hard for middle schoolers because they are not yet fluent in scripture, so guided, discussion-heavy classes are essential.</t>
         </is>
       </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
+      <c r="E33" s="3" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
         <is>
           <t>Additional (Extra Time)</t>
         </is>
       </c>
-      <c r="B33" s="2" t="n">
+      <c r="B34" s="3" t="n">
         <v>32</v>
       </c>
-      <c r="C33" s="2" t="inlineStr">
+      <c r="C34" s="3" t="inlineStr">
         <is>
           <t>As a teacher, what does your ideal Bible lesson look like?</t>
         </is>
       </c>
-      <c r="D33" s="2" t="inlineStr">
+      <c r="D34" s="3" t="inlineStr">
         <is>
           <t>A short intro/review (~5 min), a focused lesson (~15-20 min), then discussion and partner work, woven with historical/cultural context and personal reflection/application, kept moving so students stay engaged.</t>
         </is>
       </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
+      <c r="E34" s="3" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
         <is>
           <t>Additional (Extra Time)</t>
         </is>
       </c>
-      <c r="B34" s="2" t="n">
+      <c r="B35" s="3" t="n">
         <v>33</v>
       </c>
-      <c r="C34" s="2" t="inlineStr">
+      <c r="C35" s="3" t="inlineStr">
         <is>
           <t>How do you measure the success of a curriculum?</t>
         </is>
       </c>
-      <c r="D34" s="2" t="inlineStr">
+      <c r="D35" s="3" t="inlineStr">
         <is>
           <t>Students being able to apply scripture to their own lives. Her tests always ended with an open-ended prompt: 'write an example of how this applies to your life,' which showed movement from head knowledge to heart knowledge.</t>
         </is>
       </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>Auto-graded online assessments promising but the spelling penalty undermines them (see Q18). Kids using Bibles more is seen as a win (2nd).</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
         <is>
           <t>Additional (Extra Time)</t>
         </is>
       </c>
-      <c r="B35" s="2" t="n">
+      <c r="B36" s="3" t="n">
         <v>34</v>
       </c>
-      <c r="C35" s="2" t="inlineStr">
+      <c r="C36" s="3" t="inlineStr">
         <is>
           <t>Are there visual styles/trends/design approaches that would NOT work well?</t>
         </is>
       </c>
-      <c r="D35" s="2" t="inlineStr">
+      <c r="D36" s="3" t="inlineStr">
         <is>
           <t>Younger, cartoon-style depictions of people. Middle schoolers are moving away from cartoons and want to see real people they can relate to.</t>
         </is>
       </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>Avoid classical/fine-art visuals for this age (didn't connect); avoid overly juvenile song styles for upper elementary; scrolling-heavy digital layout is a negative (5th).</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
         <is>
           <t>Additional (Extra Time)</t>
         </is>
       </c>
-      <c r="B36" s="2" t="n">
+      <c r="B37" s="3" t="n">
         <v>35</v>
       </c>
-      <c r="C36" s="2" t="inlineStr">
+      <c r="C37" s="3" t="inlineStr">
         <is>
           <t>What short videos would be helpful to supplement your teaching?</t>
         </is>
       </c>
-      <c r="D36" s="2" t="inlineStr">
+      <c r="D37" s="3" t="inlineStr">
         <is>
           <t>Real-world application videos most of all, plus videos that hit the key idea and introduce/give context to the subject; relatable real-world visuals resonate most.</t>
         </is>
       </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
+      <c r="E37" s="3" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
         <is>
           <t>Additional (Extra Time)</t>
         </is>
       </c>
-      <c r="B37" s="2" t="n">
+      <c r="B38" s="3" t="n">
         <v>36</v>
       </c>
-      <c r="C37" s="2" t="inlineStr">
+      <c r="C38" s="3" t="inlineStr">
         <is>
           <t>On a scale of 1-10, how would you rate role-play activities for engagement?</t>
         </is>
       </c>
-      <c r="D37" s="2" t="inlineStr">
+      <c r="D38" s="3" t="inlineStr">
         <is>
           <t>Low. Middle schoolers often dislike being put on the spot, especially about personal faith. Fine as an optional tool if a class is open to it, but not something to use consistently.</t>
         </is>
       </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr">
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>Role play rates HIGH here — kids love it, Good Samaritan role play a standout (3rd). NOTE: opposite of the middle-school signal (rated low there).</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
         <is>
           <t>Additional (Extra Time)</t>
         </is>
       </c>
-      <c r="B38" s="2" t="n">
+      <c r="B39" s="3" t="n">
         <v>37</v>
       </c>
-      <c r="C38" s="2" t="inlineStr">
+      <c r="C39" s="3" t="inlineStr">
         <is>
           <t>What elements of a Bible curriculum do you NOT prefer?</t>
         </is>
       </c>
-      <c r="D38" s="2" t="inlineStr">
+      <c r="D39" s="3" t="inlineStr">
         <is>
           <t>Dry, boring material; 'just words on a page' or 'the next lesson in the workbook,' which brings the wrong attitude into class.</t>
         </is>
       </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="inlineStr">
+      <c r="E39" s="3" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
         <is>
           <t>Additional (Extra Time)</t>
         </is>
       </c>
-      <c r="B39" s="2" t="n">
+      <c r="B40" s="3" t="n">
         <v>38</v>
       </c>
-      <c r="C39" s="2" t="inlineStr">
+      <c r="C40" s="3" t="inlineStr">
         <is>
           <t>What gets and holds your students' attention in Bible class?</t>
         </is>
       </c>
-      <c r="D39" s="2" t="inlineStr">
+      <c r="D40" s="3" t="inlineStr">
         <is>
           <t>Engaging discussion and debate, relatable real-world visuals and video, the teacher's enthusiasm and presentation, and variety that keeps the lesson moving.</t>
         </is>
       </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr">
+      <c r="E40" s="3" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
         <is>
           <t>Additional (Extra Time)</t>
         </is>
       </c>
-      <c r="B40" s="2" t="n">
+      <c r="B41" s="3" t="n">
         <v>39</v>
       </c>
-      <c r="C40" s="2" t="inlineStr">
+      <c r="C41" s="3" t="inlineStr">
         <is>
           <t>What would a middle school Bible curriculum look like that is easy to teach and impactful?</t>
         </is>
       </c>
-      <c r="D40" s="2" t="inlineStr">
+      <c r="D41" s="3" t="inlineStr">
         <is>
           <t>The same depth and teacher resources DeepRoots provides for elementary, but with a different presentation model for middle school: not dry, relatable visuals, discussion-driven, rich in reflection/application and historical/cultural context, with enough ready-made resources that teachers are not building and vetting everything themselves. (They currently use DeepRoots for grades 3-5.)</t>
         </is>
       </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="2" t="inlineStr"/>
-      <c r="B41" s="2" t="inlineStr"/>
-      <c r="C41" s="2" t="inlineStr"/>
-      <c r="D41" s="2" t="inlineStr"/>
+      <c r="E41" s="3" t="inlineStr"/>
     </row>
     <row r="42">
-      <c r="A42" s="3" t="inlineStr">
-        <is>
-          <t>DEEPROOTS TEAM TAKEAWAYS — what we got out of this interview (said or unsaid)</t>
-        </is>
-      </c>
+      <c r="A42" s="3" t="inlineStr"/>
       <c r="B42" s="3" t="inlineStr"/>
       <c r="C42" s="3" t="inlineStr"/>
       <c r="D42" s="3" t="inlineStr"/>
+      <c r="E42" s="3" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" s="4" t="inlineStr"/>
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>DEEPROOTS TEAM TAKEAWAYS — what we got out of each interview (said or unsaid)</t>
+        </is>
+      </c>
       <c r="B43" s="4" t="inlineStr"/>
-      <c r="C43" s="4" t="inlineStr">
+      <c r="C43" s="4" t="inlineStr"/>
+      <c r="D43" s="4" t="inlineStr"/>
+      <c r="E43" s="4" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr"/>
+      <c r="B44" s="5" t="inlineStr"/>
+      <c r="C44" s="5" t="inlineStr">
         <is>
           <t>Team member</t>
         </is>
       </c>
-      <c r="D43" s="4" t="inlineStr">
-        <is>
-          <t>Your takeaways / observations</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="2" t="inlineStr"/>
-      <c r="B44" s="2" t="inlineStr"/>
-      <c r="C44" s="2" t="inlineStr">
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>Meredith Arldt — Aliso Viejo Christian School (CA) — 2026-09-24</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>Atlantic Shores Christian School (VA) — 9/29/26 (current K-5 use)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr"/>
+      <c r="B45" s="3" t="inlineStr"/>
+      <c r="C45" s="3" t="inlineStr">
         <is>
           <t>Troy Winkler</t>
         </is>
       </c>
-      <c r="D44" s="2" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="2" t="inlineStr"/>
-      <c r="B45" s="2" t="inlineStr"/>
-      <c r="C45" s="2" t="inlineStr">
+      <c r="D45" s="3" t="inlineStr"/>
+      <c r="E45" s="3" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr"/>
+      <c r="B46" s="3" t="inlineStr"/>
+      <c r="C46" s="3" t="inlineStr">
         <is>
           <t>Pat Williamson</t>
         </is>
       </c>
-      <c r="D45" s="2" t="inlineStr"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="inlineStr"/>
-      <c r="B46" s="2" t="inlineStr"/>
-      <c r="C46" s="2" t="inlineStr">
+      <c r="D46" s="3" t="inlineStr"/>
+      <c r="E46" s="3" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr"/>
+      <c r="B47" s="3" t="inlineStr"/>
+      <c r="C47" s="3" t="inlineStr">
         <is>
           <t>Nancy Wood</t>
         </is>
       </c>
-      <c r="D46" s="2" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="2" t="inlineStr"/>
-      <c r="B47" s="2" t="inlineStr"/>
-      <c r="C47" s="2" t="inlineStr">
+      <c r="D47" s="3" t="inlineStr"/>
+      <c r="E47" s="3" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr"/>
+      <c r="B48" s="3" t="inlineStr"/>
+      <c r="C48" s="3" t="inlineStr">
         <is>
           <t>Tammy Plett</t>
         </is>
       </c>
-      <c r="D47" s="2" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="inlineStr"/>
-      <c r="B48" s="2" t="inlineStr"/>
-      <c r="C48" s="2" t="inlineStr">
+      <c r="D48" s="3" t="inlineStr"/>
+      <c r="E48" s="3" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr"/>
+      <c r="B49" s="3" t="inlineStr"/>
+      <c r="C49" s="3" t="inlineStr">
         <is>
           <t>Lisa Van Vlear</t>
         </is>
       </c>
-      <c r="D48" s="2" t="inlineStr"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="2" t="inlineStr"/>
-      <c r="B49" s="2" t="inlineStr"/>
-      <c r="C49" s="2" t="inlineStr">
+      <c r="D49" s="3" t="inlineStr"/>
+      <c r="E49" s="3" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr"/>
+      <c r="B50" s="3" t="inlineStr"/>
+      <c r="C50" s="3" t="inlineStr">
         <is>
           <t>Overall / key takeaways for the curriculum</t>
         </is>
       </c>
-      <c r="D49" s="2" t="inlineStr"/>
+      <c r="D50" s="3" t="inlineStr"/>
+      <c r="E50" s="3" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="95" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Atlantic Shores Christian School — Virginia</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>Follow-up meeting 9/29/26  |  ~$11,000 account  |  Current DeepRoots K-5 customer</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Attendees: Admin Melissa Wetzel + grade-level Mentor teachers (K-5). Each grade has 3 teachers + 1 mentor; only mentors attended.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Grade</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Teacher (Mentor)</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Feedback</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Rebecca</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>All going pretty good; some early tech issues that seem worked through (maybe on their end). All K teachers project/teach from the Teacher site; rooms don't have 2 devices, so one-device teaching. Going OK this way.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Kristal</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Going well. Printed the TNs for all 1st teachers and using them. Kids too young to memorize two verses, so they use only one. Too much content for this age, but the TEs are very helpful.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>2nd</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Jessica</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Going good; parents also like the curriculum (unsure how many use the PEP). 'Intro to Jesus' unit too high-level (lower grades agreed); kids didn't like/understand the classical art; too much time explaining things like Jesus called a 'lunatic' (kids don't get it). Likes that students use their Bibles much more now.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>3rd</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Natalie</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Going well. Toggling between Student World (SW) and Teacher World (TW) is sometimes too much/confusing. Loves the content; kids love Role Play (esp. Good Samaritan). TE super helpful with so much content; loves having 10 days of content to choose from and time to dive deep. Wishes for Bible-verse songs with hand motions (finds her own now). Tried online tests — could work, but dislikes marking off for spelling.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>4th</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Robin</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Enjoying it; uses the TNs when teaching. Really wants hand motions for the memory verses — they help upper grades learn verses. (Melissa: MS/HS use hand motions for retention too, just without a song.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>5th</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Miriam</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>OK, but dislikes the scrolling format (too much to scroll). Dislikes online assessments marking off for spelling (not worth re-adjusting grades; defeats the auto-grade time savings). Content over their heads; many unchurched students make it hard (some don't know who Noah is, yet teaching substitutionary death). Songs too juvenile; prefers known 'brand name' songs (e.g., Forrest Frank).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Melissa Wetzel</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Thought things were going well; hadn't heard negative feedback beforehand; wanted to hear from the mentors. Confirmed MS/HS use hand motions for verse retention.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="n"/>
+      <c r="B13" s="3" t="n"/>
+      <c r="C13" s="3" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>OBSERVED THEMES (from the notes)</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr"/>
+      <c r="C14" s="8" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr"/>
+      <c r="B15" s="3" t="inlineStr"/>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Strong, repeated demand for memory-verse SONGS with HAND MOTIONS (3rd, 4th; admin confirms value through HS).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr"/>
+      <c r="B16" s="3" t="inlineStr"/>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Online auto-grading is wanted, but marking off for spelling is a dealbreaker — make spelling leniency configurable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr"/>
+      <c r="B17" s="3" t="inlineStr"/>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Content level/pacing runs high for younger grades ('Intro to Jesus', classical art) — add grade-appropriate scaffolding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr"/>
+      <c r="B18" s="3" t="inlineStr"/>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Role play is a hit in elementary (Good Samaritan) — opposite of the middle-school signal; keep it age-targeted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr"/>
+      <c r="B19" s="3" t="inlineStr"/>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Digital UX: reduce scrolling; the SW/TW toggle can confuse teachers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr"/>
+      <c r="B20" s="3" t="inlineStr"/>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Upper-elementary song style should avoid a juvenile tone; lean on recognizable artists.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr"/>
+      <c r="B21" s="3" t="inlineStr"/>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Many unchurched students: don't assume base Bible knowledge (some don't know who Noah is).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="n"/>
+      <c r="B22" s="3" t="n"/>
+      <c r="C22" s="3" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>DEEPROOTS TEAM TAKEAWAYS (add yours)</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr"/>
+      <c r="C23" s="4" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr"/>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Troy Winkler</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr"/>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Pat Williamson</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr"/>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Nancy Wood</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr"/>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Tammy Plett</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr"/>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Lisa Van Vlear</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add Will Weaver interview: doc + Will column in Q&A; repoint tracker to new shared sheet
Will Weaver (Des Moines Christian, admin) interview processed from Gemini
notes + transcript. Added Will column to the Q&A matrix (now Meredith +
Atlantic Shores + Will), rebuilt local workbooks, created his interview doc
and a refreshed shared Q&A sheet (all three + Atlantic feedback), and
repointed tracker links; marked Will's interview completed.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BUC7AKNsC5W1a963Yi5JKY
</commit_message>
<xml_diff>
--- a/outreach/DeepRoots_Interview_QA.xlsx
+++ b/outreach/DeepRoots_Interview_QA.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,7 +28,7 @@
     </font>
     <font>
       <i val="1"/>
-      <color rgb="000563C1"/>
+      <color rgb="00555555"/>
     </font>
     <font>
       <b val="1"/>
@@ -44,10 +44,6 @@
     <font>
       <b val="1"/>
       <sz val="13"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <color rgb="00555555"/>
     </font>
   </fonts>
   <fills count="5">
@@ -85,7 +81,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -101,7 +97,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -470,20 +465,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E50"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
     <col width="5" customWidth="1" min="2" max="2"/>
-    <col width="52" customWidth="1" min="3" max="3"/>
-    <col width="70" customWidth="1" min="4" max="4"/>
-    <col width="70" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="58" customWidth="1" min="4" max="4"/>
+    <col width="58" customWidth="1" min="5" max="5"/>
+    <col width="58" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Interview Q&amp;A (team-editable Google Sheet): https://docs.google.com/spreadsheets/d/1l05g_q15y2aV9FaNr8ABGPQdbd-yyJ0NLf2xXKy8uc4/edit</t>
+          <t>Interview Q&amp;A — DeepRoots Middle-School Bible Curriculum market research. Columns = interviewees. Bottom: DeepRoots team takeaways, then Atlantic Shores per-grade feedback.</t>
         </is>
       </c>
     </row>
@@ -505,12 +501,17 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Meredith Arldt — Aliso Viejo Christian School (CA) — 2026-09-24</t>
+          <t>Meredith Arldt — Aliso Viejo Christian School (CA) — teacher/admin — 2026-09-24</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Atlantic Shores Christian School (VA) — 9/29/26 (current K-5 use)</t>
+          <t>Atlantic Shores Christian School (VA) — current K-5 use — 9/29/26</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Will Weaver — Des Moines Christian School (IA) — Head of Spiritual Formation (admin) — 2026-09-30</t>
         </is>
       </c>
     </row>
@@ -534,6 +535,11 @@
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr"/>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Currently MS = 6-8 (this year 68 students, next year 58). Next year pulling 5th grade into a unified 5-8 middle school; 5th treated as the 'logic phase.'</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -555,6 +561,11 @@
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr"/>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>5th graders have more in common with 7th/8th than K-1; ready for inquiry ('why' questions), not just content. Discussion capacity grows: ~20 min in 6th, 25-30 min in 7th-8th as they take ownership. Student certainty on absolute moral truth tends to DECREASE in higher grades.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -580,6 +591,11 @@
           <t>Many unchurched students make deeper concepts hard (5th/Miriam): some don't even know who Noah is, yet the lesson teaches substitutionary death.</t>
         </is>
       </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Covenantal school, ~1,650 students; long-time DeepRoots elementary user (~40 students). Program goal across EE-12: 'resilient disciples' who own their faith.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -602,7 +618,12 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>LIKES: love the content (3rd); Teacher Editions/Teacher Notes very helpful across grades; 3rd likes 10 days of content to choose from with room to dive deep; kids using their Bibles more (2nd); parents like it (2nd). DISLIKES: too much content for youngest grades (1st, 2nd); 'Intro to Jesus' unit too high-level (2nd + lower grades) — e.g., explaining Jesus called a 'lunatic' went over their heads; scrolling format is too much (5th); content over students' heads in 5th.</t>
+          <t>LIKES: love the content (3rd); Teacher Editions/Teacher Notes very helpful across grades; 3rd likes 10 days of content to choose from with room to dive deep; kids using their Bibles more (2nd); parents like it (2nd). DISLIKES: too much content for youngest grades (1st, 2nd); 'Intro to Jesus' unit too high-level (2nd + lower grades); scrolling format too much (5th); content over students' heads in 5th.</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>MS Bible progression: 6th = Old Testament survey, 7th = New Testament survey, 8th = intro to worldview, apologetics &amp; ethics. Uses the Casket-Empty(-Open) mnemonic across 6/7/8 to anchor stories into scripture's meta-narrative. Long-time DeepRoots user in elementary.</t>
         </is>
       </c>
     </row>
@@ -626,6 +647,11 @@
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr"/>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Discussion-based (Harkness) conversations, growing in length by grade; family devotionals; common assessments across 6-8 enabling reteach + extension; a mandatory 5-10 min reading period at the start of every core class.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -647,6 +673,11 @@
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr"/>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>'Resilient disciples' who take ownership of their faith — able to take doctrine apart and put it back together, and articulate not just what it says but 'where it sits in your soul,' rather than regurgitate content for a grade.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -669,7 +700,12 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Teacher Editions / Teacher Notes (TEs/TNs) are the most helpful resource (1st printed &amp; uses TNs; 4th teaches from TNs; 3rd: TE super helpful with so much content).</t>
+          <t>Teacher Editions / Teacher Notes (TEs/TNs) most helpful (1st printed &amp; uses TNs; 4th teaches from TNs; 3rd: TE super helpful with so much content).</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Strong interest in usable Logic materials (DeepRoots offered optional 7th/8th logic sets). Casket-Empty mnemonic; Wheaton global student assessment 3x/year for worldview metrics.</t>
         </is>
       </c>
     </row>
@@ -693,6 +729,11 @@
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr"/>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Targets: direct instruction 20 min or less (ideally ~17); media 3-7 min; student activities 15-20 min before attention drops. Discussions: ~20 min (6th), 25-30 min (7th-8th).</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -714,6 +755,11 @@
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr"/>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Harkness roundtable discussions (even mixed 6-8 for high performers), independent projects/research, and presentations, especially in 8th.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -736,7 +782,12 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>K teachers project and teach from the Teacher site; rooms don't have 2 devices (one-device teaching). Some early tech issues, now mostly worked through (possibly local).</t>
+          <t>K teachers project/teach from the Teacher site; rooms lack 2 devices (one-device teaching); early tech issues now mostly worked through.</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Phone-free K-12; deliberately scaling back student Chromebook use (screens promote skimming/distraction). Willing to raise tuition for paper; challenges teachers to justify student tech vs. checking a box. Distinguishes beneficial teacher-side tech from student-side.</t>
         </is>
       </c>
     </row>
@@ -760,6 +811,11 @@
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr"/>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Absolute moral truth and identity are the major recurring struggles (certainty on moral truth drops in higher grades). 8th apologetics/ethics topics: reliability of scripture, pornography, social media, sexuality (problem of evil/pain reserved for high school).</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -781,6 +837,11 @@
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr"/>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>8th grade uses independent projects/research and roundtable presentations rather than a single end-of-year group project.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -802,6 +863,11 @@
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr"/>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Family devotionals as completion-based assignments; spiritual-growth assessments (student + parents + trusted adults); 7-10 min one-on-one growth conversations with EVERY middle schooler (~115/grade).</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -823,6 +889,11 @@
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr"/>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Not directly addressed (family devotionals are completion-based home assignments).</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -844,6 +915,11 @@
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr"/>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Not directly addressed (media engagement targeted to 3-7 min).</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -866,7 +942,12 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>Songs feel too juvenile for upper elementary (5th); students prefer known 'brand name' worship songs (e.g., Forrest Frank).</t>
+          <t>Songs feel too juvenile for upper elementary (5th); prefer known 'brand name' worship songs (e.g., Forrest Frank).</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>Media/video engagement targeted at 3-7 minutes.</t>
         </is>
       </c>
     </row>
@@ -891,7 +972,12 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>Classical/fine-art images didn't land — kids didn't like or understand the classical art in the Intro to Jesus unit (2nd).</t>
+          <t>Classical/fine-art images didn't land — kids didn't like/understand the classical art in the Intro to Jesus unit (2nd).</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Not directly addressed. (High-school apologetics leans on beauty/aesthetics — the 'argument from beauty.')</t>
         </is>
       </c>
     </row>
@@ -916,7 +1002,12 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>Tried the online tests; could work, but strongly dislike the auto-grader marking off for spelling (3rd, 5th) — fixing every grade defeats the time savings. 1st still prints/uses paper TNs.</t>
+          <t>Tried online tests; could work, but strongly dislike the auto-grader marking off for spelling (3rd, 5th). 1st still prints/uses paper TNs.</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>Reducing student devices; willing to pay more for paper. Teacher-side tech is fine; student-side tech is scrutinized.</t>
         </is>
       </c>
     </row>
@@ -940,6 +1031,11 @@
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr"/>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>Not directly addressed.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -961,6 +1057,11 @@
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr"/>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>Not directly addressed. (Engagement is driven by the discussion/ownership model rather than the book format.)</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
@@ -982,6 +1083,11 @@
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr"/>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>Opposite of print-limited — willing to raise tuition to cover paper costs.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
@@ -1003,6 +1109,11 @@
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr"/>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>Not directly addressed.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
@@ -1024,6 +1135,11 @@
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr"/>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>Block schedule: 75-min sessions every other day (effective ~65-70 min after a mandatory 5-10 min reading period). Direct instruction kept to &lt;=20 min, then discussion/activities fill the rest.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
@@ -1045,6 +1161,11 @@
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr"/>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>Not asked verbatim; OT/NT survey (6th/7th) plus the Casket-Empty mnemonic already organize scripture into a cohesive meta-narrative, so a Bible-events timeline is philosophically aligned.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
@@ -1066,6 +1187,11 @@
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr"/>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>Minimizing — phone-free environment and reduced Chromebook use across the board.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
@@ -1088,7 +1214,12 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>Ask: memory-verse SONGS with HAND MOTIONS (raised by 3rd &amp; 4th; 3rd finds her own now). Hand motions aid retention even MS/HS per admin Melissa (older grades without the song).</t>
+          <t>Ask: memory-verse SONGS with HAND MOTIONS (3rd, 4th; 3rd finds her own now). Hand motions aid retention even MS/HS per admin Melissa.</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>Family devotionals plus a mandatory 5-10 min reading period at the start of every core class.</t>
         </is>
       </c>
     </row>
@@ -1112,6 +1243,11 @@
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr"/>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>No dedicated MS human sexuality unit; addresses behavioral purity and orientation generally, with a senior 'theology of the body' course. Sexuality is touched within 8th-grade apologetics/ethics.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
@@ -1133,6 +1269,11 @@
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr"/>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>STRONG YES — wants to add an informal logic course to middle school if a smooth, usable curriculum exists. DeepRoots offered optional 7th/8th logic materials (Jacob to send). 5th grade already framed as the 'logic phase.'</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
@@ -1154,6 +1295,11 @@
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr"/>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>Already runs a mandatory 5-10 min reading period at the start of core classes, then discussion/inquiry (Harkness) and extension. Engagements: discussion, independent projects, presentations.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
@@ -1175,6 +1321,11 @@
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr"/>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>Leans toward paper/print (willing to raise tuition for paper; actively reducing screens).</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
@@ -1196,6 +1347,11 @@
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr"/>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>Discussion/group (Harkness) is central, alongside independent projects; both, but discussion-forward.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
@@ -1217,6 +1373,11 @@
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr"/>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>Reading period -&gt; direct instruction (&lt;=20 min, ideally ~17) -&gt; Harkness discussion and extension, built around inquiry and ownership.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
@@ -1239,7 +1400,12 @@
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>Auto-graded online assessments promising but the spelling penalty undermines them (see Q18). Kids using Bibles more is seen as a win (2nd).</t>
+          <t>Auto-graded online assessments promising but the spelling penalty undermines them. Kids using Bibles more is a win (2nd).</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>Wheaton global student assessment 3x/year (worldview/formation metrics); spiritual-growth assessments + 1:1 conferences; adding faith-outcome questions to the 5-year alumni survey. North star: 'resilient disciples.'</t>
         </is>
       </c>
     </row>
@@ -1264,7 +1430,12 @@
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>Avoid classical/fine-art visuals for this age (didn't connect); avoid overly juvenile song styles for upper elementary; scrolling-heavy digital layout is a negative (5th).</t>
+          <t>Avoid classical/fine-art visuals for this age; avoid juvenile song styles for upper elementary; scrolling-heavy layout is a negative (5th).</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>Not directly addressed.</t>
         </is>
       </c>
     </row>
@@ -1288,6 +1459,11 @@
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr"/>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>Media kept to 3-7 min; strong interest in content built on the 'argument from beauty'/aesthetics.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
@@ -1310,7 +1486,12 @@
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>Role play rates HIGH here — kids love it, Good Samaritan role play a standout (3rd). NOTE: opposite of the middle-school signal (rated low there).</t>
+          <t>Role play rates HIGH here — kids love it, Good Samaritan role play a standout (3rd). NOTE: opposite of the middle-school signal.</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>Not directly addressed.</t>
         </is>
       </c>
     </row>
@@ -1334,6 +1515,11 @@
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr"/>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>A content-regurgitation-only model (wants soul-level reflection, not facts-for-a-grade); excessive student screen time.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
@@ -1355,6 +1541,11 @@
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr"/>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>Harkness discussion, student ownership/inquiry, short direct-instruction bursts, and countering short-form-media habits (the gap between how long students CAN vs. WILL attend).</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
@@ -1376,6 +1567,11 @@
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr"/>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>Discussion/inquiry-driven with clear division targets (6th OT survey, 7th NT survey, 8th worldview/apologetics/ethics), the Casket-Empty meta-narrative, an integrated logic track, common assessments enabling reteach/extension, minimal student screens, aiming at 'resilient disciples.'</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr"/>
@@ -1383,6 +1579,7 @@
       <c r="C42" s="3" t="inlineStr"/>
       <c r="D42" s="3" t="inlineStr"/>
       <c r="E42" s="3" t="inlineStr"/>
+      <c r="F42" s="3" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
@@ -1394,6 +1591,7 @@
       <c r="C43" s="4" t="inlineStr"/>
       <c r="D43" s="4" t="inlineStr"/>
       <c r="E43" s="4" t="inlineStr"/>
+      <c r="F43" s="4" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="5" t="inlineStr"/>
@@ -1405,12 +1603,17 @@
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>Meredith Arldt — Aliso Viejo Christian School (CA) — 2026-09-24</t>
+          <t>Meredith Arldt — Aliso Viejo Christian School (CA) — teacher/admin — 2026-09-24</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t>Atlantic Shores Christian School (VA) — 9/29/26 (current K-5 use)</t>
+          <t>Atlantic Shores Christian School (VA) — current K-5 use — 9/29/26</t>
+        </is>
+      </c>
+      <c r="F44" s="5" t="inlineStr">
+        <is>
+          <t>Will Weaver — Des Moines Christian School (IA) — Head of Spiritual Formation (admin) — 2026-09-30</t>
         </is>
       </c>
     </row>
@@ -1424,6 +1627,7 @@
       </c>
       <c r="D45" s="3" t="inlineStr"/>
       <c r="E45" s="3" t="inlineStr"/>
+      <c r="F45" s="3" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr"/>
@@ -1435,6 +1639,7 @@
       </c>
       <c r="D46" s="3" t="inlineStr"/>
       <c r="E46" s="3" t="inlineStr"/>
+      <c r="F46" s="3" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr"/>
@@ -1446,6 +1651,7 @@
       </c>
       <c r="D47" s="3" t="inlineStr"/>
       <c r="E47" s="3" t="inlineStr"/>
+      <c r="F47" s="3" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="3" t="inlineStr"/>
@@ -1457,6 +1663,7 @@
       </c>
       <c r="D48" s="3" t="inlineStr"/>
       <c r="E48" s="3" t="inlineStr"/>
+      <c r="F48" s="3" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr"/>
@@ -1468,17 +1675,31 @@
       </c>
       <c r="D49" s="3" t="inlineStr"/>
       <c r="E49" s="3" t="inlineStr"/>
+      <c r="F49" s="3" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr"/>
       <c r="B50" s="3" t="inlineStr"/>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>Overall / key takeaways for the curriculum</t>
+          <t>Jacob Waller</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr"/>
       <c r="E50" s="3" t="inlineStr"/>
+      <c r="F50" s="3" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr"/>
+      <c r="B51" s="3" t="inlineStr"/>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>Overall / key takeaways for the curriculum</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr"/>
+      <c r="E51" s="3" t="inlineStr"/>
+      <c r="F51" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1491,7 +1712,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:C29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1507,16 +1728,16 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="7" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>Follow-up meeting 9/29/26  |  ~$11,000 account  |  Current DeepRoots K-5 customer</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
-        <is>
-          <t>Attendees: Admin Melissa Wetzel + grade-level Mentor teachers (K-5). Each grade has 3 teachers + 1 mentor; only mentors attended.</t>
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Attendees: Admin Melissa Wetzel + grade-level Mentor teachers (K-5).</t>
         </is>
       </c>
     </row>
@@ -1584,7 +1805,7 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Going good; parents also like the curriculum (unsure how many use the PEP). 'Intro to Jesus' unit too high-level (lower grades agreed); kids didn't like/understand the classical art; too much time explaining things like Jesus called a 'lunatic' (kids don't get it). Likes that students use their Bibles much more now.</t>
+          <t>Going good; parents also like the curriculum (unsure how many use the PEP). 'Intro to Jesus' unit too high-level (lower grades agreed); kids didn't like/understand the classical art; too much time explaining things like Jesus called a 'lunatic'. Likes that students use their Bibles much more now.</t>
         </is>
       </c>
     </row>
@@ -1601,7 +1822,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Going well. Toggling between Student World (SW) and Teacher World (TW) is sometimes too much/confusing. Loves the content; kids love Role Play (esp. Good Samaritan). TE super helpful with so much content; loves having 10 days of content to choose from and time to dive deep. Wishes for Bible-verse songs with hand motions (finds her own now). Tried online tests — could work, but dislikes marking off for spelling.</t>
+          <t>Going well. Toggling between Student World (SW) and Teacher World (TW) is sometimes too much/confusing. Loves the content; kids love Role Play (esp. Good Samaritan). TE super helpful; loves 10 days of content to choose from and time to dive deep. Wishes for Bible-verse songs with hand motions. Tried online tests, but dislikes marking off for spelling.</t>
         </is>
       </c>
     </row>
@@ -1618,7 +1839,7 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Enjoying it; uses the TNs when teaching. Really wants hand motions for the memory verses — they help upper grades learn verses. (Melissa: MS/HS use hand motions for retention too, just without a song.)</t>
+          <t>Enjoying it; uses the TNs when teaching. Really wants hand motions for the memory verses; they help upper grades learn verses. (Melissa: MS/HS use hand motions for retention too, without a song.)</t>
         </is>
       </c>
     </row>
@@ -1635,7 +1856,7 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>OK, but dislikes the scrolling format (too much to scroll). Dislikes online assessments marking off for spelling (not worth re-adjusting grades; defeats the auto-grade time savings). Content over their heads; many unchurched students make it hard (some don't know who Noah is, yet teaching substitutionary death). Songs too juvenile; prefers known 'brand name' songs (e.g., Forrest Frank).</t>
+          <t>OK, but dislikes the scrolling format. Dislikes online assessments marking off for spelling (defeats the auto-grade time savings). Content over their heads; many unchurched students make it hard. Songs too juvenile; prefers known 'brand name' songs (e.g., Forrest Frank).</t>
         </is>
       </c>
     </row>
@@ -1662,13 +1883,13 @@
       <c r="C13" s="3" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="A14" s="7" t="inlineStr">
         <is>
           <t>OBSERVED THEMES (from the notes)</t>
         </is>
       </c>
-      <c r="B14" s="8" t="inlineStr"/>
-      <c r="C14" s="8" t="inlineStr"/>
+      <c r="B14" s="7" t="inlineStr"/>
+      <c r="C14" s="7" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr"/>
@@ -1792,6 +2013,15 @@
       </c>
       <c r="C28" s="3" t="inlineStr"/>
     </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr"/>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Jacob Waller</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Migrate all five Meredith team takeaways into Q&A; point tracker at consolidated sheet
Carried over the DeepRoots team takeaways (Troy, Pat, Nancy, Tammy, Lisa)
from the earlier Meredith sheet into the Q&A takeaways block, rebuilt the
shared sheet with all three interviewees + Atlantic feedback, and repointed
tracker links to the consolidated sheet (rebased on latest).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BUC7AKNsC5W1a963Yi5JKY
</commit_message>
<xml_diff>
--- a/outreach/DeepRoots_Interview_QA.xlsx
+++ b/outreach/DeepRoots_Interview_QA.xlsx
@@ -1625,7 +1625,11 @@
           <t>Troy Winkler</t>
         </is>
       </c>
-      <c r="D45" s="3" t="inlineStr"/>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>That we need to have content relatable to that age group - video and illustrations should be more modern and age appropriate instead of cartoon animations.</t>
+        </is>
+      </c>
       <c r="E45" s="3" t="inlineStr"/>
       <c r="F45" s="3" t="inlineStr"/>
     </row>
@@ -1637,7 +1641,11 @@
           <t>Pat Williamson</t>
         </is>
       </c>
-      <c r="D46" s="3" t="inlineStr"/>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>That teachers were supplementing with outside media.</t>
+        </is>
+      </c>
       <c r="E46" s="3" t="inlineStr"/>
       <c r="F46" s="3" t="inlineStr"/>
     </row>
@@ -1649,7 +1657,11 @@
           <t>Nancy Wood</t>
         </is>
       </c>
-      <c r="D47" s="3" t="inlineStr"/>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>She was all about discussions. I think adding additional optional discussion questions would be great (and not take too much of our time) for schools like hers that have 45 minutes. Based on what she was saying, we could also do more teaching through video as well. I agree with Lisa that we could work on having more ways to assess the materials, such as IBS and MV. Maybe don't make those optional? They aren't in lower grades.</t>
+        </is>
+      </c>
       <c r="E47" s="3" t="inlineStr"/>
       <c r="F47" s="3" t="inlineStr"/>
     </row>
@@ -1661,7 +1673,11 @@
           <t>Tammy Plett</t>
         </is>
       </c>
-      <c r="D48" s="3" t="inlineStr"/>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>I loved hearing that the workbook-based curricula were 'boring and dry' in her opinion. Note that they want to move away from 'cartoon' videos and visuals at this age and look for something more realistic, relatable and like them. That is something we have heard before and should keep in mind. Love that they started Teaching for Transformation a couple of years ago and are looking to put faith into action; that is something we can and should mesh with, maybe offering our own ideas for service projects that tie into our lessons as a Digging Deeper option. Also noted that she likes to make the historical aspect come alive so they can relate; that is where our Titus Kennedy archaeological pieces come into play. It was helpful to hear how long she thinks students at this age can sit and listen to a lecture before they check out. Good to know that discussion is helpful at this age.</t>
+        </is>
+      </c>
       <c r="E48" s="3" t="inlineStr"/>
       <c r="F48" s="3" t="inlineStr"/>
     </row>
@@ -1673,7 +1689,11 @@
           <t>Lisa Van Vlear</t>
         </is>
       </c>
-      <c r="D49" s="3" t="inlineStr"/>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>Meredith mentioned several times the importance of reflection and application for the students. 'How does this affect me today?' She stressed discussion and that if the lesson were 15 minutes, the rest of class time would be devoted to discussion. She was also a fan of archaeological pictures and historical context. I appreciated that since we do that well. I don't think we should shy away from that. Since Bible class needs to be given a grade, I'm wondering if we provide enough ways for a teacher to assign a grade. We have optional quizzes and tests. Sounds like they give points for scripture memorization. I'd like to hear from a teacher who's currently teaching our G7 what she is using to give scores. We do have the IBS component that could be given a score. Given all that she mentioned, I'd be really curious to get her thoughts if she would give G7 a good look.</t>
+        </is>
+      </c>
       <c r="E49" s="3" t="inlineStr"/>
       <c r="F49" s="3" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
Team takeaways by interview: add Will Weaver block with his actual attendees
Restructured the DeepRoots Team Takeaways section into per-interview blocks,
each listing that meeting's real attendees (from the Gemini notes/calendar):
Meredith (Troy, Pat, Nancy, Tammy, Lisa) and Will (Troy, Pat, Tammy, Lisa,
Jacob Waller). Rebuilt the shared sheet and repointed tracker links.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BUC7AKNsC5W1a963Yi5JKY
</commit_message>
<xml_diff>
--- a/outreach/DeepRoots_Interview_QA.xlsx
+++ b/outreach/DeepRoots_Interview_QA.xlsx
@@ -81,7 +81,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -91,6 +91,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -465,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F51"/>
+  <dimension ref="A1:F61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1598,52 +1601,48 @@
       <c r="B44" s="5" t="inlineStr"/>
       <c r="C44" s="5" t="inlineStr">
         <is>
+          <t>MEREDITH ARLDT interview — Aliso Viejo Christian School (CA), 2026-09-24  |  Attendees: Troy Winkler, Pat Williamson, Nancy Wood, Tammy Plett, Lisa Van Vlear</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr"/>
+      <c r="E44" s="5" t="inlineStr"/>
+      <c r="F44" s="5" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="inlineStr"/>
+      <c r="B45" s="6" t="inlineStr"/>
+      <c r="C45" s="6" t="inlineStr">
+        <is>
           <t>Team member</t>
         </is>
       </c>
-      <c r="D44" s="5" t="inlineStr">
+      <c r="D45" s="6" t="inlineStr">
         <is>
           <t>Meredith Arldt — Aliso Viejo Christian School (CA) — teacher/admin — 2026-09-24</t>
         </is>
       </c>
-      <c r="E44" s="5" t="inlineStr">
+      <c r="E45" s="6" t="inlineStr">
         <is>
           <t>Atlantic Shores Christian School (VA) — current K-5 use — 9/29/26</t>
         </is>
       </c>
-      <c r="F44" s="5" t="inlineStr">
+      <c r="F45" s="6" t="inlineStr">
         <is>
           <t>Will Weaver — Des Moines Christian School (IA) — Head of Spiritual Formation (admin) — 2026-09-30</t>
         </is>
       </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="3" t="inlineStr"/>
-      <c r="B45" s="3" t="inlineStr"/>
-      <c r="C45" s="3" t="inlineStr">
-        <is>
-          <t>Troy Winkler</t>
-        </is>
-      </c>
-      <c r="D45" s="3" t="inlineStr">
-        <is>
-          <t>That we need to have content relatable to that age group - video and illustrations should be more modern and age appropriate instead of cartoon animations.</t>
-        </is>
-      </c>
-      <c r="E45" s="3" t="inlineStr"/>
-      <c r="F45" s="3" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr"/>
       <c r="B46" s="3" t="inlineStr"/>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>Pat Williamson</t>
+          <t>Troy Winkler</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>That teachers were supplementing with outside media.</t>
+          <t>That we need to have content relatable to that age group - video and illustrations should be more modern and age appropriate instead of cartoon animations.</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr"/>
@@ -1654,12 +1653,12 @@
       <c r="B47" s="3" t="inlineStr"/>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>Nancy Wood</t>
+          <t>Pat Williamson</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>She was all about discussions. I think adding additional optional discussion questions would be great (and not take too much of our time) for schools like hers that have 45 minutes. Based on what she was saying, we could also do more teaching through video as well. I agree with Lisa that we could work on having more ways to assess the materials, such as IBS and MV. Maybe don't make those optional? They aren't in lower grades.</t>
+          <t>That teachers were supplementing with outside media.</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr"/>
@@ -1670,12 +1669,12 @@
       <c r="B48" s="3" t="inlineStr"/>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>Tammy Plett</t>
+          <t>Nancy Wood</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>I loved hearing that the workbook-based curricula were 'boring and dry' in her opinion. Note that they want to move away from 'cartoon' videos and visuals at this age and look for something more realistic, relatable and like them. That is something we have heard before and should keep in mind. Love that they started Teaching for Transformation a couple of years ago and are looking to put faith into action; that is something we can and should mesh with, maybe offering our own ideas for service projects that tie into our lessons as a Digging Deeper option. Also noted that she likes to make the historical aspect come alive so they can relate; that is where our Titus Kennedy archaeological pieces come into play. It was helpful to hear how long she thinks students at this age can sit and listen to a lecture before they check out. Good to know that discussion is helpful at this age.</t>
+          <t>She was all about discussions. I think adding additional optional discussion questions would be great (and not take too much of our time) for schools like hers that have 45 minutes. Based on what she was saying, we could also do more teaching through video as well. I agree with Lisa that we could work on having more ways to assess the materials, such as IBS and MV. Maybe don't make those optional? They aren't in lower grades.</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr"/>
@@ -1686,12 +1685,12 @@
       <c r="B49" s="3" t="inlineStr"/>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>Lisa Van Vlear</t>
+          <t>Tammy Plett</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>Meredith mentioned several times the importance of reflection and application for the students. 'How does this affect me today?' She stressed discussion and that if the lesson were 15 minutes, the rest of class time would be devoted to discussion. She was also a fan of archaeological pictures and historical context. I appreciated that since we do that well. I don't think we should shy away from that. Since Bible class needs to be given a grade, I'm wondering if we provide enough ways for a teacher to assign a grade. We have optional quizzes and tests. Sounds like they give points for scripture memorization. I'd like to hear from a teacher who's currently teaching our G7 what she is using to give scores. We do have the IBS component that could be given a score. Given all that she mentioned, I'd be really curious to get her thoughts if she would give G7 a good look.</t>
+          <t>I loved hearing that the workbook-based curricula were 'boring and dry' in her opinion. Note that they want to move away from 'cartoon' videos and visuals at this age and look for something more realistic, relatable and like them. That is something we have heard before and should keep in mind. Love that they started Teaching for Transformation a couple of years ago and are looking to put faith into action; that is something we can and should mesh with, maybe offering our own ideas for service projects that tie into our lessons as a Digging Deeper option. Also noted that she likes to make the historical aspect come alive so they can relate; that is where our Titus Kennedy archaeological pieces come into play. It was helpful to hear how long she thinks students at this age can sit and listen to a lecture before they check out. Good to know that discussion is helpful at this age.</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr"/>
@@ -1702,10 +1701,14 @@
       <c r="B50" s="3" t="inlineStr"/>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>Jacob Waller</t>
-        </is>
-      </c>
-      <c r="D50" s="3" t="inlineStr"/>
+          <t>Lisa Van Vlear</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>Meredith mentioned several times the importance of reflection and application for the students. 'How does this affect me today?' She stressed discussion and that if the lesson were 15 minutes, the rest of class time would be devoted to discussion. She was also a fan of archaeological pictures and historical context. I appreciated that since we do that well. I don't think we should shy away from that. Since Bible class needs to be given a grade, I'm wondering if we provide enough ways for a teacher to assign a grade. We have optional quizzes and tests. Sounds like they give points for scripture memorization. I'd like to hear from a teacher who's currently teaching our G7 what she is using to give scores. We do have the IBS component that could be given a score. Given all that she mentioned, I'd be really curious to get her thoughts if she would give G7 a good look.</t>
+        </is>
+      </c>
       <c r="E50" s="3" t="inlineStr"/>
       <c r="F50" s="3" t="inlineStr"/>
     </row>
@@ -1720,6 +1723,130 @@
       <c r="D51" s="3" t="inlineStr"/>
       <c r="E51" s="3" t="inlineStr"/>
       <c r="F51" s="3" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="inlineStr"/>
+      <c r="B52" s="3" t="inlineStr"/>
+      <c r="C52" s="3" t="inlineStr"/>
+      <c r="D52" s="3" t="inlineStr"/>
+      <c r="E52" s="3" t="inlineStr"/>
+      <c r="F52" s="3" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr"/>
+      <c r="B53" s="5" t="inlineStr"/>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>WILL WEAVER interview — Des Moines Christian School (IA), 2026-09-30  |  Attendees: Troy Winkler, Pat Williamson, Tammy Plett, Lisa Van Vlear, Jacob Waller</t>
+        </is>
+      </c>
+      <c r="D53" s="5" t="inlineStr"/>
+      <c r="E53" s="5" t="inlineStr"/>
+      <c r="F53" s="5" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="6" t="inlineStr"/>
+      <c r="B54" s="6" t="inlineStr"/>
+      <c r="C54" s="6" t="inlineStr">
+        <is>
+          <t>Team member</t>
+        </is>
+      </c>
+      <c r="D54" s="6" t="inlineStr">
+        <is>
+          <t>Meredith Arldt — Aliso Viejo Christian School (CA) — teacher/admin — 2026-09-24</t>
+        </is>
+      </c>
+      <c r="E54" s="6" t="inlineStr">
+        <is>
+          <t>Atlantic Shores Christian School (VA) — current K-5 use — 9/29/26</t>
+        </is>
+      </c>
+      <c r="F54" s="6" t="inlineStr">
+        <is>
+          <t>Will Weaver — Des Moines Christian School (IA) — Head of Spiritual Formation (admin) — 2026-09-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="inlineStr"/>
+      <c r="B55" s="3" t="inlineStr"/>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>Troy Winkler</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr"/>
+      <c r="E55" s="3" t="inlineStr"/>
+      <c r="F55" s="3" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr"/>
+      <c r="B56" s="3" t="inlineStr"/>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>Pat Williamson</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr"/>
+      <c r="E56" s="3" t="inlineStr"/>
+      <c r="F56" s="3" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="inlineStr"/>
+      <c r="B57" s="3" t="inlineStr"/>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>Tammy Plett</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr"/>
+      <c r="E57" s="3" t="inlineStr"/>
+      <c r="F57" s="3" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="3" t="inlineStr"/>
+      <c r="B58" s="3" t="inlineStr"/>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>Lisa Van Vlear</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="inlineStr"/>
+      <c r="E58" s="3" t="inlineStr"/>
+      <c r="F58" s="3" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="3" t="inlineStr"/>
+      <c r="B59" s="3" t="inlineStr"/>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>Jacob Waller</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="inlineStr"/>
+      <c r="E59" s="3" t="inlineStr"/>
+      <c r="F59" s="3" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="3" t="inlineStr"/>
+      <c r="B60" s="3" t="inlineStr"/>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>Overall / key takeaways for the curriculum</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="inlineStr"/>
+      <c r="E60" s="3" t="inlineStr"/>
+      <c r="F60" s="3" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="3" t="inlineStr"/>
+      <c r="B61" s="3" t="inlineStr"/>
+      <c r="C61" s="3" t="inlineStr"/>
+      <c r="D61" s="3" t="inlineStr"/>
+      <c r="E61" s="3" t="inlineStr"/>
+      <c r="F61" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1741,7 +1868,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>Atlantic Shores Christian School — Virginia</t>
         </is>
@@ -1903,13 +2030,13 @@
       <c r="C13" s="3" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="inlineStr">
+      <c r="A14" s="8" t="inlineStr">
         <is>
           <t>OBSERVED THEMES (from the notes)</t>
         </is>
       </c>
-      <c r="B14" s="7" t="inlineStr"/>
-      <c r="C14" s="7" t="inlineStr"/>
+      <c r="B14" s="8" t="inlineStr"/>
+      <c r="C14" s="8" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr"/>

</xml_diff>

<commit_message>
Add Horizon Christian (OR) follow-up to Q&A workbook
Horizon Christian Elementary (Tualatin, OR) 9/28 follow-up with a
current K-5 customer, run by Tammy Plett. Mirrors the Atlantic Shores
treatment: a new Horizon column on the All Interviews master (orange)
plus a dedicated Horizon Christian (OR) Feedback tab with per-grade
feedback and observed themes. Read Me color key and tracker updated.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BUC7AKNsC5W1a963Yi5JKY
</commit_message>
<xml_diff>
--- a/outreach/DeepRoots_Interview_QA.xlsx
+++ b/outreach/DeepRoots_Interview_QA.xlsx
@@ -12,6 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Meredith Arldt" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Will Weaver" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atlantic Shores (VA) Feedback" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Horizon Christian (OR) Feedback" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -73,8 +74,13 @@
       <color rgb="00548235"/>
       <sz val="13"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00C55A11"/>
+      <sz val="13"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -98,6 +104,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00C55A11"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00404040"/>
       </patternFill>
     </fill>
@@ -114,6 +125,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E9DFF3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
     <fill>
@@ -148,7 +164,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -160,8 +176,9 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -173,10 +190,10 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -185,13 +202,16 @@
     <xf numFmtId="0" fontId="6" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -200,17 +220,25 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -577,7 +605,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A17"/>
+  <dimension ref="A1:A18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -624,7 +652,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>- Atlantic Shores (VA) Feedback: a current K-5 customer's per-grade feedback (different shape from the interviews).</t>
+          <t>- Current-customer feedback tabs (Atlantic Shores VA, Horizon Christian OR): per-grade feedback from schools already using DeepRoots K-5 (different shape from the interviews).</t>
         </is>
       </c>
     </row>
@@ -687,6 +715,13 @@
       <c r="A17" s="6" t="inlineStr">
         <is>
           <t>Atlantic Shores (VA)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>Horizon Christian (OR)</t>
         </is>
       </c>
     </row>
@@ -702,7 +737,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F43"/>
+  <dimension ref="A1:G43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -711,1126 +746,1224 @@
     <col width="52" customWidth="1" min="4" max="4"/>
     <col width="52" customWidth="1" min="5" max="5"/>
     <col width="52" customWidth="1" min="6" max="6"/>
+    <col width="52" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>DeepRoots Interview Q&amp;A — All Interviews (side by side)</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>Section</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="9" t="inlineStr">
         <is>
           <t>Q#</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="C3" s="9" t="inlineStr">
         <is>
           <t>Question</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="D3" s="10" t="inlineStr">
         <is>
           <t>Meredith Arldt</t>
         </is>
       </c>
-      <c r="E3" s="10" t="inlineStr">
+      <c r="E3" s="11" t="inlineStr">
         <is>
           <t>Atlantic Shores (VA)</t>
         </is>
       </c>
-      <c r="F3" s="11" t="inlineStr">
+      <c r="F3" s="12" t="inlineStr">
         <is>
           <t>Will Weaver</t>
         </is>
       </c>
+      <c r="G3" s="13" t="inlineStr">
+        <is>
+          <t>Horizon Christian (OR)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="12" t="inlineStr"/>
-      <c r="B4" s="12" t="inlineStr"/>
-      <c r="C4" s="12" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr"/>
+      <c r="B4" s="14" t="inlineStr"/>
+      <c r="C4" s="14" t="inlineStr">
         <is>
           <t>(question)</t>
         </is>
       </c>
-      <c r="D4" s="13" t="inlineStr">
+      <c r="D4" s="15" t="inlineStr">
         <is>
           <t>Aliso Viejo Christian (CA) 9/24</t>
         </is>
       </c>
-      <c r="E4" s="14" t="inlineStr">
+      <c r="E4" s="16" t="inlineStr">
         <is>
           <t>Atlantic Shores (VA) K-5 use 9/29</t>
         </is>
       </c>
-      <c r="F4" s="15" t="inlineStr">
+      <c r="F4" s="17" t="inlineStr">
         <is>
           <t>Des Moines Christian (IA) 9/30</t>
         </is>
       </c>
+      <c r="G4" s="18" t="inlineStr">
+        <is>
+          <t>Horizon Christian (OR) K-5 use 9/28</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="16" t="inlineStr">
+      <c r="A5" s="19" t="inlineStr">
         <is>
           <t>Marketing &amp; Sales</t>
         </is>
       </c>
-      <c r="B5" s="17" t="n">
+      <c r="B5" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="C5" s="17" t="inlineStr">
+      <c r="C5" s="20" t="inlineStr">
         <is>
           <t>How does your school categorize Middle School / Junior High (5-8, 6-8, 7-8)?</t>
         </is>
       </c>
-      <c r="D5" s="18" t="inlineStr">
+      <c r="D5" s="21" t="inlineStr">
         <is>
           <t>Middle school is 6th, 7th, and 8th grade (6-8).</t>
         </is>
       </c>
-      <c r="E5" s="19" t="inlineStr"/>
-      <c r="F5" s="20" t="inlineStr">
+      <c r="E5" s="22" t="inlineStr"/>
+      <c r="F5" s="23" t="inlineStr">
         <is>
           <t>Currently MS = 6-8 (this year 68 students, next year 58). Next year pulling 5th grade into a unified 5-8 middle school; 5th treated as the 'logic phase.'</t>
         </is>
       </c>
+      <c r="G5" s="24" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="19" t="inlineStr">
         <is>
           <t>Marketing &amp; Sales</t>
         </is>
       </c>
-      <c r="B6" s="17" t="n">
+      <c r="B6" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="C6" s="17" t="inlineStr">
+      <c r="C6" s="20" t="inlineStr">
         <is>
           <t>What are the primary differences between a 6th, 7th, and 8th grade student (developmentally, spiritually, emotionally)?</t>
         </is>
       </c>
-      <c r="D6" s="18" t="inlineStr">
+      <c r="D6" s="21" t="inlineStr">
         <is>
           <t>Students begin actively questioning their own faith and searching for personal identity ('why do I believe what I believe?') amid outside influences like social media. 6th graders want independence but still want the safety net of mom and dad, going back and forth. 7th graders like to push and challenge ('their own little beast'). 8th graders can get 'a little too big for their own.' Spirituality is hard at this age because it is not always tangible.</t>
         </is>
       </c>
-      <c r="E6" s="19" t="inlineStr"/>
-      <c r="F6" s="20" t="inlineStr">
+      <c r="E6" s="22" t="inlineStr"/>
+      <c r="F6" s="23" t="inlineStr">
         <is>
           <t>5th graders have more in common with 7th/8th than K-1; ready for inquiry ('why' questions), not just content. Discussion capacity grows: ~20 min in 6th, 25-30 min in 7th-8th as they take ownership. Student certainty on absolute moral truth tends to DECREASE in higher grades.</t>
         </is>
       </c>
+      <c r="G6" s="24" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="19" t="inlineStr">
         <is>
           <t>Marketing &amp; Sales</t>
         </is>
       </c>
-      <c r="B7" s="17" t="n">
+      <c r="B7" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="C7" s="17" t="inlineStr">
+      <c r="C7" s="20" t="inlineStr">
         <is>
           <t>How do you best reach both churched and unchurched students? Is this an issue for you? What works best?</t>
         </is>
       </c>
-      <c r="D7" s="18" t="inlineStr">
+      <c r="D7" s="21" t="inlineStr">
         <is>
           <t>About 60% of the school population identifies with a church home; 40% do not. They are intentional about corporate worship (for some students it is their only weekly worship) and adopted the Teaching for Transformation framework (from CASE) two years ago, with flex projects that put faith into action. They are also rebuilding the historically broken bridge with their associated church to connect unchurched families with pastoral staff.</t>
         </is>
       </c>
-      <c r="E7" s="19" t="inlineStr">
+      <c r="E7" s="22" t="inlineStr">
         <is>
           <t>Many unchurched students make deeper concepts hard (5th/Miriam): some don't even know who Noah is, yet the lesson teaches substitutionary death.</t>
         </is>
       </c>
-      <c r="F7" s="20" t="inlineStr">
+      <c r="F7" s="23" t="inlineStr">
         <is>
           <t>Covenantal school, ~1,650 students; long-time DeepRoots elementary user (~40 students). Program goal across EE-12: 'resilient disciples' who own their faith.</t>
         </is>
       </c>
+      <c r="G7" s="24" t="inlineStr">
+        <is>
+          <t>Many unchurched students (G4): confused by unfamiliar terms like 'Sanhedrin' and by using multiple Bible translations (their students use NIV). Asked for a single translation. 'Intro to Jesus' is the key unit for unchurched kids.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="16" t="inlineStr">
+      <c r="A8" s="19" t="inlineStr">
         <is>
           <t>Marketing &amp; Sales</t>
         </is>
       </c>
-      <c r="B8" s="17" t="n">
+      <c r="B8" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="C8" s="17" t="inlineStr">
+      <c r="C8" s="20" t="inlineStr">
         <is>
           <t>What do you like or dislike about your current Bible curriculum?</t>
         </is>
       </c>
-      <c r="D8" s="18" t="inlineStr">
+      <c r="D8" s="21" t="inlineStr">
         <is>
           <t>Currently workbook-based: Purposeful Design (Daring Deliverers), and Positive Action (Character Counts for 6th, Wise Up for 8th). All workbook-based and 'pretty dry and boring.' The goal is to keep Bible from feeling like just another academic class and to focus on students' hearts, not grade their faith.</t>
         </is>
       </c>
-      <c r="E8" s="19" t="inlineStr">
+      <c r="E8" s="22" t="inlineStr">
         <is>
           <t>LIKES: love the content (3rd); Teacher Editions/Teacher Notes very helpful across grades; 3rd likes 10 days of content to choose from with room to dive deep; kids using their Bibles more (2nd); parents like it (2nd). DISLIKES: too much content for youngest grades (1st, 2nd); 'Intro to Jesus' unit too high-level (2nd + lower grades); scrolling format too much (5th); content over students' heads in 5th.</t>
         </is>
       </c>
-      <c r="F8" s="20" t="inlineStr">
+      <c r="F8" s="23" t="inlineStr">
         <is>
           <t>MS Bible progression: 6th = Old Testament survey, 7th = New Testament survey, 8th = intro to worldview, apologetics &amp; ethics. Uses the Casket-Empty(-Open) mnemonic across 6/7/8 to anchor stories into scripture's meta-narrative. Long-time DeepRoots user in elementary.</t>
         </is>
       </c>
+      <c r="G8" s="24" t="inlineStr">
+        <is>
+          <t>Overall going well K-5. Kids love the songs (G1) and the discussions; K praises the variety of activities for different learners ('variety is key'). Clunky to get used to at first (G1). Projecting the visuals is clunky across ALL grades.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="16" t="inlineStr">
+      <c r="A9" s="19" t="inlineStr">
         <is>
           <t>Marketing &amp; Sales</t>
         </is>
       </c>
-      <c r="B9" s="17" t="n">
+      <c r="B9" s="20" t="n">
         <v>5</v>
       </c>
-      <c r="C9" s="17" t="inlineStr">
+      <c r="C9" s="20" t="inlineStr">
         <is>
           <t>What elements would you like to see in it each week?</t>
         </is>
       </c>
-      <c r="D9" s="18" t="inlineStr">
+      <c r="D9" s="21" t="inlineStr">
         <is>
           <t>More reflection and personal application ('how does this resonate with you today? what do we do with this?'). Historical and cultural context so students understand the significance of events. Treat biblical figures and events as real history, not 'stories' or fairy tales.</t>
         </is>
       </c>
-      <c r="E9" s="19" t="inlineStr"/>
-      <c r="F9" s="20" t="inlineStr">
+      <c r="E9" s="22" t="inlineStr"/>
+      <c r="F9" s="23" t="inlineStr">
         <is>
           <t>Discussion-based (Harkness) conversations, growing in length by grade; family devotionals; common assessments across 6-8 enabling reteach + extension; a mandatory 5-10 min reading period at the start of every core class.</t>
         </is>
       </c>
+      <c r="G9" s="24" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="16" t="inlineStr">
+      <c r="A10" s="19" t="inlineStr">
         <is>
           <t>Marketing &amp; Sales</t>
         </is>
       </c>
-      <c r="B10" s="17" t="n">
+      <c r="B10" s="20" t="n">
         <v>6</v>
       </c>
-      <c r="C10" s="17" t="inlineStr">
+      <c r="C10" s="20" t="inlineStr">
         <is>
           <t>What core ideals do you wish each student left your class identifying with?</t>
         </is>
       </c>
-      <c r="D10" s="18" t="inlineStr">
+      <c r="D10" s="21" t="inlineStr">
         <is>
           <t>Moving from head knowledge to heart knowledge; a real identity in Christ; applying scripture to their own lives; striving to be the best version of who God created them to be.</t>
         </is>
       </c>
-      <c r="E10" s="19" t="inlineStr"/>
-      <c r="F10" s="20" t="inlineStr">
+      <c r="E10" s="22" t="inlineStr"/>
+      <c r="F10" s="23" t="inlineStr">
         <is>
           <t>'Resilient disciples' who take ownership of their faith — able to take doctrine apart and put it back together, and articulate not just what it says but 'where it sits in your soul,' rather than regurgitate content for a grade.</t>
         </is>
       </c>
+      <c r="G10" s="24" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="16" t="inlineStr">
+      <c r="A11" s="19" t="inlineStr">
         <is>
           <t>Marketing &amp; Sales</t>
         </is>
       </c>
-      <c r="B11" s="17" t="n">
+      <c r="B11" s="20" t="n">
         <v>7</v>
       </c>
-      <c r="C11" s="17" t="inlineStr">
+      <c r="C11" s="20" t="inlineStr">
         <is>
           <t>What types of resources (videos, activities, etc.) are most helpful for you as a teacher?</t>
         </is>
       </c>
-      <c r="D11" s="18" t="inlineStr">
+      <c r="D11" s="21" t="inlineStr">
         <is>
           <t>Short videos (about 1.5-5 minutes), historical family trees, Bible timelines, primary documents, original-language (Greek/Hebrew) references, and cultural/archaeological references (e.g., an archaeological Bible). Note: curating and vetting these is the most time-consuming part for teachers, so ready-made, vetted resources would help most.</t>
         </is>
       </c>
-      <c r="E11" s="19" t="inlineStr">
+      <c r="E11" s="22" t="inlineStr">
         <is>
           <t>Teacher Editions / Teacher Notes (TEs/TNs) most helpful (1st printed &amp; uses TNs; 4th teaches from TNs; 3rd: TE super helpful with so much content).</t>
         </is>
       </c>
-      <c r="F11" s="20" t="inlineStr">
+      <c r="F11" s="23" t="inlineStr">
         <is>
           <t>Strong interest in usable Logic materials (DeepRoots offered optional 7th/8th logic sets). Casket-Empty mnemonic; Wheaton global student assessment 3x/year for worldview metrics.</t>
         </is>
       </c>
+      <c r="G11" s="24" t="inlineStr">
+        <is>
+          <t>Wants Teaching Essentials split out by unit (not one long doc) with the key elements listed inline (Bible reading passage, memory verse) so teachers aren't juggling multiple sources; printed TNs are too long.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="16" t="inlineStr">
+      <c r="A12" s="19" t="inlineStr">
         <is>
           <t>Editorial</t>
         </is>
       </c>
-      <c r="B12" s="17" t="n">
+      <c r="B12" s="20" t="n">
         <v>8</v>
       </c>
-      <c r="C12" s="17" t="inlineStr">
+      <c r="C12" s="20" t="inlineStr">
         <is>
           <t>How many minutes can students pay attention to teaching, reading, discussion, activities?</t>
         </is>
       </c>
-      <c r="D12" s="18" t="inlineStr">
+      <c r="D12" s="21" t="inlineStr">
         <is>
           <t>Lecture/teaching is kept to 15-20 minutes max before moving into discussion. A typical rhythm is a ~5-minute intro/review, a 10-15 minute lesson, then discussion. Class is mostly discussion-based; some reading.</t>
         </is>
       </c>
-      <c r="E12" s="19" t="inlineStr"/>
-      <c r="F12" s="20" t="inlineStr">
+      <c r="E12" s="22" t="inlineStr"/>
+      <c r="F12" s="23" t="inlineStr">
         <is>
           <t>Targets: direct instruction 20 min or less (ideally ~17); media 3-7 min; student activities 15-20 min before attention drops. Discussions: ~20 min (6th), 25-30 min (7th-8th).</t>
         </is>
       </c>
+      <c r="G12" s="24" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="16" t="inlineStr">
+      <c r="A13" s="19" t="inlineStr">
         <is>
           <t>Editorial</t>
         </is>
       </c>
-      <c r="B13" s="17" t="n">
+      <c r="B13" s="20" t="n">
         <v>9</v>
       </c>
-      <c r="C13" s="17" t="inlineStr">
+      <c r="C13" s="20" t="inlineStr">
         <is>
           <t>What kind of engagements do students enjoy most (by grade)?</t>
         </is>
       </c>
-      <c r="D13" s="18" t="inlineStr">
+      <c r="D13" s="21" t="inlineStr">
         <is>
           <t>Discussion-based work and things they can relate to (real-world video, relatable visuals), partner work, and interactive questions. Discussion is the biggest draw across middle school.</t>
         </is>
       </c>
-      <c r="E13" s="19" t="inlineStr"/>
-      <c r="F13" s="20" t="inlineStr">
+      <c r="E13" s="22" t="inlineStr"/>
+      <c r="F13" s="23" t="inlineStr">
         <is>
           <t>Harkness roundtable discussions (even mixed 6-8 for high performers), independent projects/research, and presentations, especially in 8th.</t>
         </is>
       </c>
+      <c r="G13" s="24" t="inlineStr">
+        <is>
+          <t>Kids love the songs and the discussions (K/G1); variety of activities valued (K).</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="16" t="inlineStr">
+      <c r="A14" s="19" t="inlineStr">
         <is>
           <t>Editorial</t>
         </is>
       </c>
-      <c r="B14" s="17" t="n">
+      <c r="B14" s="20" t="n">
         <v>10</v>
       </c>
-      <c r="C14" s="17" t="inlineStr">
+      <c r="C14" s="20" t="inlineStr">
         <is>
           <t>How do you use screens and technology in your classroom?</t>
         </is>
       </c>
-      <c r="D14" s="18" t="inlineStr">
+      <c r="D14" s="21" t="inlineStr">
         <is>
           <t>Google Classroom is the platform; laptops are provided but screen time is intentionally limited (parents appreciate this). Currently projection-based; installing BenQ interactive smartboards by January (grant-funded), with teacher training.</t>
         </is>
       </c>
-      <c r="E14" s="19" t="inlineStr">
+      <c r="E14" s="22" t="inlineStr">
         <is>
           <t>K teachers project/teach from the Teacher site; rooms lack 2 devices (one-device teaching); early tech issues now mostly worked through.</t>
         </is>
       </c>
-      <c r="F14" s="20" t="inlineStr">
+      <c r="F14" s="23" t="inlineStr">
         <is>
           <t>Phone-free K-12; deliberately scaling back student Chromebook use (screens promote skimming/distraction). Willing to raise tuition for paper; challenges teachers to justify student tech vs. checking a box. Distinguishes beneficial teacher-side tech from student-side.</t>
         </is>
       </c>
+      <c r="G14" s="24" t="inlineStr">
+        <is>
+          <t>Projecting the visuals/script is clunky for all grades; no student devices at school. A slideshow version (with show/hide slides) is the top ask.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="16" t="inlineStr">
+      <c r="A15" s="19" t="inlineStr">
         <is>
           <t>Editorial</t>
         </is>
       </c>
-      <c r="B15" s="17" t="n">
+      <c r="B15" s="20" t="n">
         <v>11</v>
       </c>
-      <c r="C15" s="17" t="inlineStr">
+      <c r="C15" s="20" t="inlineStr">
         <is>
           <t>What questions/issues do you see students wrestling with (by grade)?</t>
         </is>
       </c>
-      <c r="D15" s="18" t="inlineStr">
+      <c r="D15" s="21" t="inlineStr">
         <is>
           <t>Reconciling 'what my parents taught me' with 'what do I actually believe'; identity in Christ versus societal pressure and peer acceptance; influence of social media; and nominal Christianity ('Christian in name only') where students know the Sunday-school answers but haven't moved it from head to heart.</t>
         </is>
       </c>
-      <c r="E15" s="19" t="inlineStr"/>
-      <c r="F15" s="20" t="inlineStr">
+      <c r="E15" s="22" t="inlineStr"/>
+      <c r="F15" s="23" t="inlineStr">
         <is>
           <t>Absolute moral truth and identity are the major recurring struggles (certainty on moral truth drops in higher grades). 8th apologetics/ethics topics: reliability of scripture, pornography, social media, sexuality (problem of evil/pain reserved for high school).</t>
         </is>
       </c>
+      <c r="G15" s="24" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="16" t="inlineStr">
+      <c r="A16" s="19" t="inlineStr">
         <is>
           <t>Editorial</t>
         </is>
       </c>
-      <c r="B16" s="17" t="n">
+      <c r="B16" s="20" t="n">
         <v>12</v>
       </c>
-      <c r="C16" s="17" t="inlineStr">
+      <c r="C16" s="20" t="inlineStr">
         <is>
           <t>Would you use an end-of-year project students prepare as a group? (Yes/No/Maybe)</t>
         </is>
       </c>
-      <c r="D16" s="18" t="inlineStr">
+      <c r="D16" s="21" t="inlineStr">
         <is>
           <t>Maybe / planning to: no big end-of-year project currently (some project element in the final exam), but she wants to add an 8th-grade capstone project tied to Teaching for Transformation as students move into high school.</t>
         </is>
       </c>
-      <c r="E16" s="19" t="inlineStr"/>
-      <c r="F16" s="20" t="inlineStr">
+      <c r="E16" s="22" t="inlineStr"/>
+      <c r="F16" s="23" t="inlineStr">
         <is>
           <t>8th grade uses independent projects/research and roundtable presentations rather than a single end-of-year group project.</t>
         </is>
       </c>
+      <c r="G16" s="24" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="16" t="inlineStr">
+      <c r="A17" s="19" t="inlineStr">
         <is>
           <t>Editorial</t>
         </is>
       </c>
-      <c r="B17" s="17" t="n">
+      <c r="B17" s="20" t="n">
         <v>13</v>
       </c>
-      <c r="C17" s="17" t="inlineStr">
+      <c r="C17" s="20" t="inlineStr">
         <is>
           <t>What tools have helped with parent engagement?</t>
         </is>
       </c>
-      <c r="D17" s="18" t="inlineStr">
+      <c r="D17" s="21" t="inlineStr">
         <is>
           <t>A required number of service hours per semester draws families in (parents help get middle schoolers to service projects and often serve together around a shared passion). Also communicating the grading approach clearly at tours, and rebuilding the church connection.</t>
         </is>
       </c>
-      <c r="E17" s="19" t="inlineStr"/>
-      <c r="F17" s="20" t="inlineStr">
+      <c r="E17" s="22" t="inlineStr"/>
+      <c r="F17" s="23" t="inlineStr">
         <is>
           <t>Family devotionals as completion-based assignments; spiritual-growth assessments (student + parents + trusted adults); 7-10 min one-on-one growth conversations with EVERY middle schooler (~115/grade).</t>
         </is>
       </c>
+      <c r="G17" s="24" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="16" t="inlineStr">
+      <c r="A18" s="19" t="inlineStr">
         <is>
           <t>Editorial</t>
         </is>
       </c>
-      <c r="B18" s="17" t="n">
+      <c r="B18" s="20" t="n">
         <v>14</v>
       </c>
-      <c r="C18" s="17" t="inlineStr">
+      <c r="C18" s="20" t="inlineStr">
         <is>
           <t>What is your school's homework policy (by grade)?</t>
         </is>
       </c>
-      <c r="D18" s="18" t="inlineStr">
+      <c r="D18" s="21" t="inlineStr">
         <is>
           <t>Not directly addressed in this interview.</t>
         </is>
       </c>
-      <c r="E18" s="19" t="inlineStr"/>
-      <c r="F18" s="20" t="inlineStr">
+      <c r="E18" s="22" t="inlineStr"/>
+      <c r="F18" s="23" t="inlineStr">
         <is>
           <t>Not directly addressed (family devotionals are completion-based home assignments).</t>
         </is>
       </c>
+      <c r="G18" s="24" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="16" t="inlineStr">
+      <c r="A19" s="19" t="inlineStr">
         <is>
           <t>Production</t>
         </is>
       </c>
-      <c r="B19" s="17" t="n">
+      <c r="B19" s="20" t="n">
         <v>15</v>
       </c>
-      <c r="C19" s="17" t="inlineStr">
+      <c r="C19" s="20" t="inlineStr">
         <is>
           <t>What videos do you currently show, and how do you use them?</t>
         </is>
       </c>
-      <c r="D19" s="18" t="inlineStr">
+      <c r="D19" s="21" t="inlineStr">
         <is>
           <t>Right Now Media and YouTube clips; one recurring activity has students take a Christian song and build a Bible-study object lesson around it. All videos are vetted by the teacher/administrator before showing.</t>
         </is>
       </c>
-      <c r="E19" s="19" t="inlineStr"/>
-      <c r="F19" s="20" t="inlineStr">
+      <c r="E19" s="22" t="inlineStr"/>
+      <c r="F19" s="23" t="inlineStr">
         <is>
           <t>Not directly addressed (media engagement targeted to 3-7 min).</t>
         </is>
       </c>
+      <c r="G19" s="24" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="16" t="inlineStr">
+      <c r="A20" s="19" t="inlineStr">
         <is>
           <t>Production</t>
         </is>
       </c>
-      <c r="B20" s="17" t="n">
+      <c r="B20" s="20" t="n">
         <v>16</v>
       </c>
-      <c r="C20" s="17" t="inlineStr">
+      <c r="C20" s="20" t="inlineStr">
         <is>
           <t>What length of video is most engaging? (30s-1m / 1-2m / 2-3m / 3m+)</t>
         </is>
       </c>
-      <c r="D20" s="18" t="inlineStr">
+      <c r="D20" s="21" t="inlineStr">
         <is>
           <t>Short: generally no more than ~5 minutes, with song-based clips around 1.5-2 minutes, to match attention spans.</t>
         </is>
       </c>
-      <c r="E20" s="19" t="inlineStr">
+      <c r="E20" s="22" t="inlineStr">
         <is>
           <t>Songs feel too juvenile for upper elementary (5th); prefer known 'brand name' worship songs (e.g., Forrest Frank).</t>
         </is>
       </c>
-      <c r="F20" s="20" t="inlineStr">
+      <c r="F20" s="23" t="inlineStr">
         <is>
           <t>Media/video engagement targeted at 3-7 minutes.</t>
         </is>
       </c>
+      <c r="G20" s="24" t="inlineStr">
+        <is>
+          <t>G5 uses some of our videos and supplements with others she finds herself.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="16" t="inlineStr">
+      <c r="A21" s="19" t="inlineStr">
         <is>
           <t>Production</t>
         </is>
       </c>
-      <c r="B21" s="17" t="n">
+      <c r="B21" s="20" t="n">
         <v>17</v>
       </c>
-      <c r="C21" s="17" t="inlineStr">
+      <c r="C21" s="20" t="inlineStr">
         <is>
           <t>What types of visuals are most effective for middle schoolers?</t>
         </is>
       </c>
-      <c r="D21" s="18" t="inlineStr">
+      <c r="D21" s="21" t="inlineStr">
         <is>
           <t>Real-life, relatable people (not cartoons); charts and graphs, family trees, timelines, historical artwork/renderings, primary documents, archaeological images, and maps. She favors visuals students can see themselves in.</t>
         </is>
       </c>
-      <c r="E21" s="19" t="inlineStr">
+      <c r="E21" s="22" t="inlineStr">
         <is>
           <t>Classical/fine-art images didn't land — kids didn't like/understand the classical art in the Intro to Jesus unit (2nd).</t>
         </is>
       </c>
-      <c r="F21" s="20" t="inlineStr">
+      <c r="F21" s="23" t="inlineStr">
         <is>
           <t>Not directly addressed. (High-school apologetics leans on beauty/aesthetics — the 'argument from beauty.')</t>
         </is>
       </c>
+      <c r="G21" s="24" t="inlineStr">
+        <is>
+          <t>G5 initially felt visuals were too young (kindergartener photos) — traced to starting with the 'Intro to Jesus' unit; the rest of the G5 visuals are age-appropriate. Need a differentiated 'Intro to Jesus' (upper vs lower elementary).</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="16" t="inlineStr">
+      <c r="A22" s="19" t="inlineStr">
         <is>
           <t>Production</t>
         </is>
       </c>
-      <c r="B22" s="17" t="n">
+      <c r="B22" s="20" t="n">
         <v>18</v>
       </c>
-      <c r="C22" s="17" t="inlineStr">
+      <c r="C22" s="20" t="inlineStr">
         <is>
           <t>Do you prefer digital assessments or printables?</t>
         </is>
       </c>
-      <c r="D22" s="18" t="inlineStr">
+      <c r="D22" s="21" t="inlineStr">
         <is>
           <t>Leaning digital: with the move to Google Classroom (year two), they are less tied to printables; students interact with lessons and submit work electronically.</t>
         </is>
       </c>
-      <c r="E22" s="19" t="inlineStr">
+      <c r="E22" s="22" t="inlineStr">
         <is>
           <t>Tried online tests; could work, but strongly dislike the auto-grader marking off for spelling (3rd, 5th). 1st still prints/uses paper TNs.</t>
         </is>
       </c>
-      <c r="F22" s="20" t="inlineStr">
+      <c r="F22" s="23" t="inlineStr">
         <is>
           <t>Reducing student devices; willing to pay more for paper. Teacher-side tech is fine; student-side tech is scrutinized.</t>
         </is>
       </c>
+      <c r="G22" s="24" t="inlineStr">
+        <is>
+          <t>No student devices at school; want PRINTABLE pre- and post-assessments for all grade levels.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="16" t="inlineStr">
+      <c r="A23" s="19" t="inlineStr">
         <is>
           <t>Production</t>
         </is>
       </c>
-      <c r="B23" s="17" t="n">
+      <c r="B23" s="20" t="n">
         <v>19</v>
       </c>
-      <c r="C23" s="17" t="inlineStr">
+      <c r="C23" s="20" t="inlineStr">
         <is>
           <t>What balance between text and visuals on a typical student page?</t>
         </is>
       </c>
-      <c r="D23" s="18" t="inlineStr">
+      <c r="D23" s="21" t="inlineStr">
         <is>
           <t>A balanced mix of text and visuals (stated explicitly). As a former English teacher she values the written word and dissecting scripture, and also sees strong value in relatable visuals.</t>
         </is>
       </c>
-      <c r="E23" s="19" t="inlineStr"/>
-      <c r="F23" s="20" t="inlineStr">
+      <c r="E23" s="22" t="inlineStr"/>
+      <c r="F23" s="23" t="inlineStr">
         <is>
           <t>Not directly addressed.</t>
         </is>
       </c>
+      <c r="G23" s="24" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="16" t="inlineStr">
+      <c r="A24" s="19" t="inlineStr">
         <is>
           <t>Production</t>
         </is>
       </c>
-      <c r="B24" s="17" t="n">
+      <c r="B24" s="20" t="n">
         <v>20</v>
       </c>
-      <c r="C24" s="17" t="inlineStr">
+      <c r="C24" s="20" t="inlineStr">
         <is>
           <t>What would make a middle schooler pick up the curriculum rather than see it as 'just another textbook'?</t>
         </is>
       </c>
-      <c r="D24" s="18" t="inlineStr">
+      <c r="D24" s="21" t="inlineStr">
         <is>
           <t>Relatable, real-world visuals plus the teacher's presentation and enthusiasm. Avoiding dry, workbook-feeling material; keeping it discussion-driven and engaging. The teacher's delivery makes a big difference.</t>
         </is>
       </c>
-      <c r="E24" s="19" t="inlineStr"/>
-      <c r="F24" s="20" t="inlineStr">
+      <c r="E24" s="22" t="inlineStr"/>
+      <c r="F24" s="23" t="inlineStr">
         <is>
           <t>Not directly addressed. (Engagement is driven by the discussion/ownership model rather than the book format.)</t>
         </is>
       </c>
+      <c r="G24" s="24" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="16" t="inlineStr">
+      <c r="A25" s="19" t="inlineStr">
         <is>
           <t>Production</t>
         </is>
       </c>
-      <c r="B25" s="17" t="n">
+      <c r="B25" s="20" t="n">
         <v>21</v>
       </c>
-      <c r="C25" s="17" t="inlineStr">
+      <c r="C25" s="20" t="inlineStr">
         <is>
           <t>Are you limited by the amount of material you can print?</t>
         </is>
       </c>
-      <c r="D25" s="18" t="inlineStr">
+      <c r="D25" s="21" t="inlineStr">
         <is>
           <t>Not really limited. Teachers are asked to reduce paper where possible, but the school is well-resourced (budget, laptops, Google Classroom) and prints less in middle school than in elementary.</t>
         </is>
       </c>
-      <c r="E25" s="19" t="inlineStr"/>
-      <c r="F25" s="20" t="inlineStr">
+      <c r="E25" s="22" t="inlineStr"/>
+      <c r="F25" s="23" t="inlineStr">
         <is>
           <t>Opposite of print-limited — willing to raise tuition to cover paper costs.</t>
         </is>
       </c>
+      <c r="G25" s="24" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="16" t="inlineStr">
+      <c r="A26" s="19" t="inlineStr">
         <is>
           <t>Production</t>
         </is>
       </c>
-      <c r="B26" s="17" t="n">
+      <c r="B26" s="20" t="n">
         <v>22</v>
       </c>
-      <c r="C26" s="17" t="inlineStr">
+      <c r="C26" s="20" t="inlineStr">
         <is>
           <t>If an activity required non-standard supplies (e.g., food), would the school provide funds or would the teacher?</t>
         </is>
       </c>
-      <c r="D26" s="18" t="inlineStr">
+      <c r="D26" s="21" t="inlineStr">
         <is>
           <t>The school provides funds. Teachers have money set aside each year for curriculum and supplies; she orders what they need and tracks spending. In nine years she has never told a teacher 'no' to a resource request.</t>
         </is>
       </c>
-      <c r="E26" s="19" t="inlineStr"/>
-      <c r="F26" s="20" t="inlineStr">
+      <c r="E26" s="22" t="inlineStr"/>
+      <c r="F26" s="23" t="inlineStr">
         <is>
           <t>Not directly addressed.</t>
         </is>
       </c>
+      <c r="G26" s="24" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="16" t="inlineStr">
-        <is>
-          <t>Additional (Extra Time)</t>
-        </is>
-      </c>
-      <c r="B27" s="17" t="n">
+      <c r="A27" s="19" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B27" s="20" t="n">
         <v>23</v>
       </c>
-      <c r="C27" s="17" t="inlineStr">
+      <c r="C27" s="20" t="inlineStr">
         <is>
           <t>After 20 minutes of essential material, how much additional time would you like optional material to fill?</t>
         </is>
       </c>
-      <c r="D27" s="18" t="inlineStr">
+      <c r="D27" s="21" t="inlineStr">
         <is>
           <t>Since class is mostly discussion-based, if the core lesson runs about 20 minutes, guided discussion can take the majority of the remaining class time.</t>
         </is>
       </c>
-      <c r="E27" s="19" t="inlineStr"/>
-      <c r="F27" s="20" t="inlineStr">
+      <c r="E27" s="22" t="inlineStr"/>
+      <c r="F27" s="23" t="inlineStr">
         <is>
           <t>Block schedule: 75-min sessions every other day (effective ~65-70 min after a mandatory 5-10 min reading period). Direct instruction kept to &lt;=20 min, then discussion/activities fill the rest.</t>
         </is>
       </c>
+      <c r="G27" s="24" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="16" t="inlineStr">
-        <is>
-          <t>Additional (Extra Time)</t>
-        </is>
-      </c>
-      <c r="B28" s="17" t="n">
+      <c r="A28" s="19" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B28" s="20" t="n">
         <v>24</v>
       </c>
-      <c r="C28" s="17" t="inlineStr">
+      <c r="C28" s="20" t="inlineStr">
         <is>
           <t>Would you be interested in a multi-subject Timeline centered on Bible events (with optional Empires, Literature, Music/Arts, People, Inventions, clickable summaries and media)?</t>
         </is>
       </c>
-      <c r="D28" s="18" t="inlineStr">
+      <c r="D28" s="21" t="inlineStr">
         <is>
           <t>Not asked verbatim, but very likely yes: she strongly values timelines (built family trees and displayed a Bible timeline so students could see how events were organized) and finds chronology a real challenge for students.</t>
         </is>
       </c>
-      <c r="E28" s="19" t="inlineStr"/>
-      <c r="F28" s="20" t="inlineStr">
+      <c r="E28" s="22" t="inlineStr"/>
+      <c r="F28" s="23" t="inlineStr">
         <is>
           <t>Not asked verbatim; OT/NT survey (6th/7th) plus the Casket-Empty mnemonic already organize scripture into a cohesive meta-narrative, so a Bible-events timeline is philosophically aligned.</t>
         </is>
       </c>
+      <c r="G28" s="24" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="16" t="inlineStr">
-        <is>
-          <t>Additional (Extra Time)</t>
-        </is>
-      </c>
-      <c r="B29" s="17" t="n">
+      <c r="A29" s="19" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B29" s="20" t="n">
         <v>25</v>
       </c>
-      <c r="C29" s="17" t="inlineStr">
+      <c r="C29" s="20" t="inlineStr">
         <is>
           <t>Approximately how many minutes of screen time/technology would you permit in Bible class?</t>
         </is>
       </c>
-      <c r="D29" s="18" t="inlineStr">
+      <c r="D29" s="21" t="inlineStr">
         <is>
           <t>No specific number given; screen time is intentionally limited and balanced across the day rather than used continuously.</t>
         </is>
       </c>
-      <c r="E29" s="19" t="inlineStr"/>
-      <c r="F29" s="20" t="inlineStr">
+      <c r="E29" s="22" t="inlineStr"/>
+      <c r="F29" s="23" t="inlineStr">
         <is>
           <t>Minimizing — phone-free environment and reduced Chromebook use across the board.</t>
         </is>
       </c>
+      <c r="G29" s="24" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="16" t="inlineStr">
-        <is>
-          <t>Additional (Extra Time)</t>
-        </is>
-      </c>
-      <c r="B30" s="17" t="n">
+      <c r="A30" s="19" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B30" s="20" t="n">
         <v>26</v>
       </c>
-      <c r="C30" s="17" t="inlineStr">
+      <c r="C30" s="20" t="inlineStr">
         <is>
           <t>What tools have you found most effective for encouraging Bible reading at home?</t>
         </is>
       </c>
-      <c r="D30" s="18" t="inlineStr">
+      <c r="D30" s="21" t="inlineStr">
         <is>
           <t>Not directly addressed in this interview.</t>
         </is>
       </c>
-      <c r="E30" s="19" t="inlineStr">
+      <c r="E30" s="22" t="inlineStr">
         <is>
           <t>Ask: memory-verse SONGS with HAND MOTIONS (3rd, 4th; 3rd finds her own now). Hand motions aid retention even MS/HS per admin Melissa.</t>
         </is>
       </c>
-      <c r="F30" s="20" t="inlineStr">
+      <c r="F30" s="23" t="inlineStr">
         <is>
           <t>Family devotionals plus a mandatory 5-10 min reading period at the start of every core class.</t>
         </is>
       </c>
+      <c r="G30" s="24" t="inlineStr">
+        <is>
+          <t>G1 can't cover all unit material, so prefers ONE memory verse per unit instead of two (use the week-2 tested verse). One G1 teacher is improvising ASL hand motions to aid memory.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
-      <c r="A31" s="16" t="inlineStr">
-        <is>
-          <t>Additional (Extra Time)</t>
-        </is>
-      </c>
-      <c r="B31" s="17" t="n">
+      <c r="A31" s="19" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B31" s="20" t="n">
         <v>27</v>
       </c>
-      <c r="C31" s="17" t="inlineStr">
+      <c r="C31" s="20" t="inlineStr">
         <is>
           <t>If the curriculum offered an optional human sexuality unit, how would you use it?</t>
         </is>
       </c>
-      <c r="D31" s="18" t="inlineStr">
+      <c r="D31" s="21" t="inlineStr">
         <is>
           <t>They would not teach it at school; human sexuality is treated as a parent matter and left entirely to parents. They already skip such lessons (e.g., a unit 10 in the 8th-grade book) and coordinate with teachers to do so.</t>
         </is>
       </c>
-      <c r="E31" s="19" t="inlineStr"/>
-      <c r="F31" s="20" t="inlineStr">
+      <c r="E31" s="22" t="inlineStr"/>
+      <c r="F31" s="23" t="inlineStr">
         <is>
           <t>No dedicated MS human sexuality unit; addresses behavioral purity and orientation generally, with a senior 'theology of the body' course. Sexuality is touched within 8th-grade apologetics/ethics.</t>
         </is>
       </c>
+      <c r="G31" s="24" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="16" t="inlineStr">
-        <is>
-          <t>Additional (Extra Time)</t>
-        </is>
-      </c>
-      <c r="B32" s="17" t="n">
+      <c r="A32" s="19" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B32" s="20" t="n">
         <v>28</v>
       </c>
-      <c r="C32" s="17" t="inlineStr">
+      <c r="C32" s="20" t="inlineStr">
         <is>
           <t>Would you be interested in a separate Logic course, primarily taught through videos and reinforced with worksheets?</t>
         </is>
       </c>
-      <c r="D32" s="18" t="inlineStr">
+      <c r="D32" s="21" t="inlineStr">
         <is>
           <t>Yes / interested, but video-based delivery matters: teachers would likely need videos of someone presenting the material to feel comfortable, rather than lecture- or worksheet-only.</t>
         </is>
       </c>
-      <c r="E32" s="19" t="inlineStr"/>
-      <c r="F32" s="20" t="inlineStr">
+      <c r="E32" s="22" t="inlineStr"/>
+      <c r="F32" s="23" t="inlineStr">
         <is>
           <t>STRONG YES — wants to add an informal logic course to middle school if a smooth, usable curriculum exists. DeepRoots offered optional 7th/8th logic materials (Jacob to send). 5th grade already framed as the 'logic phase.'</t>
         </is>
       </c>
+      <c r="G32" s="24" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="16" t="inlineStr">
-        <is>
-          <t>Additional (Extra Time)</t>
-        </is>
-      </c>
-      <c r="B33" s="17" t="n">
+      <c r="A33" s="19" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B33" s="20" t="n">
         <v>29</v>
       </c>
-      <c r="C33" s="17" t="inlineStr">
+      <c r="C33" s="20" t="inlineStr">
         <is>
           <t>With 5 minutes of independent reading + 15 minutes of teaching/engagement, would you use optional deeper material? What engagements?</t>
         </is>
       </c>
-      <c r="D33" s="18" t="inlineStr">
+      <c r="D33" s="21" t="inlineStr">
         <is>
           <t>Yes. She likes a ~5-minute reflection/journaling opening, then a lesson (~20 minutes total), then discussion. Engagements: discussion, journaling/reflection, returning to scripture, and partner work.</t>
         </is>
       </c>
-      <c r="E33" s="19" t="inlineStr"/>
-      <c r="F33" s="20" t="inlineStr">
+      <c r="E33" s="22" t="inlineStr"/>
+      <c r="F33" s="23" t="inlineStr">
         <is>
           <t>Already runs a mandatory 5-10 min reading period at the start of core classes, then discussion/inquiry (Harkness) and extension. Engagements: discussion, independent projects, presentations.</t>
         </is>
       </c>
+      <c r="G33" s="24" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="16" t="inlineStr">
-        <is>
-          <t>Additional (Extra Time)</t>
-        </is>
-      </c>
-      <c r="B34" s="17" t="n">
+      <c r="A34" s="19" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B34" s="20" t="n">
         <v>30</v>
       </c>
-      <c r="C34" s="17" t="inlineStr">
+      <c r="C34" s="20" t="inlineStr">
         <is>
           <t>How important is handling a printable reference book (Course Pack) vs. an online reference?</t>
         </is>
       </c>
-      <c r="D34" s="18" t="inlineStr">
+      <c r="D34" s="21" t="inlineStr">
         <is>
           <t>Mixed, leaning digital with the Google Classroom move, but she still values the written word and dissecting scripture, so there is real value in a text reference for some students.</t>
         </is>
       </c>
-      <c r="E34" s="19" t="inlineStr"/>
-      <c r="F34" s="20" t="inlineStr">
+      <c r="E34" s="22" t="inlineStr"/>
+      <c r="F34" s="23" t="inlineStr">
         <is>
           <t>Leans toward paper/print (willing to raise tuition for paper; actively reducing screens).</t>
         </is>
       </c>
+      <c r="G34" s="24" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="16" t="inlineStr">
-        <is>
-          <t>Additional (Extra Time)</t>
-        </is>
-      </c>
-      <c r="B35" s="17" t="n">
+      <c r="A35" s="19" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B35" s="20" t="n">
         <v>31</v>
       </c>
-      <c r="C35" s="17" t="inlineStr">
+      <c r="C35" s="20" t="inlineStr">
         <is>
           <t>Individual quiet work vs. group activity: which do you prefer? Which do students prefer?</t>
         </is>
       </c>
-      <c r="D35" s="18" t="inlineStr">
+      <c r="D35" s="21" t="inlineStr">
         <is>
           <t>Group/discussion for both. Independent Bible study is hard for middle schoolers because they are not yet fluent in scripture, so guided, discussion-heavy classes are essential.</t>
         </is>
       </c>
-      <c r="E35" s="19" t="inlineStr"/>
-      <c r="F35" s="20" t="inlineStr">
+      <c r="E35" s="22" t="inlineStr"/>
+      <c r="F35" s="23" t="inlineStr">
         <is>
           <t>Discussion/group (Harkness) is central, alongside independent projects; both, but discussion-forward.</t>
         </is>
       </c>
+      <c r="G35" s="24" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" s="16" t="inlineStr">
-        <is>
-          <t>Additional (Extra Time)</t>
-        </is>
-      </c>
-      <c r="B36" s="17" t="n">
+      <c r="A36" s="19" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B36" s="20" t="n">
         <v>32</v>
       </c>
-      <c r="C36" s="17" t="inlineStr">
+      <c r="C36" s="20" t="inlineStr">
         <is>
           <t>As a teacher, what does your ideal Bible lesson look like?</t>
         </is>
       </c>
-      <c r="D36" s="18" t="inlineStr">
+      <c r="D36" s="21" t="inlineStr">
         <is>
           <t>A short intro/review (~5 min), a focused lesson (~15-20 min), then discussion and partner work, woven with historical/cultural context and personal reflection/application, kept moving so students stay engaged.</t>
         </is>
       </c>
-      <c r="E36" s="19" t="inlineStr"/>
-      <c r="F36" s="20" t="inlineStr">
+      <c r="E36" s="22" t="inlineStr"/>
+      <c r="F36" s="23" t="inlineStr">
         <is>
           <t>Reading period -&gt; direct instruction (&lt;=20 min, ideally ~17) -&gt; Harkness discussion and extension, built around inquiry and ownership.</t>
         </is>
       </c>
+      <c r="G36" s="24" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="16" t="inlineStr">
-        <is>
-          <t>Additional (Extra Time)</t>
-        </is>
-      </c>
-      <c r="B37" s="17" t="n">
+      <c r="A37" s="19" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B37" s="20" t="n">
         <v>33</v>
       </c>
-      <c r="C37" s="17" t="inlineStr">
+      <c r="C37" s="20" t="inlineStr">
         <is>
           <t>How do you measure the success of a curriculum?</t>
         </is>
       </c>
-      <c r="D37" s="18" t="inlineStr">
+      <c r="D37" s="21" t="inlineStr">
         <is>
           <t>Students being able to apply scripture to their own lives. Her tests always ended with an open-ended prompt: 'write an example of how this applies to your life,' which showed movement from head knowledge to heart knowledge.</t>
         </is>
       </c>
-      <c r="E37" s="19" t="inlineStr">
+      <c r="E37" s="22" t="inlineStr">
         <is>
           <t>Auto-graded online assessments promising but the spelling penalty undermines them. Kids using Bibles more is a win (2nd).</t>
         </is>
       </c>
-      <c r="F37" s="20" t="inlineStr">
+      <c r="F37" s="23" t="inlineStr">
         <is>
           <t>Wheaton global student assessment 3x/year (worldview/formation metrics); spiritual-growth assessments + 1:1 conferences; adding faith-outcome questions to the 5-year alumni survey. North star: 'resilient disciples.'</t>
         </is>
       </c>
+      <c r="G37" s="24" t="inlineStr">
+        <is>
+          <t>G4 test questions too verbose / over some students' heads (esp. unchurched); matching &amp; fill-in-the-blank easier than short answer. Want printable pre/post assessments for all grades.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
-      <c r="A38" s="16" t="inlineStr">
-        <is>
-          <t>Additional (Extra Time)</t>
-        </is>
-      </c>
-      <c r="B38" s="17" t="n">
+      <c r="A38" s="19" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B38" s="20" t="n">
         <v>34</v>
       </c>
-      <c r="C38" s="17" t="inlineStr">
+      <c r="C38" s="20" t="inlineStr">
         <is>
           <t>Are there visual styles/trends/design approaches that would NOT work well?</t>
         </is>
       </c>
-      <c r="D38" s="18" t="inlineStr">
+      <c r="D38" s="21" t="inlineStr">
         <is>
           <t>Younger, cartoon-style depictions of people. Middle schoolers are moving away from cartoons and want to see real people they can relate to.</t>
         </is>
       </c>
-      <c r="E38" s="19" t="inlineStr">
+      <c r="E38" s="22" t="inlineStr">
         <is>
           <t>Avoid classical/fine-art visuals for this age; avoid juvenile song styles for upper elementary; scrolling-heavy layout is a negative (5th).</t>
         </is>
       </c>
-      <c r="F38" s="20" t="inlineStr">
+      <c r="F38" s="23" t="inlineStr">
         <is>
           <t>Not directly addressed.</t>
         </is>
       </c>
+      <c r="G38" s="24" t="inlineStr">
+        <is>
+          <t>Photos of kindergarteners don't relate for older grades; need age-appropriate visuals (and a differentiated 'Intro to Jesus' unit).</t>
+        </is>
+      </c>
     </row>
     <row r="39">
-      <c r="A39" s="16" t="inlineStr">
-        <is>
-          <t>Additional (Extra Time)</t>
-        </is>
-      </c>
-      <c r="B39" s="17" t="n">
+      <c r="A39" s="19" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B39" s="20" t="n">
         <v>35</v>
       </c>
-      <c r="C39" s="17" t="inlineStr">
+      <c r="C39" s="20" t="inlineStr">
         <is>
           <t>What short videos would be helpful to supplement your teaching?</t>
         </is>
       </c>
-      <c r="D39" s="18" t="inlineStr">
+      <c r="D39" s="21" t="inlineStr">
         <is>
           <t>Real-world application videos most of all, plus videos that hit the key idea and introduce/give context to the subject; relatable real-world visuals resonate most.</t>
         </is>
       </c>
-      <c r="E39" s="19" t="inlineStr"/>
-      <c r="F39" s="20" t="inlineStr">
+      <c r="E39" s="22" t="inlineStr"/>
+      <c r="F39" s="23" t="inlineStr">
         <is>
           <t>Media kept to 3-7 min; strong interest in content built on the 'argument from beauty'/aesthetics.</t>
         </is>
       </c>
+      <c r="G39" s="24" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="16" t="inlineStr">
-        <is>
-          <t>Additional (Extra Time)</t>
-        </is>
-      </c>
-      <c r="B40" s="17" t="n">
+      <c r="A40" s="19" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B40" s="20" t="n">
         <v>36</v>
       </c>
-      <c r="C40" s="17" t="inlineStr">
+      <c r="C40" s="20" t="inlineStr">
         <is>
           <t>On a scale of 1-10, how would you rate role-play activities for engagement?</t>
         </is>
       </c>
-      <c r="D40" s="18" t="inlineStr">
+      <c r="D40" s="21" t="inlineStr">
         <is>
           <t>Low. Middle schoolers often dislike being put on the spot, especially about personal faith. Fine as an optional tool if a class is open to it, but not something to use consistently.</t>
         </is>
       </c>
-      <c r="E40" s="19" t="inlineStr">
+      <c r="E40" s="22" t="inlineStr">
         <is>
           <t>Role play rates HIGH here — kids love it, Good Samaritan role play a standout (3rd). NOTE: opposite of the middle-school signal.</t>
         </is>
       </c>
-      <c r="F40" s="20" t="inlineStr">
+      <c r="F40" s="23" t="inlineStr">
         <is>
           <t>Not directly addressed.</t>
         </is>
       </c>
+      <c r="G40" s="24" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" s="16" t="inlineStr">
-        <is>
-          <t>Additional (Extra Time)</t>
-        </is>
-      </c>
-      <c r="B41" s="17" t="n">
+      <c r="A41" s="19" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B41" s="20" t="n">
         <v>37</v>
       </c>
-      <c r="C41" s="17" t="inlineStr">
+      <c r="C41" s="20" t="inlineStr">
         <is>
           <t>What elements of a Bible curriculum do you NOT prefer?</t>
         </is>
       </c>
-      <c r="D41" s="18" t="inlineStr">
+      <c r="D41" s="21" t="inlineStr">
         <is>
           <t>Dry, boring material; 'just words on a page' or 'the next lesson in the workbook,' which brings the wrong attitude into class.</t>
         </is>
       </c>
-      <c r="E41" s="19" t="inlineStr"/>
-      <c r="F41" s="20" t="inlineStr">
+      <c r="E41" s="22" t="inlineStr"/>
+      <c r="F41" s="23" t="inlineStr">
         <is>
           <t>A content-regurgitation-only model (wants soul-level reflection, not facts-for-a-grade); excessive student screen time.</t>
         </is>
       </c>
+      <c r="G41" s="24" t="inlineStr"/>
     </row>
     <row r="42">
-      <c r="A42" s="16" t="inlineStr">
-        <is>
-          <t>Additional (Extra Time)</t>
-        </is>
-      </c>
-      <c r="B42" s="17" t="n">
+      <c r="A42" s="19" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B42" s="20" t="n">
         <v>38</v>
       </c>
-      <c r="C42" s="17" t="inlineStr">
+      <c r="C42" s="20" t="inlineStr">
         <is>
           <t>What gets and holds your students' attention in Bible class?</t>
         </is>
       </c>
-      <c r="D42" s="18" t="inlineStr">
+      <c r="D42" s="21" t="inlineStr">
         <is>
           <t>Engaging discussion and debate, relatable real-world visuals and video, the teacher's enthusiasm and presentation, and variety that keeps the lesson moving.</t>
         </is>
       </c>
-      <c r="E42" s="19" t="inlineStr"/>
-      <c r="F42" s="20" t="inlineStr">
+      <c r="E42" s="22" t="inlineStr"/>
+      <c r="F42" s="23" t="inlineStr">
         <is>
           <t>Harkness discussion, student ownership/inquiry, short direct-instruction bursts, and countering short-form-media habits (the gap between how long students CAN vs. WILL attend).</t>
         </is>
       </c>
+      <c r="G42" s="24" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" s="16" t="inlineStr">
-        <is>
-          <t>Additional (Extra Time)</t>
-        </is>
-      </c>
-      <c r="B43" s="17" t="n">
+      <c r="A43" s="19" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B43" s="20" t="n">
         <v>39</v>
       </c>
-      <c r="C43" s="17" t="inlineStr">
+      <c r="C43" s="20" t="inlineStr">
         <is>
           <t>What would a middle school Bible curriculum look like that is easy to teach and impactful?</t>
         </is>
       </c>
-      <c r="D43" s="18" t="inlineStr">
+      <c r="D43" s="21" t="inlineStr">
         <is>
           <t>The same depth and teacher resources DeepRoots provides for elementary, but with a different presentation model for middle school: not dry, relatable visuals, discussion-driven, rich in reflection/application and historical/cultural context, with enough ready-made resources that teachers are not building and vetting everything themselves. (They currently use DeepRoots for grades 3-5.)</t>
         </is>
       </c>
-      <c r="E43" s="19" t="inlineStr"/>
-      <c r="F43" s="20" t="inlineStr">
+      <c r="E43" s="22" t="inlineStr"/>
+      <c r="F43" s="23" t="inlineStr">
         <is>
           <t>Discussion/inquiry-driven with clear division targets (6th OT survey, 7th NT survey, 8th worldview/apologetics/ethics), the Casket-Empty meta-narrative, an integrated logic track, common assessments enabling reteach/extension, minimal student screens, aiming at 'resilient disciples.'</t>
+        </is>
+      </c>
+      <c r="G43" s="24" t="inlineStr">
+        <is>
+          <t>A slideshow version where teachers choose which slides to show/hide; a single Bible translation (moving to all ESV); Teaching Essentials organized by unit with elements inline; printable pre/post assessments; age-appropriate visuals.</t>
         </is>
       </c>
     </row>
@@ -1856,914 +1989,914 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="21" t="inlineStr">
+      <c r="A1" s="25" t="inlineStr">
         <is>
           <t>Interview with Meredith Arldt</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="22" t="inlineStr">
+      <c r="A2" s="26" t="inlineStr">
         <is>
           <t>Aliso Viejo Christian School (CA)  |  teacher / administrator  |  interviewed 2026-09-24</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="22" t="inlineStr">
+      <c r="A3" s="26" t="inlineStr">
         <is>
           <t>Attendees: Troy Winkler, Pat Williamson, Nancy Wood, Tammy Plett, Lisa Van Vlear</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>Section</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="10" t="inlineStr">
         <is>
           <t>Q#</t>
         </is>
       </c>
-      <c r="C5" s="9" t="inlineStr">
+      <c r="C5" s="10" t="inlineStr">
         <is>
           <t>Question</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="D5" s="10" t="inlineStr">
         <is>
           <t>Answer</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="19" t="inlineStr">
         <is>
           <t>Marketing &amp; Sales</t>
         </is>
       </c>
-      <c r="B6" s="17" t="n">
+      <c r="B6" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="C6" s="17" t="inlineStr">
+      <c r="C6" s="20" t="inlineStr">
         <is>
           <t>How does your school categorize Middle School / Junior High (5-8, 6-8, 7-8)?</t>
         </is>
       </c>
-      <c r="D6" s="17" t="inlineStr">
+      <c r="D6" s="20" t="inlineStr">
         <is>
           <t>Middle school is 6th, 7th, and 8th grade (6-8).</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="19" t="inlineStr">
         <is>
           <t>Marketing &amp; Sales</t>
         </is>
       </c>
-      <c r="B7" s="17" t="n">
+      <c r="B7" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="C7" s="17" t="inlineStr">
+      <c r="C7" s="20" t="inlineStr">
         <is>
           <t>What are the primary differences between a 6th, 7th, and 8th grade student (developmentally, spiritually, emotionally)?</t>
         </is>
       </c>
-      <c r="D7" s="17" t="inlineStr">
+      <c r="D7" s="20" t="inlineStr">
         <is>
           <t>Students begin actively questioning their own faith and searching for personal identity ('why do I believe what I believe?') amid outside influences like social media. 6th graders want independence but still want the safety net of mom and dad, going back and forth. 7th graders like to push and challenge ('their own little beast'). 8th graders can get 'a little too big for their own.' Spirituality is hard at this age because it is not always tangible.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="16" t="inlineStr">
+      <c r="A8" s="19" t="inlineStr">
         <is>
           <t>Marketing &amp; Sales</t>
         </is>
       </c>
-      <c r="B8" s="17" t="n">
+      <c r="B8" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="C8" s="17" t="inlineStr">
+      <c r="C8" s="20" t="inlineStr">
         <is>
           <t>How do you best reach both churched and unchurched students? Is this an issue for you? What works best?</t>
         </is>
       </c>
-      <c r="D8" s="17" t="inlineStr">
+      <c r="D8" s="20" t="inlineStr">
         <is>
           <t>About 60% of the school population identifies with a church home; 40% do not. They are intentional about corporate worship (for some students it is their only weekly worship) and adopted the Teaching for Transformation framework (from CASE) two years ago, with flex projects that put faith into action. They are also rebuilding the historically broken bridge with their associated church to connect unchurched families with pastoral staff.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="16" t="inlineStr">
+      <c r="A9" s="19" t="inlineStr">
         <is>
           <t>Marketing &amp; Sales</t>
         </is>
       </c>
-      <c r="B9" s="17" t="n">
+      <c r="B9" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="C9" s="17" t="inlineStr">
+      <c r="C9" s="20" t="inlineStr">
         <is>
           <t>What do you like or dislike about your current Bible curriculum?</t>
         </is>
       </c>
-      <c r="D9" s="17" t="inlineStr">
+      <c r="D9" s="20" t="inlineStr">
         <is>
           <t>Currently workbook-based: Purposeful Design (Daring Deliverers), and Positive Action (Character Counts for 6th, Wise Up for 8th). All workbook-based and 'pretty dry and boring.' The goal is to keep Bible from feeling like just another academic class and to focus on students' hearts, not grade their faith.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="16" t="inlineStr">
+      <c r="A10" s="19" t="inlineStr">
         <is>
           <t>Marketing &amp; Sales</t>
         </is>
       </c>
-      <c r="B10" s="17" t="n">
+      <c r="B10" s="20" t="n">
         <v>5</v>
       </c>
-      <c r="C10" s="17" t="inlineStr">
+      <c r="C10" s="20" t="inlineStr">
         <is>
           <t>What elements would you like to see in it each week?</t>
         </is>
       </c>
-      <c r="D10" s="17" t="inlineStr">
+      <c r="D10" s="20" t="inlineStr">
         <is>
           <t>More reflection and personal application ('how does this resonate with you today? what do we do with this?'). Historical and cultural context so students understand the significance of events. Treat biblical figures and events as real history, not 'stories' or fairy tales.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="16" t="inlineStr">
+      <c r="A11" s="19" t="inlineStr">
         <is>
           <t>Marketing &amp; Sales</t>
         </is>
       </c>
-      <c r="B11" s="17" t="n">
+      <c r="B11" s="20" t="n">
         <v>6</v>
       </c>
-      <c r="C11" s="17" t="inlineStr">
+      <c r="C11" s="20" t="inlineStr">
         <is>
           <t>What core ideals do you wish each student left your class identifying with?</t>
         </is>
       </c>
-      <c r="D11" s="17" t="inlineStr">
+      <c r="D11" s="20" t="inlineStr">
         <is>
           <t>Moving from head knowledge to heart knowledge; a real identity in Christ; applying scripture to their own lives; striving to be the best version of who God created them to be.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="16" t="inlineStr">
+      <c r="A12" s="19" t="inlineStr">
         <is>
           <t>Marketing &amp; Sales</t>
         </is>
       </c>
-      <c r="B12" s="17" t="n">
+      <c r="B12" s="20" t="n">
         <v>7</v>
       </c>
-      <c r="C12" s="17" t="inlineStr">
+      <c r="C12" s="20" t="inlineStr">
         <is>
           <t>What types of resources (videos, activities, etc.) are most helpful for you as a teacher?</t>
         </is>
       </c>
-      <c r="D12" s="17" t="inlineStr">
+      <c r="D12" s="20" t="inlineStr">
         <is>
           <t>Short videos (about 1.5-5 minutes), historical family trees, Bible timelines, primary documents, original-language (Greek/Hebrew) references, and cultural/archaeological references (e.g., an archaeological Bible). Note: curating and vetting these is the most time-consuming part for teachers, so ready-made, vetted resources would help most.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="16" t="inlineStr">
+      <c r="A13" s="19" t="inlineStr">
         <is>
           <t>Editorial</t>
         </is>
       </c>
-      <c r="B13" s="17" t="n">
+      <c r="B13" s="20" t="n">
         <v>8</v>
       </c>
-      <c r="C13" s="17" t="inlineStr">
+      <c r="C13" s="20" t="inlineStr">
         <is>
           <t>How many minutes can students pay attention to teaching, reading, discussion, activities?</t>
         </is>
       </c>
-      <c r="D13" s="17" t="inlineStr">
+      <c r="D13" s="20" t="inlineStr">
         <is>
           <t>Lecture/teaching is kept to 15-20 minutes max before moving into discussion. A typical rhythm is a ~5-minute intro/review, a 10-15 minute lesson, then discussion. Class is mostly discussion-based; some reading.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="16" t="inlineStr">
+      <c r="A14" s="19" t="inlineStr">
         <is>
           <t>Editorial</t>
         </is>
       </c>
-      <c r="B14" s="17" t="n">
+      <c r="B14" s="20" t="n">
         <v>9</v>
       </c>
-      <c r="C14" s="17" t="inlineStr">
+      <c r="C14" s="20" t="inlineStr">
         <is>
           <t>What kind of engagements do students enjoy most (by grade)?</t>
         </is>
       </c>
-      <c r="D14" s="17" t="inlineStr">
+      <c r="D14" s="20" t="inlineStr">
         <is>
           <t>Discussion-based work and things they can relate to (real-world video, relatable visuals), partner work, and interactive questions. Discussion is the biggest draw across middle school.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="16" t="inlineStr">
+      <c r="A15" s="19" t="inlineStr">
         <is>
           <t>Editorial</t>
         </is>
       </c>
-      <c r="B15" s="17" t="n">
+      <c r="B15" s="20" t="n">
         <v>10</v>
       </c>
-      <c r="C15" s="17" t="inlineStr">
+      <c r="C15" s="20" t="inlineStr">
         <is>
           <t>How do you use screens and technology in your classroom?</t>
         </is>
       </c>
-      <c r="D15" s="17" t="inlineStr">
+      <c r="D15" s="20" t="inlineStr">
         <is>
           <t>Google Classroom is the platform; laptops are provided but screen time is intentionally limited (parents appreciate this). Currently projection-based; installing BenQ interactive smartboards by January (grant-funded), with teacher training.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="16" t="inlineStr">
+      <c r="A16" s="19" t="inlineStr">
         <is>
           <t>Editorial</t>
         </is>
       </c>
-      <c r="B16" s="17" t="n">
+      <c r="B16" s="20" t="n">
         <v>11</v>
       </c>
-      <c r="C16" s="17" t="inlineStr">
+      <c r="C16" s="20" t="inlineStr">
         <is>
           <t>What questions/issues do you see students wrestling with (by grade)?</t>
         </is>
       </c>
-      <c r="D16" s="17" t="inlineStr">
+      <c r="D16" s="20" t="inlineStr">
         <is>
           <t>Reconciling 'what my parents taught me' with 'what do I actually believe'; identity in Christ versus societal pressure and peer acceptance; influence of social media; and nominal Christianity ('Christian in name only') where students know the Sunday-school answers but haven't moved it from head to heart.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="16" t="inlineStr">
+      <c r="A17" s="19" t="inlineStr">
         <is>
           <t>Editorial</t>
         </is>
       </c>
-      <c r="B17" s="17" t="n">
+      <c r="B17" s="20" t="n">
         <v>12</v>
       </c>
-      <c r="C17" s="17" t="inlineStr">
+      <c r="C17" s="20" t="inlineStr">
         <is>
           <t>Would you use an end-of-year project students prepare as a group? (Yes/No/Maybe)</t>
         </is>
       </c>
-      <c r="D17" s="17" t="inlineStr">
+      <c r="D17" s="20" t="inlineStr">
         <is>
           <t>Maybe / planning to: no big end-of-year project currently (some project element in the final exam), but she wants to add an 8th-grade capstone project tied to Teaching for Transformation as students move into high school.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="16" t="inlineStr">
+      <c r="A18" s="19" t="inlineStr">
         <is>
           <t>Editorial</t>
         </is>
       </c>
-      <c r="B18" s="17" t="n">
+      <c r="B18" s="20" t="n">
         <v>13</v>
       </c>
-      <c r="C18" s="17" t="inlineStr">
+      <c r="C18" s="20" t="inlineStr">
         <is>
           <t>What tools have helped with parent engagement?</t>
         </is>
       </c>
-      <c r="D18" s="17" t="inlineStr">
+      <c r="D18" s="20" t="inlineStr">
         <is>
           <t>A required number of service hours per semester draws families in (parents help get middle schoolers to service projects and often serve together around a shared passion). Also communicating the grading approach clearly at tours, and rebuilding the church connection.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="16" t="inlineStr">
+      <c r="A19" s="19" t="inlineStr">
         <is>
           <t>Editorial</t>
         </is>
       </c>
-      <c r="B19" s="17" t="n">
+      <c r="B19" s="20" t="n">
         <v>14</v>
       </c>
-      <c r="C19" s="17" t="inlineStr">
+      <c r="C19" s="20" t="inlineStr">
         <is>
           <t>What is your school's homework policy (by grade)?</t>
         </is>
       </c>
-      <c r="D19" s="17" t="inlineStr">
+      <c r="D19" s="20" t="inlineStr">
         <is>
           <t>Not directly addressed in this interview.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="16" t="inlineStr">
+      <c r="A20" s="19" t="inlineStr">
         <is>
           <t>Production</t>
         </is>
       </c>
-      <c r="B20" s="17" t="n">
+      <c r="B20" s="20" t="n">
         <v>15</v>
       </c>
-      <c r="C20" s="17" t="inlineStr">
+      <c r="C20" s="20" t="inlineStr">
         <is>
           <t>What videos do you currently show, and how do you use them?</t>
         </is>
       </c>
-      <c r="D20" s="17" t="inlineStr">
+      <c r="D20" s="20" t="inlineStr">
         <is>
           <t>Right Now Media and YouTube clips; one recurring activity has students take a Christian song and build a Bible-study object lesson around it. All videos are vetted by the teacher/administrator before showing.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="16" t="inlineStr">
+      <c r="A21" s="19" t="inlineStr">
         <is>
           <t>Production</t>
         </is>
       </c>
-      <c r="B21" s="17" t="n">
+      <c r="B21" s="20" t="n">
         <v>16</v>
       </c>
-      <c r="C21" s="17" t="inlineStr">
+      <c r="C21" s="20" t="inlineStr">
         <is>
           <t>What length of video is most engaging? (30s-1m / 1-2m / 2-3m / 3m+)</t>
         </is>
       </c>
-      <c r="D21" s="17" t="inlineStr">
+      <c r="D21" s="20" t="inlineStr">
         <is>
           <t>Short: generally no more than ~5 minutes, with song-based clips around 1.5-2 minutes, to match attention spans.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="16" t="inlineStr">
+      <c r="A22" s="19" t="inlineStr">
         <is>
           <t>Production</t>
         </is>
       </c>
-      <c r="B22" s="17" t="n">
+      <c r="B22" s="20" t="n">
         <v>17</v>
       </c>
-      <c r="C22" s="17" t="inlineStr">
+      <c r="C22" s="20" t="inlineStr">
         <is>
           <t>What types of visuals are most effective for middle schoolers?</t>
         </is>
       </c>
-      <c r="D22" s="17" t="inlineStr">
+      <c r="D22" s="20" t="inlineStr">
         <is>
           <t>Real-life, relatable people (not cartoons); charts and graphs, family trees, timelines, historical artwork/renderings, primary documents, archaeological images, and maps. She favors visuals students can see themselves in.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="16" t="inlineStr">
+      <c r="A23" s="19" t="inlineStr">
         <is>
           <t>Production</t>
         </is>
       </c>
-      <c r="B23" s="17" t="n">
+      <c r="B23" s="20" t="n">
         <v>18</v>
       </c>
-      <c r="C23" s="17" t="inlineStr">
+      <c r="C23" s="20" t="inlineStr">
         <is>
           <t>Do you prefer digital assessments or printables?</t>
         </is>
       </c>
-      <c r="D23" s="17" t="inlineStr">
+      <c r="D23" s="20" t="inlineStr">
         <is>
           <t>Leaning digital: with the move to Google Classroom (year two), they are less tied to printables; students interact with lessons and submit work electronically.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="16" t="inlineStr">
+      <c r="A24" s="19" t="inlineStr">
         <is>
           <t>Production</t>
         </is>
       </c>
-      <c r="B24" s="17" t="n">
+      <c r="B24" s="20" t="n">
         <v>19</v>
       </c>
-      <c r="C24" s="17" t="inlineStr">
+      <c r="C24" s="20" t="inlineStr">
         <is>
           <t>What balance between text and visuals on a typical student page?</t>
         </is>
       </c>
-      <c r="D24" s="17" t="inlineStr">
+      <c r="D24" s="20" t="inlineStr">
         <is>
           <t>A balanced mix of text and visuals (stated explicitly). As a former English teacher she values the written word and dissecting scripture, and also sees strong value in relatable visuals.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="16" t="inlineStr">
+      <c r="A25" s="19" t="inlineStr">
         <is>
           <t>Production</t>
         </is>
       </c>
-      <c r="B25" s="17" t="n">
+      <c r="B25" s="20" t="n">
         <v>20</v>
       </c>
-      <c r="C25" s="17" t="inlineStr">
+      <c r="C25" s="20" t="inlineStr">
         <is>
           <t>What would make a middle schooler pick up the curriculum rather than see it as 'just another textbook'?</t>
         </is>
       </c>
-      <c r="D25" s="17" t="inlineStr">
+      <c r="D25" s="20" t="inlineStr">
         <is>
           <t>Relatable, real-world visuals plus the teacher's presentation and enthusiasm. Avoiding dry, workbook-feeling material; keeping it discussion-driven and engaging. The teacher's delivery makes a big difference.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="16" t="inlineStr">
+      <c r="A26" s="19" t="inlineStr">
         <is>
           <t>Production</t>
         </is>
       </c>
-      <c r="B26" s="17" t="n">
+      <c r="B26" s="20" t="n">
         <v>21</v>
       </c>
-      <c r="C26" s="17" t="inlineStr">
+      <c r="C26" s="20" t="inlineStr">
         <is>
           <t>Are you limited by the amount of material you can print?</t>
         </is>
       </c>
-      <c r="D26" s="17" t="inlineStr">
+      <c r="D26" s="20" t="inlineStr">
         <is>
           <t>Not really limited. Teachers are asked to reduce paper where possible, but the school is well-resourced (budget, laptops, Google Classroom) and prints less in middle school than in elementary.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="16" t="inlineStr">
+      <c r="A27" s="19" t="inlineStr">
         <is>
           <t>Production</t>
         </is>
       </c>
-      <c r="B27" s="17" t="n">
+      <c r="B27" s="20" t="n">
         <v>22</v>
       </c>
-      <c r="C27" s="17" t="inlineStr">
+      <c r="C27" s="20" t="inlineStr">
         <is>
           <t>If an activity required non-standard supplies (e.g., food), would the school provide funds or would the teacher?</t>
         </is>
       </c>
-      <c r="D27" s="17" t="inlineStr">
+      <c r="D27" s="20" t="inlineStr">
         <is>
           <t>The school provides funds. Teachers have money set aside each year for curriculum and supplies; she orders what they need and tracks spending. In nine years she has never told a teacher 'no' to a resource request.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="16" t="inlineStr">
-        <is>
-          <t>Additional (Extra Time)</t>
-        </is>
-      </c>
-      <c r="B28" s="17" t="n">
+      <c r="A28" s="19" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B28" s="20" t="n">
         <v>23</v>
       </c>
-      <c r="C28" s="17" t="inlineStr">
+      <c r="C28" s="20" t="inlineStr">
         <is>
           <t>After 20 minutes of essential material, how much additional time would you like optional material to fill?</t>
         </is>
       </c>
-      <c r="D28" s="17" t="inlineStr">
+      <c r="D28" s="20" t="inlineStr">
         <is>
           <t>Since class is mostly discussion-based, if the core lesson runs about 20 minutes, guided discussion can take the majority of the remaining class time.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="16" t="inlineStr">
-        <is>
-          <t>Additional (Extra Time)</t>
-        </is>
-      </c>
-      <c r="B29" s="17" t="n">
+      <c r="A29" s="19" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B29" s="20" t="n">
         <v>24</v>
       </c>
-      <c r="C29" s="17" t="inlineStr">
+      <c r="C29" s="20" t="inlineStr">
         <is>
           <t>Would you be interested in a multi-subject Timeline centered on Bible events (with optional Empires, Literature, Music/Arts, People, Inventions, clickable summaries and media)?</t>
         </is>
       </c>
-      <c r="D29" s="17" t="inlineStr">
+      <c r="D29" s="20" t="inlineStr">
         <is>
           <t>Not asked verbatim, but very likely yes: she strongly values timelines (built family trees and displayed a Bible timeline so students could see how events were organized) and finds chronology a real challenge for students.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="16" t="inlineStr">
-        <is>
-          <t>Additional (Extra Time)</t>
-        </is>
-      </c>
-      <c r="B30" s="17" t="n">
+      <c r="A30" s="19" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B30" s="20" t="n">
         <v>25</v>
       </c>
-      <c r="C30" s="17" t="inlineStr">
+      <c r="C30" s="20" t="inlineStr">
         <is>
           <t>Approximately how many minutes of screen time/technology would you permit in Bible class?</t>
         </is>
       </c>
-      <c r="D30" s="17" t="inlineStr">
+      <c r="D30" s="20" t="inlineStr">
         <is>
           <t>No specific number given; screen time is intentionally limited and balanced across the day rather than used continuously.</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="16" t="inlineStr">
-        <is>
-          <t>Additional (Extra Time)</t>
-        </is>
-      </c>
-      <c r="B31" s="17" t="n">
+      <c r="A31" s="19" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B31" s="20" t="n">
         <v>26</v>
       </c>
-      <c r="C31" s="17" t="inlineStr">
+      <c r="C31" s="20" t="inlineStr">
         <is>
           <t>What tools have you found most effective for encouraging Bible reading at home?</t>
         </is>
       </c>
-      <c r="D31" s="17" t="inlineStr">
+      <c r="D31" s="20" t="inlineStr">
         <is>
           <t>Not directly addressed in this interview.</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="16" t="inlineStr">
-        <is>
-          <t>Additional (Extra Time)</t>
-        </is>
-      </c>
-      <c r="B32" s="17" t="n">
+      <c r="A32" s="19" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B32" s="20" t="n">
         <v>27</v>
       </c>
-      <c r="C32" s="17" t="inlineStr">
+      <c r="C32" s="20" t="inlineStr">
         <is>
           <t>If the curriculum offered an optional human sexuality unit, how would you use it?</t>
         </is>
       </c>
-      <c r="D32" s="17" t="inlineStr">
+      <c r="D32" s="20" t="inlineStr">
         <is>
           <t>They would not teach it at school; human sexuality is treated as a parent matter and left entirely to parents. They already skip such lessons (e.g., a unit 10 in the 8th-grade book) and coordinate with teachers to do so.</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="16" t="inlineStr">
-        <is>
-          <t>Additional (Extra Time)</t>
-        </is>
-      </c>
-      <c r="B33" s="17" t="n">
+      <c r="A33" s="19" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B33" s="20" t="n">
         <v>28</v>
       </c>
-      <c r="C33" s="17" t="inlineStr">
+      <c r="C33" s="20" t="inlineStr">
         <is>
           <t>Would you be interested in a separate Logic course, primarily taught through videos and reinforced with worksheets?</t>
         </is>
       </c>
-      <c r="D33" s="17" t="inlineStr">
+      <c r="D33" s="20" t="inlineStr">
         <is>
           <t>Yes / interested, but video-based delivery matters: teachers would likely need videos of someone presenting the material to feel comfortable, rather than lecture- or worksheet-only.</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="16" t="inlineStr">
-        <is>
-          <t>Additional (Extra Time)</t>
-        </is>
-      </c>
-      <c r="B34" s="17" t="n">
+      <c r="A34" s="19" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B34" s="20" t="n">
         <v>29</v>
       </c>
-      <c r="C34" s="17" t="inlineStr">
+      <c r="C34" s="20" t="inlineStr">
         <is>
           <t>With 5 minutes of independent reading + 15 minutes of teaching/engagement, would you use optional deeper material? What engagements?</t>
         </is>
       </c>
-      <c r="D34" s="17" t="inlineStr">
+      <c r="D34" s="20" t="inlineStr">
         <is>
           <t>Yes. She likes a ~5-minute reflection/journaling opening, then a lesson (~20 minutes total), then discussion. Engagements: discussion, journaling/reflection, returning to scripture, and partner work.</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="16" t="inlineStr">
-        <is>
-          <t>Additional (Extra Time)</t>
-        </is>
-      </c>
-      <c r="B35" s="17" t="n">
+      <c r="A35" s="19" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B35" s="20" t="n">
         <v>30</v>
       </c>
-      <c r="C35" s="17" t="inlineStr">
+      <c r="C35" s="20" t="inlineStr">
         <is>
           <t>How important is handling a printable reference book (Course Pack) vs. an online reference?</t>
         </is>
       </c>
-      <c r="D35" s="17" t="inlineStr">
+      <c r="D35" s="20" t="inlineStr">
         <is>
           <t>Mixed, leaning digital with the Google Classroom move, but she still values the written word and dissecting scripture, so there is real value in a text reference for some students.</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="16" t="inlineStr">
-        <is>
-          <t>Additional (Extra Time)</t>
-        </is>
-      </c>
-      <c r="B36" s="17" t="n">
+      <c r="A36" s="19" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B36" s="20" t="n">
         <v>31</v>
       </c>
-      <c r="C36" s="17" t="inlineStr">
+      <c r="C36" s="20" t="inlineStr">
         <is>
           <t>Individual quiet work vs. group activity: which do you prefer? Which do students prefer?</t>
         </is>
       </c>
-      <c r="D36" s="17" t="inlineStr">
+      <c r="D36" s="20" t="inlineStr">
         <is>
           <t>Group/discussion for both. Independent Bible study is hard for middle schoolers because they are not yet fluent in scripture, so guided, discussion-heavy classes are essential.</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="16" t="inlineStr">
-        <is>
-          <t>Additional (Extra Time)</t>
-        </is>
-      </c>
-      <c r="B37" s="17" t="n">
+      <c r="A37" s="19" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B37" s="20" t="n">
         <v>32</v>
       </c>
-      <c r="C37" s="17" t="inlineStr">
+      <c r="C37" s="20" t="inlineStr">
         <is>
           <t>As a teacher, what does your ideal Bible lesson look like?</t>
         </is>
       </c>
-      <c r="D37" s="17" t="inlineStr">
+      <c r="D37" s="20" t="inlineStr">
         <is>
           <t>A short intro/review (~5 min), a focused lesson (~15-20 min), then discussion and partner work, woven with historical/cultural context and personal reflection/application, kept moving so students stay engaged.</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="16" t="inlineStr">
-        <is>
-          <t>Additional (Extra Time)</t>
-        </is>
-      </c>
-      <c r="B38" s="17" t="n">
+      <c r="A38" s="19" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B38" s="20" t="n">
         <v>33</v>
       </c>
-      <c r="C38" s="17" t="inlineStr">
+      <c r="C38" s="20" t="inlineStr">
         <is>
           <t>How do you measure the success of a curriculum?</t>
         </is>
       </c>
-      <c r="D38" s="17" t="inlineStr">
+      <c r="D38" s="20" t="inlineStr">
         <is>
           <t>Students being able to apply scripture to their own lives. Her tests always ended with an open-ended prompt: 'write an example of how this applies to your life,' which showed movement from head knowledge to heart knowledge.</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="16" t="inlineStr">
-        <is>
-          <t>Additional (Extra Time)</t>
-        </is>
-      </c>
-      <c r="B39" s="17" t="n">
+      <c r="A39" s="19" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B39" s="20" t="n">
         <v>34</v>
       </c>
-      <c r="C39" s="17" t="inlineStr">
+      <c r="C39" s="20" t="inlineStr">
         <is>
           <t>Are there visual styles/trends/design approaches that would NOT work well?</t>
         </is>
       </c>
-      <c r="D39" s="17" t="inlineStr">
+      <c r="D39" s="20" t="inlineStr">
         <is>
           <t>Younger, cartoon-style depictions of people. Middle schoolers are moving away from cartoons and want to see real people they can relate to.</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="16" t="inlineStr">
-        <is>
-          <t>Additional (Extra Time)</t>
-        </is>
-      </c>
-      <c r="B40" s="17" t="n">
+      <c r="A40" s="19" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B40" s="20" t="n">
         <v>35</v>
       </c>
-      <c r="C40" s="17" t="inlineStr">
+      <c r="C40" s="20" t="inlineStr">
         <is>
           <t>What short videos would be helpful to supplement your teaching?</t>
         </is>
       </c>
-      <c r="D40" s="17" t="inlineStr">
+      <c r="D40" s="20" t="inlineStr">
         <is>
           <t>Real-world application videos most of all, plus videos that hit the key idea and introduce/give context to the subject; relatable real-world visuals resonate most.</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="16" t="inlineStr">
-        <is>
-          <t>Additional (Extra Time)</t>
-        </is>
-      </c>
-      <c r="B41" s="17" t="n">
+      <c r="A41" s="19" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B41" s="20" t="n">
         <v>36</v>
       </c>
-      <c r="C41" s="17" t="inlineStr">
+      <c r="C41" s="20" t="inlineStr">
         <is>
           <t>On a scale of 1-10, how would you rate role-play activities for engagement?</t>
         </is>
       </c>
-      <c r="D41" s="17" t="inlineStr">
+      <c r="D41" s="20" t="inlineStr">
         <is>
           <t>Low. Middle schoolers often dislike being put on the spot, especially about personal faith. Fine as an optional tool if a class is open to it, but not something to use consistently.</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="16" t="inlineStr">
-        <is>
-          <t>Additional (Extra Time)</t>
-        </is>
-      </c>
-      <c r="B42" s="17" t="n">
+      <c r="A42" s="19" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B42" s="20" t="n">
         <v>37</v>
       </c>
-      <c r="C42" s="17" t="inlineStr">
+      <c r="C42" s="20" t="inlineStr">
         <is>
           <t>What elements of a Bible curriculum do you NOT prefer?</t>
         </is>
       </c>
-      <c r="D42" s="17" t="inlineStr">
+      <c r="D42" s="20" t="inlineStr">
         <is>
           <t>Dry, boring material; 'just words on a page' or 'the next lesson in the workbook,' which brings the wrong attitude into class.</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="16" t="inlineStr">
-        <is>
-          <t>Additional (Extra Time)</t>
-        </is>
-      </c>
-      <c r="B43" s="17" t="n">
+      <c r="A43" s="19" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B43" s="20" t="n">
         <v>38</v>
       </c>
-      <c r="C43" s="17" t="inlineStr">
+      <c r="C43" s="20" t="inlineStr">
         <is>
           <t>What gets and holds your students' attention in Bible class?</t>
         </is>
       </c>
-      <c r="D43" s="17" t="inlineStr">
+      <c r="D43" s="20" t="inlineStr">
         <is>
           <t>Engaging discussion and debate, relatable real-world visuals and video, the teacher's enthusiasm and presentation, and variety that keeps the lesson moving.</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="16" t="inlineStr">
-        <is>
-          <t>Additional (Extra Time)</t>
-        </is>
-      </c>
-      <c r="B44" s="17" t="n">
+      <c r="A44" s="19" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B44" s="20" t="n">
         <v>39</v>
       </c>
-      <c r="C44" s="17" t="inlineStr">
+      <c r="C44" s="20" t="inlineStr">
         <is>
           <t>What would a middle school Bible curriculum look like that is easy to teach and impactful?</t>
         </is>
       </c>
-      <c r="D44" s="17" t="inlineStr">
+      <c r="D44" s="20" t="inlineStr">
         <is>
           <t>The same depth and teacher resources DeepRoots provides for elementary, but with a different presentation model for middle school: not dry, relatable visuals, discussion-driven, rich in reflection/application and historical/cultural context, with enough ready-made resources that teachers are not building and vetting everything themselves. (They currently use DeepRoots for grades 3-5.)</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="23" t="inlineStr">
+      <c r="A46" s="27" t="inlineStr">
         <is>
           <t>DEEPROOTS TEAM TAKEAWAYS — Meredith Arldt interview (said or unsaid)</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="24" t="inlineStr">
+      <c r="A47" s="28" t="inlineStr">
         <is>
           <t>Team member (attendee)</t>
         </is>
       </c>
-      <c r="B47" s="24" t="inlineStr"/>
-      <c r="C47" s="24" t="inlineStr"/>
-      <c r="D47" s="24" t="inlineStr">
+      <c r="B47" s="28" t="inlineStr"/>
+      <c r="C47" s="28" t="inlineStr"/>
+      <c r="D47" s="28" t="inlineStr">
         <is>
           <t>Takeaways / observations</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="25" t="inlineStr">
+      <c r="A48" s="29" t="inlineStr">
         <is>
           <t>Troy Winkler</t>
         </is>
       </c>
-      <c r="B48" s="25" t="inlineStr"/>
-      <c r="C48" s="25" t="inlineStr"/>
-      <c r="D48" s="25" t="inlineStr">
+      <c r="B48" s="29" t="inlineStr"/>
+      <c r="C48" s="29" t="inlineStr"/>
+      <c r="D48" s="29" t="inlineStr">
         <is>
           <t>That we need to have content relatable to that age group - video and illustrations should be more modern and age appropriate instead of cartoon animations.</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="25" t="inlineStr">
+      <c r="A49" s="29" t="inlineStr">
         <is>
           <t>Pat Williamson</t>
         </is>
       </c>
-      <c r="B49" s="25" t="inlineStr"/>
-      <c r="C49" s="25" t="inlineStr"/>
-      <c r="D49" s="25" t="inlineStr">
+      <c r="B49" s="29" t="inlineStr"/>
+      <c r="C49" s="29" t="inlineStr"/>
+      <c r="D49" s="29" t="inlineStr">
         <is>
           <t>That teachers were supplementing with outside media.</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="25" t="inlineStr">
+      <c r="A50" s="29" t="inlineStr">
         <is>
           <t>Nancy Wood</t>
         </is>
       </c>
-      <c r="B50" s="25" t="inlineStr"/>
-      <c r="C50" s="25" t="inlineStr"/>
-      <c r="D50" s="25" t="inlineStr">
+      <c r="B50" s="29" t="inlineStr"/>
+      <c r="C50" s="29" t="inlineStr"/>
+      <c r="D50" s="29" t="inlineStr">
         <is>
           <t>She was all about discussions. I think adding additional optional discussion questions would be great (and not take too much of our time) for schools like hers that have 45 minutes. Based on what she was saying, we could also do more teaching through video as well. I agree with Lisa that we could work on having more ways to assess the materials, such as IBS and MV. Maybe don't make those optional? They aren't in lower grades.</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="25" t="inlineStr">
+      <c r="A51" s="29" t="inlineStr">
         <is>
           <t>Tammy Plett</t>
         </is>
       </c>
-      <c r="B51" s="25" t="inlineStr"/>
-      <c r="C51" s="25" t="inlineStr"/>
-      <c r="D51" s="25" t="inlineStr">
+      <c r="B51" s="29" t="inlineStr"/>
+      <c r="C51" s="29" t="inlineStr"/>
+      <c r="D51" s="29" t="inlineStr">
         <is>
           <t>I loved hearing that the workbook-based curricula were 'boring and dry' in her opinion. Note that they want to move away from 'cartoon' videos and visuals at this age and look for something more realistic, relatable and like them. That is something we have heard before and should keep in mind. Love that they started Teaching for Transformation a couple of years ago and are looking to put faith into action; that is something we can and should mesh with, maybe offering our own ideas for service projects that tie into our lessons as a Digging Deeper option. Also noted that she likes to make the historical aspect come alive so they can relate; that is where our Titus Kennedy archaeological pieces come into play. It was helpful to hear how long she thinks students at this age can sit and listen to a lecture before they check out. Good to know that discussion is helpful at this age.</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="25" t="inlineStr">
+      <c r="A52" s="29" t="inlineStr">
         <is>
           <t>Lisa Van Vlear</t>
         </is>
       </c>
-      <c r="B52" s="25" t="inlineStr"/>
-      <c r="C52" s="25" t="inlineStr"/>
-      <c r="D52" s="25" t="inlineStr">
+      <c r="B52" s="29" t="inlineStr"/>
+      <c r="C52" s="29" t="inlineStr"/>
+      <c r="D52" s="29" t="inlineStr">
         <is>
           <t>Meredith mentioned several times the importance of reflection and application for the students. 'How does this affect me today?' She stressed discussion and that if the lesson were 15 minutes, the rest of class time would be devoted to discussion. She was also a fan of archaeological pictures and historical context. I appreciated that since we do that well. I don't think we should shy away from that. Since Bible class needs to be given a grade, I'm wondering if we provide enough ways for a teacher to assign a grade. We have optional quizzes and tests. Sounds like they give points for scripture memorization. I'd like to hear from a teacher who's currently teaching our G7 what she is using to give scores. We do have the IBS component that could be given a score. Given all that she mentioned, I'd be really curious to get her thoughts if she would give G7 a good look.</t>
         </is>
@@ -2801,898 +2934,898 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="26" t="inlineStr">
+      <c r="A1" s="30" t="inlineStr">
         <is>
           <t>Interview with Will Weaver</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="22" t="inlineStr">
+      <c r="A2" s="26" t="inlineStr">
         <is>
           <t>Des Moines Christian School (IA)  |  Head of Spiritual Formation (admin)  |  interviewed 2026-09-30</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="22" t="inlineStr">
+      <c r="A3" s="26" t="inlineStr">
         <is>
           <t>Attendees: Troy Winkler, Pat Williamson, Tammy Plett, Lisa Van Vlear, Jacob Waller</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="inlineStr">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Section</t>
         </is>
       </c>
-      <c r="B5" s="11" t="inlineStr">
+      <c r="B5" s="12" t="inlineStr">
         <is>
           <t>Q#</t>
         </is>
       </c>
-      <c r="C5" s="11" t="inlineStr">
+      <c r="C5" s="12" t="inlineStr">
         <is>
           <t>Question</t>
         </is>
       </c>
-      <c r="D5" s="11" t="inlineStr">
+      <c r="D5" s="12" t="inlineStr">
         <is>
           <t>Answer</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="19" t="inlineStr">
         <is>
           <t>Marketing &amp; Sales</t>
         </is>
       </c>
-      <c r="B6" s="17" t="n">
+      <c r="B6" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="C6" s="17" t="inlineStr">
+      <c r="C6" s="20" t="inlineStr">
         <is>
           <t>How does your school categorize Middle School / Junior High (5-8, 6-8, 7-8)?</t>
         </is>
       </c>
-      <c r="D6" s="17" t="inlineStr">
+      <c r="D6" s="20" t="inlineStr">
         <is>
           <t>Currently MS = 6-8 (this year 68 students, next year 58). Next year pulling 5th grade into a unified 5-8 middle school; 5th treated as the 'logic phase.'</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="19" t="inlineStr">
         <is>
           <t>Marketing &amp; Sales</t>
         </is>
       </c>
-      <c r="B7" s="17" t="n">
+      <c r="B7" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="C7" s="17" t="inlineStr">
+      <c r="C7" s="20" t="inlineStr">
         <is>
           <t>What are the primary differences between a 6th, 7th, and 8th grade student (developmentally, spiritually, emotionally)?</t>
         </is>
       </c>
-      <c r="D7" s="17" t="inlineStr">
+      <c r="D7" s="20" t="inlineStr">
         <is>
           <t>5th graders have more in common with 7th/8th than K-1; ready for inquiry ('why' questions), not just content. Discussion capacity grows: ~20 min in 6th, 25-30 min in 7th-8th as they take ownership. Student certainty on absolute moral truth tends to DECREASE in higher grades.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="16" t="inlineStr">
+      <c r="A8" s="19" t="inlineStr">
         <is>
           <t>Marketing &amp; Sales</t>
         </is>
       </c>
-      <c r="B8" s="17" t="n">
+      <c r="B8" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="C8" s="17" t="inlineStr">
+      <c r="C8" s="20" t="inlineStr">
         <is>
           <t>How do you best reach both churched and unchurched students? Is this an issue for you? What works best?</t>
         </is>
       </c>
-      <c r="D8" s="17" t="inlineStr">
+      <c r="D8" s="20" t="inlineStr">
         <is>
           <t>Covenantal school, ~1,650 students; long-time DeepRoots elementary user (~40 students). Program goal across EE-12: 'resilient disciples' who own their faith.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="16" t="inlineStr">
+      <c r="A9" s="19" t="inlineStr">
         <is>
           <t>Marketing &amp; Sales</t>
         </is>
       </c>
-      <c r="B9" s="17" t="n">
+      <c r="B9" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="C9" s="17" t="inlineStr">
+      <c r="C9" s="20" t="inlineStr">
         <is>
           <t>What do you like or dislike about your current Bible curriculum?</t>
         </is>
       </c>
-      <c r="D9" s="17" t="inlineStr">
+      <c r="D9" s="20" t="inlineStr">
         <is>
           <t>MS Bible progression: 6th = Old Testament survey, 7th = New Testament survey, 8th = intro to worldview, apologetics &amp; ethics. Uses the Casket-Empty(-Open) mnemonic across 6/7/8 to anchor stories into scripture's meta-narrative. Long-time DeepRoots user in elementary.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="16" t="inlineStr">
+      <c r="A10" s="19" t="inlineStr">
         <is>
           <t>Marketing &amp; Sales</t>
         </is>
       </c>
-      <c r="B10" s="17" t="n">
+      <c r="B10" s="20" t="n">
         <v>5</v>
       </c>
-      <c r="C10" s="17" t="inlineStr">
+      <c r="C10" s="20" t="inlineStr">
         <is>
           <t>What elements would you like to see in it each week?</t>
         </is>
       </c>
-      <c r="D10" s="17" t="inlineStr">
+      <c r="D10" s="20" t="inlineStr">
         <is>
           <t>Discussion-based (Harkness) conversations, growing in length by grade; family devotionals; common assessments across 6-8 enabling reteach + extension; a mandatory 5-10 min reading period at the start of every core class.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="16" t="inlineStr">
+      <c r="A11" s="19" t="inlineStr">
         <is>
           <t>Marketing &amp; Sales</t>
         </is>
       </c>
-      <c r="B11" s="17" t="n">
+      <c r="B11" s="20" t="n">
         <v>6</v>
       </c>
-      <c r="C11" s="17" t="inlineStr">
+      <c r="C11" s="20" t="inlineStr">
         <is>
           <t>What core ideals do you wish each student left your class identifying with?</t>
         </is>
       </c>
-      <c r="D11" s="17" t="inlineStr">
+      <c r="D11" s="20" t="inlineStr">
         <is>
           <t>'Resilient disciples' who take ownership of their faith — able to take doctrine apart and put it back together, and articulate not just what it says but 'where it sits in your soul,' rather than regurgitate content for a grade.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="16" t="inlineStr">
+      <c r="A12" s="19" t="inlineStr">
         <is>
           <t>Marketing &amp; Sales</t>
         </is>
       </c>
-      <c r="B12" s="17" t="n">
+      <c r="B12" s="20" t="n">
         <v>7</v>
       </c>
-      <c r="C12" s="17" t="inlineStr">
+      <c r="C12" s="20" t="inlineStr">
         <is>
           <t>What types of resources (videos, activities, etc.) are most helpful for you as a teacher?</t>
         </is>
       </c>
-      <c r="D12" s="17" t="inlineStr">
+      <c r="D12" s="20" t="inlineStr">
         <is>
           <t>Strong interest in usable Logic materials (DeepRoots offered optional 7th/8th logic sets). Casket-Empty mnemonic; Wheaton global student assessment 3x/year for worldview metrics.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="16" t="inlineStr">
+      <c r="A13" s="19" t="inlineStr">
         <is>
           <t>Editorial</t>
         </is>
       </c>
-      <c r="B13" s="17" t="n">
+      <c r="B13" s="20" t="n">
         <v>8</v>
       </c>
-      <c r="C13" s="17" t="inlineStr">
+      <c r="C13" s="20" t="inlineStr">
         <is>
           <t>How many minutes can students pay attention to teaching, reading, discussion, activities?</t>
         </is>
       </c>
-      <c r="D13" s="17" t="inlineStr">
+      <c r="D13" s="20" t="inlineStr">
         <is>
           <t>Targets: direct instruction 20 min or less (ideally ~17); media 3-7 min; student activities 15-20 min before attention drops. Discussions: ~20 min (6th), 25-30 min (7th-8th).</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="16" t="inlineStr">
+      <c r="A14" s="19" t="inlineStr">
         <is>
           <t>Editorial</t>
         </is>
       </c>
-      <c r="B14" s="17" t="n">
+      <c r="B14" s="20" t="n">
         <v>9</v>
       </c>
-      <c r="C14" s="17" t="inlineStr">
+      <c r="C14" s="20" t="inlineStr">
         <is>
           <t>What kind of engagements do students enjoy most (by grade)?</t>
         </is>
       </c>
-      <c r="D14" s="17" t="inlineStr">
+      <c r="D14" s="20" t="inlineStr">
         <is>
           <t>Harkness roundtable discussions (even mixed 6-8 for high performers), independent projects/research, and presentations, especially in 8th.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="16" t="inlineStr">
+      <c r="A15" s="19" t="inlineStr">
         <is>
           <t>Editorial</t>
         </is>
       </c>
-      <c r="B15" s="17" t="n">
+      <c r="B15" s="20" t="n">
         <v>10</v>
       </c>
-      <c r="C15" s="17" t="inlineStr">
+      <c r="C15" s="20" t="inlineStr">
         <is>
           <t>How do you use screens and technology in your classroom?</t>
         </is>
       </c>
-      <c r="D15" s="17" t="inlineStr">
+      <c r="D15" s="20" t="inlineStr">
         <is>
           <t>Phone-free K-12; deliberately scaling back student Chromebook use (screens promote skimming/distraction). Willing to raise tuition for paper; challenges teachers to justify student tech vs. checking a box. Distinguishes beneficial teacher-side tech from student-side.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="16" t="inlineStr">
+      <c r="A16" s="19" t="inlineStr">
         <is>
           <t>Editorial</t>
         </is>
       </c>
-      <c r="B16" s="17" t="n">
+      <c r="B16" s="20" t="n">
         <v>11</v>
       </c>
-      <c r="C16" s="17" t="inlineStr">
+      <c r="C16" s="20" t="inlineStr">
         <is>
           <t>What questions/issues do you see students wrestling with (by grade)?</t>
         </is>
       </c>
-      <c r="D16" s="17" t="inlineStr">
+      <c r="D16" s="20" t="inlineStr">
         <is>
           <t>Absolute moral truth and identity are the major recurring struggles (certainty on moral truth drops in higher grades). 8th apologetics/ethics topics: reliability of scripture, pornography, social media, sexuality (problem of evil/pain reserved for high school).</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="16" t="inlineStr">
+      <c r="A17" s="19" t="inlineStr">
         <is>
           <t>Editorial</t>
         </is>
       </c>
-      <c r="B17" s="17" t="n">
+      <c r="B17" s="20" t="n">
         <v>12</v>
       </c>
-      <c r="C17" s="17" t="inlineStr">
+      <c r="C17" s="20" t="inlineStr">
         <is>
           <t>Would you use an end-of-year project students prepare as a group? (Yes/No/Maybe)</t>
         </is>
       </c>
-      <c r="D17" s="17" t="inlineStr">
+      <c r="D17" s="20" t="inlineStr">
         <is>
           <t>8th grade uses independent projects/research and roundtable presentations rather than a single end-of-year group project.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="16" t="inlineStr">
+      <c r="A18" s="19" t="inlineStr">
         <is>
           <t>Editorial</t>
         </is>
       </c>
-      <c r="B18" s="17" t="n">
+      <c r="B18" s="20" t="n">
         <v>13</v>
       </c>
-      <c r="C18" s="17" t="inlineStr">
+      <c r="C18" s="20" t="inlineStr">
         <is>
           <t>What tools have helped with parent engagement?</t>
         </is>
       </c>
-      <c r="D18" s="17" t="inlineStr">
+      <c r="D18" s="20" t="inlineStr">
         <is>
           <t>Family devotionals as completion-based assignments; spiritual-growth assessments (student + parents + trusted adults); 7-10 min one-on-one growth conversations with EVERY middle schooler (~115/grade).</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="16" t="inlineStr">
+      <c r="A19" s="19" t="inlineStr">
         <is>
           <t>Editorial</t>
         </is>
       </c>
-      <c r="B19" s="17" t="n">
+      <c r="B19" s="20" t="n">
         <v>14</v>
       </c>
-      <c r="C19" s="17" t="inlineStr">
+      <c r="C19" s="20" t="inlineStr">
         <is>
           <t>What is your school's homework policy (by grade)?</t>
         </is>
       </c>
-      <c r="D19" s="17" t="inlineStr">
+      <c r="D19" s="20" t="inlineStr">
         <is>
           <t>Not directly addressed (family devotionals are completion-based home assignments).</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="16" t="inlineStr">
+      <c r="A20" s="19" t="inlineStr">
         <is>
           <t>Production</t>
         </is>
       </c>
-      <c r="B20" s="17" t="n">
+      <c r="B20" s="20" t="n">
         <v>15</v>
       </c>
-      <c r="C20" s="17" t="inlineStr">
+      <c r="C20" s="20" t="inlineStr">
         <is>
           <t>What videos do you currently show, and how do you use them?</t>
         </is>
       </c>
-      <c r="D20" s="17" t="inlineStr">
+      <c r="D20" s="20" t="inlineStr">
         <is>
           <t>Not directly addressed (media engagement targeted to 3-7 min).</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="16" t="inlineStr">
+      <c r="A21" s="19" t="inlineStr">
         <is>
           <t>Production</t>
         </is>
       </c>
-      <c r="B21" s="17" t="n">
+      <c r="B21" s="20" t="n">
         <v>16</v>
       </c>
-      <c r="C21" s="17" t="inlineStr">
+      <c r="C21" s="20" t="inlineStr">
         <is>
           <t>What length of video is most engaging? (30s-1m / 1-2m / 2-3m / 3m+)</t>
         </is>
       </c>
-      <c r="D21" s="17" t="inlineStr">
+      <c r="D21" s="20" t="inlineStr">
         <is>
           <t>Media/video engagement targeted at 3-7 minutes.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="16" t="inlineStr">
+      <c r="A22" s="19" t="inlineStr">
         <is>
           <t>Production</t>
         </is>
       </c>
-      <c r="B22" s="17" t="n">
+      <c r="B22" s="20" t="n">
         <v>17</v>
       </c>
-      <c r="C22" s="17" t="inlineStr">
+      <c r="C22" s="20" t="inlineStr">
         <is>
           <t>What types of visuals are most effective for middle schoolers?</t>
         </is>
       </c>
-      <c r="D22" s="17" t="inlineStr">
+      <c r="D22" s="20" t="inlineStr">
         <is>
           <t>Not directly addressed. (High-school apologetics leans on beauty/aesthetics — the 'argument from beauty.')</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="16" t="inlineStr">
+      <c r="A23" s="19" t="inlineStr">
         <is>
           <t>Production</t>
         </is>
       </c>
-      <c r="B23" s="17" t="n">
+      <c r="B23" s="20" t="n">
         <v>18</v>
       </c>
-      <c r="C23" s="17" t="inlineStr">
+      <c r="C23" s="20" t="inlineStr">
         <is>
           <t>Do you prefer digital assessments or printables?</t>
         </is>
       </c>
-      <c r="D23" s="17" t="inlineStr">
+      <c r="D23" s="20" t="inlineStr">
         <is>
           <t>Reducing student devices; willing to pay more for paper. Teacher-side tech is fine; student-side tech is scrutinized.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="16" t="inlineStr">
+      <c r="A24" s="19" t="inlineStr">
         <is>
           <t>Production</t>
         </is>
       </c>
-      <c r="B24" s="17" t="n">
+      <c r="B24" s="20" t="n">
         <v>19</v>
       </c>
-      <c r="C24" s="17" t="inlineStr">
+      <c r="C24" s="20" t="inlineStr">
         <is>
           <t>What balance between text and visuals on a typical student page?</t>
         </is>
       </c>
-      <c r="D24" s="17" t="inlineStr">
+      <c r="D24" s="20" t="inlineStr">
         <is>
           <t>Not directly addressed.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="16" t="inlineStr">
+      <c r="A25" s="19" t="inlineStr">
         <is>
           <t>Production</t>
         </is>
       </c>
-      <c r="B25" s="17" t="n">
+      <c r="B25" s="20" t="n">
         <v>20</v>
       </c>
-      <c r="C25" s="17" t="inlineStr">
+      <c r="C25" s="20" t="inlineStr">
         <is>
           <t>What would make a middle schooler pick up the curriculum rather than see it as 'just another textbook'?</t>
         </is>
       </c>
-      <c r="D25" s="17" t="inlineStr">
+      <c r="D25" s="20" t="inlineStr">
         <is>
           <t>Not directly addressed. (Engagement is driven by the discussion/ownership model rather than the book format.)</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="16" t="inlineStr">
+      <c r="A26" s="19" t="inlineStr">
         <is>
           <t>Production</t>
         </is>
       </c>
-      <c r="B26" s="17" t="n">
+      <c r="B26" s="20" t="n">
         <v>21</v>
       </c>
-      <c r="C26" s="17" t="inlineStr">
+      <c r="C26" s="20" t="inlineStr">
         <is>
           <t>Are you limited by the amount of material you can print?</t>
         </is>
       </c>
-      <c r="D26" s="17" t="inlineStr">
+      <c r="D26" s="20" t="inlineStr">
         <is>
           <t>Opposite of print-limited — willing to raise tuition to cover paper costs.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="16" t="inlineStr">
+      <c r="A27" s="19" t="inlineStr">
         <is>
           <t>Production</t>
         </is>
       </c>
-      <c r="B27" s="17" t="n">
+      <c r="B27" s="20" t="n">
         <v>22</v>
       </c>
-      <c r="C27" s="17" t="inlineStr">
+      <c r="C27" s="20" t="inlineStr">
         <is>
           <t>If an activity required non-standard supplies (e.g., food), would the school provide funds or would the teacher?</t>
         </is>
       </c>
-      <c r="D27" s="17" t="inlineStr">
+      <c r="D27" s="20" t="inlineStr">
         <is>
           <t>Not directly addressed.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="16" t="inlineStr">
-        <is>
-          <t>Additional (Extra Time)</t>
-        </is>
-      </c>
-      <c r="B28" s="17" t="n">
+      <c r="A28" s="19" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B28" s="20" t="n">
         <v>23</v>
       </c>
-      <c r="C28" s="17" t="inlineStr">
+      <c r="C28" s="20" t="inlineStr">
         <is>
           <t>After 20 minutes of essential material, how much additional time would you like optional material to fill?</t>
         </is>
       </c>
-      <c r="D28" s="17" t="inlineStr">
+      <c r="D28" s="20" t="inlineStr">
         <is>
           <t>Block schedule: 75-min sessions every other day (effective ~65-70 min after a mandatory 5-10 min reading period). Direct instruction kept to &lt;=20 min, then discussion/activities fill the rest.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="16" t="inlineStr">
-        <is>
-          <t>Additional (Extra Time)</t>
-        </is>
-      </c>
-      <c r="B29" s="17" t="n">
+      <c r="A29" s="19" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B29" s="20" t="n">
         <v>24</v>
       </c>
-      <c r="C29" s="17" t="inlineStr">
+      <c r="C29" s="20" t="inlineStr">
         <is>
           <t>Would you be interested in a multi-subject Timeline centered on Bible events (with optional Empires, Literature, Music/Arts, People, Inventions, clickable summaries and media)?</t>
         </is>
       </c>
-      <c r="D29" s="17" t="inlineStr">
+      <c r="D29" s="20" t="inlineStr">
         <is>
           <t>Not asked verbatim; OT/NT survey (6th/7th) plus the Casket-Empty mnemonic already organize scripture into a cohesive meta-narrative, so a Bible-events timeline is philosophically aligned.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="16" t="inlineStr">
-        <is>
-          <t>Additional (Extra Time)</t>
-        </is>
-      </c>
-      <c r="B30" s="17" t="n">
+      <c r="A30" s="19" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B30" s="20" t="n">
         <v>25</v>
       </c>
-      <c r="C30" s="17" t="inlineStr">
+      <c r="C30" s="20" t="inlineStr">
         <is>
           <t>Approximately how many minutes of screen time/technology would you permit in Bible class?</t>
         </is>
       </c>
-      <c r="D30" s="17" t="inlineStr">
+      <c r="D30" s="20" t="inlineStr">
         <is>
           <t>Minimizing — phone-free environment and reduced Chromebook use across the board.</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="16" t="inlineStr">
-        <is>
-          <t>Additional (Extra Time)</t>
-        </is>
-      </c>
-      <c r="B31" s="17" t="n">
+      <c r="A31" s="19" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B31" s="20" t="n">
         <v>26</v>
       </c>
-      <c r="C31" s="17" t="inlineStr">
+      <c r="C31" s="20" t="inlineStr">
         <is>
           <t>What tools have you found most effective for encouraging Bible reading at home?</t>
         </is>
       </c>
-      <c r="D31" s="17" t="inlineStr">
+      <c r="D31" s="20" t="inlineStr">
         <is>
           <t>Family devotionals plus a mandatory 5-10 min reading period at the start of every core class.</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="16" t="inlineStr">
-        <is>
-          <t>Additional (Extra Time)</t>
-        </is>
-      </c>
-      <c r="B32" s="17" t="n">
+      <c r="A32" s="19" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B32" s="20" t="n">
         <v>27</v>
       </c>
-      <c r="C32" s="17" t="inlineStr">
+      <c r="C32" s="20" t="inlineStr">
         <is>
           <t>If the curriculum offered an optional human sexuality unit, how would you use it?</t>
         </is>
       </c>
-      <c r="D32" s="17" t="inlineStr">
+      <c r="D32" s="20" t="inlineStr">
         <is>
           <t>No dedicated MS human sexuality unit; addresses behavioral purity and orientation generally, with a senior 'theology of the body' course. Sexuality is touched within 8th-grade apologetics/ethics.</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="16" t="inlineStr">
-        <is>
-          <t>Additional (Extra Time)</t>
-        </is>
-      </c>
-      <c r="B33" s="17" t="n">
+      <c r="A33" s="19" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B33" s="20" t="n">
         <v>28</v>
       </c>
-      <c r="C33" s="17" t="inlineStr">
+      <c r="C33" s="20" t="inlineStr">
         <is>
           <t>Would you be interested in a separate Logic course, primarily taught through videos and reinforced with worksheets?</t>
         </is>
       </c>
-      <c r="D33" s="17" t="inlineStr">
+      <c r="D33" s="20" t="inlineStr">
         <is>
           <t>STRONG YES — wants to add an informal logic course to middle school if a smooth, usable curriculum exists. DeepRoots offered optional 7th/8th logic materials (Jacob to send). 5th grade already framed as the 'logic phase.'</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="16" t="inlineStr">
-        <is>
-          <t>Additional (Extra Time)</t>
-        </is>
-      </c>
-      <c r="B34" s="17" t="n">
+      <c r="A34" s="19" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B34" s="20" t="n">
         <v>29</v>
       </c>
-      <c r="C34" s="17" t="inlineStr">
+      <c r="C34" s="20" t="inlineStr">
         <is>
           <t>With 5 minutes of independent reading + 15 minutes of teaching/engagement, would you use optional deeper material? What engagements?</t>
         </is>
       </c>
-      <c r="D34" s="17" t="inlineStr">
+      <c r="D34" s="20" t="inlineStr">
         <is>
           <t>Already runs a mandatory 5-10 min reading period at the start of core classes, then discussion/inquiry (Harkness) and extension. Engagements: discussion, independent projects, presentations.</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="16" t="inlineStr">
-        <is>
-          <t>Additional (Extra Time)</t>
-        </is>
-      </c>
-      <c r="B35" s="17" t="n">
+      <c r="A35" s="19" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B35" s="20" t="n">
         <v>30</v>
       </c>
-      <c r="C35" s="17" t="inlineStr">
+      <c r="C35" s="20" t="inlineStr">
         <is>
           <t>How important is handling a printable reference book (Course Pack) vs. an online reference?</t>
         </is>
       </c>
-      <c r="D35" s="17" t="inlineStr">
+      <c r="D35" s="20" t="inlineStr">
         <is>
           <t>Leans toward paper/print (willing to raise tuition for paper; actively reducing screens).</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="16" t="inlineStr">
-        <is>
-          <t>Additional (Extra Time)</t>
-        </is>
-      </c>
-      <c r="B36" s="17" t="n">
+      <c r="A36" s="19" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B36" s="20" t="n">
         <v>31</v>
       </c>
-      <c r="C36" s="17" t="inlineStr">
+      <c r="C36" s="20" t="inlineStr">
         <is>
           <t>Individual quiet work vs. group activity: which do you prefer? Which do students prefer?</t>
         </is>
       </c>
-      <c r="D36" s="17" t="inlineStr">
+      <c r="D36" s="20" t="inlineStr">
         <is>
           <t>Discussion/group (Harkness) is central, alongside independent projects; both, but discussion-forward.</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="16" t="inlineStr">
-        <is>
-          <t>Additional (Extra Time)</t>
-        </is>
-      </c>
-      <c r="B37" s="17" t="n">
+      <c r="A37" s="19" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B37" s="20" t="n">
         <v>32</v>
       </c>
-      <c r="C37" s="17" t="inlineStr">
+      <c r="C37" s="20" t="inlineStr">
         <is>
           <t>As a teacher, what does your ideal Bible lesson look like?</t>
         </is>
       </c>
-      <c r="D37" s="17" t="inlineStr">
+      <c r="D37" s="20" t="inlineStr">
         <is>
           <t>Reading period -&gt; direct instruction (&lt;=20 min, ideally ~17) -&gt; Harkness discussion and extension, built around inquiry and ownership.</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="16" t="inlineStr">
-        <is>
-          <t>Additional (Extra Time)</t>
-        </is>
-      </c>
-      <c r="B38" s="17" t="n">
+      <c r="A38" s="19" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B38" s="20" t="n">
         <v>33</v>
       </c>
-      <c r="C38" s="17" t="inlineStr">
+      <c r="C38" s="20" t="inlineStr">
         <is>
           <t>How do you measure the success of a curriculum?</t>
         </is>
       </c>
-      <c r="D38" s="17" t="inlineStr">
+      <c r="D38" s="20" t="inlineStr">
         <is>
           <t>Wheaton global student assessment 3x/year (worldview/formation metrics); spiritual-growth assessments + 1:1 conferences; adding faith-outcome questions to the 5-year alumni survey. North star: 'resilient disciples.'</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="16" t="inlineStr">
-        <is>
-          <t>Additional (Extra Time)</t>
-        </is>
-      </c>
-      <c r="B39" s="17" t="n">
+      <c r="A39" s="19" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B39" s="20" t="n">
         <v>34</v>
       </c>
-      <c r="C39" s="17" t="inlineStr">
+      <c r="C39" s="20" t="inlineStr">
         <is>
           <t>Are there visual styles/trends/design approaches that would NOT work well?</t>
         </is>
       </c>
-      <c r="D39" s="17" t="inlineStr">
+      <c r="D39" s="20" t="inlineStr">
         <is>
           <t>Not directly addressed.</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="16" t="inlineStr">
-        <is>
-          <t>Additional (Extra Time)</t>
-        </is>
-      </c>
-      <c r="B40" s="17" t="n">
+      <c r="A40" s="19" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B40" s="20" t="n">
         <v>35</v>
       </c>
-      <c r="C40" s="17" t="inlineStr">
+      <c r="C40" s="20" t="inlineStr">
         <is>
           <t>What short videos would be helpful to supplement your teaching?</t>
         </is>
       </c>
-      <c r="D40" s="17" t="inlineStr">
+      <c r="D40" s="20" t="inlineStr">
         <is>
           <t>Media kept to 3-7 min; strong interest in content built on the 'argument from beauty'/aesthetics.</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="16" t="inlineStr">
-        <is>
-          <t>Additional (Extra Time)</t>
-        </is>
-      </c>
-      <c r="B41" s="17" t="n">
+      <c r="A41" s="19" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B41" s="20" t="n">
         <v>36</v>
       </c>
-      <c r="C41" s="17" t="inlineStr">
+      <c r="C41" s="20" t="inlineStr">
         <is>
           <t>On a scale of 1-10, how would you rate role-play activities for engagement?</t>
         </is>
       </c>
-      <c r="D41" s="17" t="inlineStr">
+      <c r="D41" s="20" t="inlineStr">
         <is>
           <t>Not directly addressed.</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="16" t="inlineStr">
-        <is>
-          <t>Additional (Extra Time)</t>
-        </is>
-      </c>
-      <c r="B42" s="17" t="n">
+      <c r="A42" s="19" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B42" s="20" t="n">
         <v>37</v>
       </c>
-      <c r="C42" s="17" t="inlineStr">
+      <c r="C42" s="20" t="inlineStr">
         <is>
           <t>What elements of a Bible curriculum do you NOT prefer?</t>
         </is>
       </c>
-      <c r="D42" s="17" t="inlineStr">
+      <c r="D42" s="20" t="inlineStr">
         <is>
           <t>A content-regurgitation-only model (wants soul-level reflection, not facts-for-a-grade); excessive student screen time.</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="16" t="inlineStr">
-        <is>
-          <t>Additional (Extra Time)</t>
-        </is>
-      </c>
-      <c r="B43" s="17" t="n">
+      <c r="A43" s="19" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B43" s="20" t="n">
         <v>38</v>
       </c>
-      <c r="C43" s="17" t="inlineStr">
+      <c r="C43" s="20" t="inlineStr">
         <is>
           <t>What gets and holds your students' attention in Bible class?</t>
         </is>
       </c>
-      <c r="D43" s="17" t="inlineStr">
+      <c r="D43" s="20" t="inlineStr">
         <is>
           <t>Harkness discussion, student ownership/inquiry, short direct-instruction bursts, and countering short-form-media habits (the gap between how long students CAN vs. WILL attend).</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="16" t="inlineStr">
-        <is>
-          <t>Additional (Extra Time)</t>
-        </is>
-      </c>
-      <c r="B44" s="17" t="n">
+      <c r="A44" s="19" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B44" s="20" t="n">
         <v>39</v>
       </c>
-      <c r="C44" s="17" t="inlineStr">
+      <c r="C44" s="20" t="inlineStr">
         <is>
           <t>What would a middle school Bible curriculum look like that is easy to teach and impactful?</t>
         </is>
       </c>
-      <c r="D44" s="17" t="inlineStr">
+      <c r="D44" s="20" t="inlineStr">
         <is>
           <t>Discussion/inquiry-driven with clear division targets (6th OT survey, 7th NT survey, 8th worldview/apologetics/ethics), the Casket-Empty meta-narrative, an integrated logic track, common assessments enabling reteach/extension, minimal student screens, aiming at 'resilient disciples.'</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="27" t="inlineStr">
+      <c r="A46" s="31" t="inlineStr">
         <is>
           <t>DEEPROOTS TEAM TAKEAWAYS — Will Weaver interview (said or unsaid)</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="24" t="inlineStr">
+      <c r="A47" s="28" t="inlineStr">
         <is>
           <t>Team member (attendee)</t>
         </is>
       </c>
-      <c r="B47" s="24" t="inlineStr"/>
-      <c r="C47" s="24" t="inlineStr"/>
-      <c r="D47" s="24" t="inlineStr">
+      <c r="B47" s="28" t="inlineStr"/>
+      <c r="C47" s="28" t="inlineStr"/>
+      <c r="D47" s="28" t="inlineStr">
         <is>
           <t>Takeaways / observations</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="25" t="inlineStr">
+      <c r="A48" s="29" t="inlineStr">
         <is>
           <t>Troy Winkler</t>
         </is>
       </c>
-      <c r="B48" s="25" t="inlineStr"/>
-      <c r="C48" s="25" t="inlineStr"/>
-      <c r="D48" s="25" t="inlineStr"/>
+      <c r="B48" s="29" t="inlineStr"/>
+      <c r="C48" s="29" t="inlineStr"/>
+      <c r="D48" s="29" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" s="25" t="inlineStr">
+      <c r="A49" s="29" t="inlineStr">
         <is>
           <t>Pat Williamson</t>
         </is>
       </c>
-      <c r="B49" s="25" t="inlineStr"/>
-      <c r="C49" s="25" t="inlineStr"/>
-      <c r="D49" s="25" t="inlineStr"/>
+      <c r="B49" s="29" t="inlineStr"/>
+      <c r="C49" s="29" t="inlineStr"/>
+      <c r="D49" s="29" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" s="25" t="inlineStr">
+      <c r="A50" s="29" t="inlineStr">
         <is>
           <t>Tammy Plett</t>
         </is>
       </c>
-      <c r="B50" s="25" t="inlineStr"/>
-      <c r="C50" s="25" t="inlineStr"/>
-      <c r="D50" s="25" t="inlineStr"/>
+      <c r="B50" s="29" t="inlineStr"/>
+      <c r="C50" s="29" t="inlineStr"/>
+      <c r="D50" s="29" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" s="25" t="inlineStr">
+      <c r="A51" s="29" t="inlineStr">
         <is>
           <t>Lisa Van Vlear</t>
         </is>
       </c>
-      <c r="B51" s="25" t="inlineStr"/>
-      <c r="C51" s="25" t="inlineStr"/>
-      <c r="D51" s="25" t="inlineStr"/>
+      <c r="B51" s="29" t="inlineStr"/>
+      <c r="C51" s="29" t="inlineStr"/>
+      <c r="D51" s="29" t="inlineStr"/>
     </row>
     <row r="52">
-      <c r="A52" s="25" t="inlineStr">
+      <c r="A52" s="29" t="inlineStr">
         <is>
           <t>Jacob Waller</t>
         </is>
       </c>
-      <c r="B52" s="25" t="inlineStr"/>
-      <c r="C52" s="25" t="inlineStr"/>
-      <c r="D52" s="25" t="inlineStr"/>
+      <c r="B52" s="29" t="inlineStr"/>
+      <c r="C52" s="29" t="inlineStr"/>
+      <c r="D52" s="29" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -3725,21 +3858,21 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="28" t="inlineStr">
+      <c r="A1" s="32" t="inlineStr">
         <is>
           <t>Atlantic Shores Christian School — Virginia</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="22" t="inlineStr">
+      <c r="A2" s="26" t="inlineStr">
         <is>
           <t>Follow-up meeting 9/29/26  |  ~$11,000 account  |  current DeepRoots K-5 customer</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="22" t="inlineStr">
+      <c r="A3" s="26" t="inlineStr">
         <is>
           <t>Attendees: Admin Melissa Wetzel + grade-level Mentor teachers (K-5).</t>
         </is>
@@ -3763,126 +3896,126 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="17" t="inlineStr">
+      <c r="A6" s="20" t="inlineStr">
         <is>
           <t>K</t>
         </is>
       </c>
-      <c r="B6" s="17" t="inlineStr">
+      <c r="B6" s="20" t="inlineStr">
         <is>
           <t>Rebecca</t>
         </is>
       </c>
-      <c r="C6" s="17" t="inlineStr">
+      <c r="C6" s="20" t="inlineStr">
         <is>
           <t>All going pretty good; some early tech issues that seem worked through (maybe on their end). All K teachers project/teach from the Teacher site; rooms don't have 2 devices, so one-device teaching. Going OK this way.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="17" t="inlineStr">
+      <c r="A7" s="20" t="inlineStr">
         <is>
           <t>1st</t>
         </is>
       </c>
-      <c r="B7" s="17" t="inlineStr">
+      <c r="B7" s="20" t="inlineStr">
         <is>
           <t>Kristal</t>
         </is>
       </c>
-      <c r="C7" s="17" t="inlineStr">
+      <c r="C7" s="20" t="inlineStr">
         <is>
           <t>Going well. Printed the TNs for all 1st teachers and using them. Kids too young to memorize two verses, so they use only one. Too much content for this age, but the TEs are very helpful.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="17" t="inlineStr">
+      <c r="A8" s="20" t="inlineStr">
         <is>
           <t>2nd</t>
         </is>
       </c>
-      <c r="B8" s="17" t="inlineStr">
+      <c r="B8" s="20" t="inlineStr">
         <is>
           <t>Jessica</t>
         </is>
       </c>
-      <c r="C8" s="17" t="inlineStr">
+      <c r="C8" s="20" t="inlineStr">
         <is>
           <t>Going good; parents also like the curriculum (unsure how many use the PEP). 'Intro to Jesus' unit too high-level (lower grades agreed); kids didn't like/understand the classical art; too much time explaining things like Jesus called a 'lunatic'. Likes that students use their Bibles much more now.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="17" t="inlineStr">
+      <c r="A9" s="20" t="inlineStr">
         <is>
           <t>3rd</t>
         </is>
       </c>
-      <c r="B9" s="17" t="inlineStr">
+      <c r="B9" s="20" t="inlineStr">
         <is>
           <t>Natalie</t>
         </is>
       </c>
-      <c r="C9" s="17" t="inlineStr">
+      <c r="C9" s="20" t="inlineStr">
         <is>
           <t>Going well. Toggling between Student World (SW) and Teacher World (TW) is sometimes too much/confusing. Loves the content; kids love Role Play (esp. Good Samaritan). TE super helpful; loves 10 days of content to choose from and time to dive deep. Wishes for Bible-verse songs with hand motions. Tried online tests, but dislikes marking off for spelling.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="17" t="inlineStr">
+      <c r="A10" s="20" t="inlineStr">
         <is>
           <t>4th</t>
         </is>
       </c>
-      <c r="B10" s="17" t="inlineStr">
+      <c r="B10" s="20" t="inlineStr">
         <is>
           <t>Robin</t>
         </is>
       </c>
-      <c r="C10" s="17" t="inlineStr">
+      <c r="C10" s="20" t="inlineStr">
         <is>
           <t>Enjoying it; uses the TNs when teaching. Really wants hand motions for the memory verses; they help upper grades learn verses. (Melissa: MS/HS use hand motions for retention too, without a song.)</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="17" t="inlineStr">
+      <c r="A11" s="20" t="inlineStr">
         <is>
           <t>5th</t>
         </is>
       </c>
-      <c r="B11" s="17" t="inlineStr">
+      <c r="B11" s="20" t="inlineStr">
         <is>
           <t>Miriam</t>
         </is>
       </c>
-      <c r="C11" s="17" t="inlineStr">
+      <c r="C11" s="20" t="inlineStr">
         <is>
           <t>OK, but dislikes the scrolling format. Dislikes online assessments marking off for spelling (defeats the auto-grade time savings). Content over their heads; many unchurched students make it hard. Songs too juvenile; prefers known 'brand name' songs (e.g., Forrest Frank).</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="17" t="inlineStr">
+      <c r="A12" s="20" t="inlineStr">
         <is>
           <t>Admin</t>
         </is>
       </c>
-      <c r="B12" s="17" t="inlineStr">
+      <c r="B12" s="20" t="inlineStr">
         <is>
           <t>Melissa Wetzel</t>
         </is>
       </c>
-      <c r="C12" s="17" t="inlineStr">
+      <c r="C12" s="20" t="inlineStr">
         <is>
           <t>Thought things were going well; hadn't heard negative feedback beforehand; wanted to hear from the mentors. Confirmed MS/HS use hand motions for verse retention.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="29" t="inlineStr">
+      <c r="A14" s="33" t="inlineStr">
         <is>
           <t>OBSERVED THEMES (from the notes)</t>
         </is>
@@ -3891,7 +4024,7 @@
     <row r="15">
       <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr"/>
-      <c r="C15" s="25" t="inlineStr">
+      <c r="C15" s="29" t="inlineStr">
         <is>
           <t>Strong, repeated demand for memory-verse SONGS with HAND MOTIONS (3rd, 4th; admin confirms value through HS).</t>
         </is>
@@ -3900,7 +4033,7 @@
     <row r="16">
       <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr"/>
-      <c r="C16" s="25" t="inlineStr">
+      <c r="C16" s="29" t="inlineStr">
         <is>
           <t>Online auto-grading is wanted, but marking off for spelling is a dealbreaker — make spelling leniency configurable.</t>
         </is>
@@ -3909,7 +4042,7 @@
     <row r="17">
       <c r="A17" t="inlineStr"/>
       <c r="B17" t="inlineStr"/>
-      <c r="C17" s="25" t="inlineStr">
+      <c r="C17" s="29" t="inlineStr">
         <is>
           <t>Content level/pacing runs high for younger grades ('Intro to Jesus', classical art) — add grade-appropriate scaffolding.</t>
         </is>
@@ -3918,7 +4051,7 @@
     <row r="18">
       <c r="A18" t="inlineStr"/>
       <c r="B18" t="inlineStr"/>
-      <c r="C18" s="25" t="inlineStr">
+      <c r="C18" s="29" t="inlineStr">
         <is>
           <t>Role play is a hit in elementary (Good Samaritan) — opposite of the middle-school signal; keep it age-targeted.</t>
         </is>
@@ -3927,7 +4060,7 @@
     <row r="19">
       <c r="A19" t="inlineStr"/>
       <c r="B19" t="inlineStr"/>
-      <c r="C19" s="25" t="inlineStr">
+      <c r="C19" s="29" t="inlineStr">
         <is>
           <t>Digital UX: reduce scrolling; the SW/TW toggle can confuse teachers.</t>
         </is>
@@ -3936,7 +4069,7 @@
     <row r="20">
       <c r="A20" t="inlineStr"/>
       <c r="B20" t="inlineStr"/>
-      <c r="C20" s="25" t="inlineStr">
+      <c r="C20" s="29" t="inlineStr">
         <is>
           <t>Upper-elementary song style should avoid a juvenile tone; lean on recognizable artists.</t>
         </is>
@@ -3945,9 +4078,205 @@
     <row r="21">
       <c r="A21" t="inlineStr"/>
       <c r="B21" t="inlineStr"/>
-      <c r="C21" s="25" t="inlineStr">
+      <c r="C21" s="29" t="inlineStr">
         <is>
           <t>Many unchurched students: don't assume base Bible knowledge (some don't know who Noah is).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00C55A11"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="95" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="34" t="inlineStr">
+        <is>
+          <t>Horizon Christian Elementary School — Tualatin, OR</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="26" t="inlineStr">
+        <is>
+          <t>Follow-up meeting 9/28/26  |  current DeepRoots K-5 customer  |  Sales ambassador: Tammy Plett (TP)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="26" t="inlineStr">
+        <is>
+          <t>Attendees: K-5 vice principal Chris Cain + teaching staff (K-5, 3 teachers per grade). Notes captured K, G1, G4, G5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Grade</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Teacher / staff</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Feedback</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="20" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="B6" s="20" t="inlineStr">
+        <is>
+          <t>K teachers</t>
+        </is>
+      </c>
+      <c r="C6" s="20" t="inlineStr">
+        <is>
+          <t>Going well; students are enjoying it. Like the layout with a variety of activities to reach different types of learners. 'Variety is key!'</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="20" t="inlineStr">
+        <is>
+          <t>G1</t>
+        </is>
+      </c>
+      <c r="B7" s="20" t="inlineStr">
+        <is>
+          <t>1st-grade teachers</t>
+        </is>
+      </c>
+      <c r="C7" s="20" t="inlineStr">
+        <is>
+          <t>Overall going well. Clunky getting used to at first but improving. Kids love the songs. One teacher is creating her own ASL hand motions for the memory verses to help students remember. Love the discussions. Can't cover all the material in each unit, so would prefer just one memory verse rather than two (suggested using the week-2 tested verse). Projecting the visuals is clunky (echoed by all grades); a slideshow version is in the works.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="20" t="inlineStr">
+        <is>
+          <t>G4</t>
+        </is>
+      </c>
+      <c r="B8" s="20" t="inlineStr">
+        <is>
+          <t>4th-grade teachers</t>
+        </is>
+      </c>
+      <c r="C8" s="20" t="inlineStr">
+        <is>
+          <t>Test questions are too verbose and over some students' heads. Many unchurched students get hung up on unfamiliar words like 'Sanhedrin,' making short-answer hard; matching &amp; fill-in-the-blank are easier. Students use NIV Bibles; using multiple translations for memory verses confuses students (especially the unchurched). Asked for a single translation; told DeepRoots is moving to all ESV.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="20" t="inlineStr">
+        <is>
+          <t>G5</t>
+        </is>
+      </c>
+      <c r="B9" s="20" t="inlineStr">
+        <is>
+          <t>5th-grade teachers</t>
+        </is>
+      </c>
+      <c r="C9" s="20" t="inlineStr">
+        <is>
+          <t>Projecting feels clunky, like reading a script instead of discussing; would rather prep the lesson and then discuss. Hard to navigate projection when not covering all material (slideshow with show/hide slides would help). Uses some of our videos plus her own; wasn't using our visuals thinking them too young (kindergartener photos) — this came from starting with the 'Intro to Jesus' unit; the rest of the G5 visuals are age-appropriate. Wants printable pre/post assessments for all grades (no student devices at school). Wants Teaching Essentials split by unit with elements (Bible reading passage, memory verse) listed inline; printed TNs are too long.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="35" t="inlineStr">
+        <is>
+          <t>OBSERVED THEMES (from the notes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr"/>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" s="29" t="inlineStr">
+        <is>
+          <t>Projecting the visuals is clunky across ALL grades — a slideshow version (let teachers show/hide slides) is the top ask.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr"/>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" s="29" t="inlineStr">
+        <is>
+          <t>Move to a SINGLE Bible translation (switching to all ESV) — multiple translations confuse students, especially the unchurched.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr"/>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" s="29" t="inlineStr">
+        <is>
+          <t>Memory verses: allow ONE per unit for lower grades (not two); ASL/hand motions are valued (a G1 teacher is improvising her own).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr"/>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" s="29" t="inlineStr">
+        <is>
+          <t>Assessments: test wording is too advanced/verbose for younger and unchurched students (prefer matching/fill-in-the-blank); provide PRINTABLE pre- and post-assessments for all grades (no student devices).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr"/>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" s="29" t="inlineStr">
+        <is>
+          <t>Differentiate the 'Intro to Jesus' unit (upper vs lower elementary) — it's the key unit for unchurched kids and shouldn't set the tone for all visuals.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr"/>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" s="29" t="inlineStr">
+        <is>
+          <t>Teaching Essentials: split by unit and surface key elements inline (Bible reading passage, memory verse) so teachers don't juggle multiple docs; printed TNs are too long.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr"/>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" s="29" t="inlineStr">
+        <is>
+          <t>Strengths: variety of activities (K), songs and discussions loved (K/G1); overall going well across grades.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Tradeshow Responses tab to interview Q&A mirror workbook
Mirror the live "Tradeshow Responses" tab: 2 Google Form survey
responses (Carol Ann Cox, Josiah Gosyne) with answers mapped to the
overlapping questions in our 39-question set (Q1, Q2, Q4, Q5/Q39, Q8,
Q11). Styled to match the workbook (grey tab, white header, frozen
header, wrapped cells).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BUC7AKNsC5W1a963Yi5JKY
</commit_message>
<xml_diff>
--- a/outreach/DeepRoots_Interview_QA.xlsx
+++ b/outreach/DeepRoots_Interview_QA.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Interviews" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Meredith Arldt" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Will Weaver" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wendy Wagoner" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ironbridge (Nicole + Crystal)" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dayspring (Donna + Angela)" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atlantic Shores (VA) Feedback" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Horizon Christian (OR) Feedback" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Read Me" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="All Interviews" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Meredith Arldt" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Will Weaver" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Wendy Wagoner" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Ironbridge (Nicole + Crystal)" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Dayspring (Donna + Angela)" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Atlantic Shores (VA) Feedback" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Horizon Christian (OR) Feedback" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Tradeshow Responses" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -25,7 +26,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="16">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -97,8 +98,17 @@
       <color rgb="00C55A11"/>
       <sz val="13"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00757575"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <color rgb="00595959"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="18">
+  <fills count="19">
     <fill>
       <patternFill/>
     </fill>
@@ -185,6 +195,12 @@
         <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00757575"/>
+        <bgColor rgb="00757575"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -212,7 +228,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -323,6 +339,13 @@
     <xf numFmtId="0" fontId="3" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -835,6 +858,261 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00757575"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="46" customWidth="1" min="9" max="9"/>
+    <col width="46" customWidth="1" min="10" max="10"/>
+    <col width="46" customWidth="1" min="11" max="11"/>
+    <col width="46" customWidth="1" min="12" max="12"/>
+    <col width="46" customWidth="1" min="13" max="13"/>
+    <col width="46" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="54" t="inlineStr">
+        <is>
+          <t>Tradeshow Responses — Middle-School Bible Curriculum Input (Google Form)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="55" t="inlineStr">
+        <is>
+          <t>Quick survey responses gathered at the tradeshow. The answer columns map to our 39-question set where they overlap (Q1, Q2, Q4, Q5/Q39, Q8, Q11, Q15). 2 responses so far — this tab grows as more come in. 'Wants a call?' flags who agreed to a follow-up conversation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="56" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B4" s="56" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C4" s="56" t="inlineStr">
+        <is>
+          <t>School</t>
+        </is>
+      </c>
+      <c r="D4" s="56" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="E4" s="56" t="inlineStr">
+        <is>
+          <t>City</t>
+        </is>
+      </c>
+      <c r="F4" s="56" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="G4" s="56" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="H4" s="56" t="inlineStr">
+        <is>
+          <t>Wants a call?</t>
+        </is>
+      </c>
+      <c r="I4" s="56" t="inlineStr">
+        <is>
+          <t>Q1 · MS categorization</t>
+        </is>
+      </c>
+      <c r="J4" s="56" t="inlineStr">
+        <is>
+          <t>Q2 · 6th/7th/8th differences</t>
+        </is>
+      </c>
+      <c r="K4" s="56" t="inlineStr">
+        <is>
+          <t>Q4 · Like/dislike current curriculum</t>
+        </is>
+      </c>
+      <c r="L4" s="56" t="inlineStr">
+        <is>
+          <t>Q5/Q39 · Essential to include (build-your-own)</t>
+        </is>
+      </c>
+      <c r="M4" s="56" t="inlineStr">
+        <is>
+          <t>Q8 · Attention span (lecture)</t>
+        </is>
+      </c>
+      <c r="N4" s="56" t="inlineStr">
+        <is>
+          <t>Q11 · Student struggles by grade</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="41" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B5" s="41" t="inlineStr">
+        <is>
+          <t>Carol Ann Cox</t>
+        </is>
+      </c>
+      <c r="C5" s="41" t="inlineStr">
+        <is>
+          <t>Faith Christian School</t>
+        </is>
+      </c>
+      <c r="D5" s="41" t="inlineStr">
+        <is>
+          <t>Middle School Supervisor</t>
+        </is>
+      </c>
+      <c r="E5" s="41" t="inlineStr"/>
+      <c r="F5" s="41" t="inlineStr"/>
+      <c r="G5" s="41" t="inlineStr">
+        <is>
+          <t>carolc@faithramseur.org</t>
+        </is>
+      </c>
+      <c r="H5" s="41" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I5" s="41" t="inlineStr">
+        <is>
+          <t>6th–8th</t>
+        </is>
+      </c>
+      <c r="J5" s="41" t="inlineStr">
+        <is>
+          <t>6th grade- beginning to learn independence and responsibility; some drama among the girls- hurtful comments, friendship challenges; boys have sexual interests and sometimes don’t care about how crude or bold they are.</t>
+        </is>
+      </c>
+      <c r="K5" s="41" t="inlineStr">
+        <is>
+          <t>6th grade lever seems a bit too juvenile. Bible verses are passages that are sometimes difficult to understand and apply to life as a preteen/teenager</t>
+        </is>
+      </c>
+      <c r="L5" s="41" t="inlineStr">
+        <is>
+          <t>How to truly live as a Christian day-by-day, putting God first without being g “holier than thou”</t>
+        </is>
+      </c>
+      <c r="M5" s="41" t="inlineStr">
+        <is>
+          <t>Average- 15 min</t>
+        </is>
+      </c>
+      <c r="N5" s="41" t="inlineStr">
+        <is>
+          <t>6th- mom &amp; dad not in church, not living godly lives, yet students are hearing about godly lives at school. How do you balance that?
+7th- parents enabling “lazy” school work; lack of desire to do their best 
+8th- uncertainty of how Christians stand strong against ungodly pressures</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="41" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B6" s="41" t="inlineStr">
+        <is>
+          <t>Josiah Gosyne</t>
+        </is>
+      </c>
+      <c r="C6" s="41" t="inlineStr">
+        <is>
+          <t>Pinewood Christian Academy</t>
+        </is>
+      </c>
+      <c r="D6" s="41" t="inlineStr">
+        <is>
+          <t>Bible Teacher</t>
+        </is>
+      </c>
+      <c r="E6" s="41" t="inlineStr">
+        <is>
+          <t>Middleburg</t>
+        </is>
+      </c>
+      <c r="F6" s="41" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="G6" s="41" t="inlineStr">
+        <is>
+          <t>josiah.gosyne@pcaknights.org</t>
+        </is>
+      </c>
+      <c r="H6" s="41" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I6" s="41" t="inlineStr">
+        <is>
+          <t>6th–8th</t>
+        </is>
+      </c>
+      <c r="J6" s="41" t="inlineStr">
+        <is>
+          <t>I think that the difference separate grades are sixth grade definitely still feels like young students. Seven and eighth grade you can tell that there has been a jump in emotional complexity, even though that might yet display itself in maturity and eighth grade is pretty much the same way there’s been a jump and emotional complexity, they are experiencing a lot of different new things and emotions, and with that comes extra intelligence and extra thinking, which is a really welcome site. Sixth grade definitely still demonstrates to me that they are like little children, even though they are not beginning to respond to higher intellectual ideas.</t>
+        </is>
+      </c>
+      <c r="K6" s="41" t="inlineStr">
+        <is>
+          <t>Very monotonous but thorough, lots of notes but not a lot of fun engaging things</t>
+        </is>
+      </c>
+      <c r="L6" s="41" t="inlineStr">
+        <is>
+          <t>Funny that you see this because I am currently building my own curriculum. Sixth grade we’re focusing on the core attributes of God. Seventh grade is Old Testament whereas eighth grade is New Testament survey. Currently there is a lot of theological discussion among seventh and eighth grade, even though that theological discussion is often impaired with just theory of what actually happened which seems to work well although more fun and engaging things need to be factored into this so that the kids don’t feel like they’re in one long monotonous loop. Sixth grade is a lot trickier because they are still little children and they still need some very kid like encouragement and kid like help that to balance out their learning so that one is tougher and I personally I’m still working through it however they have demonstrated the abilities to understand difficult concepts, even if they have to be broken down more than usual</t>
+        </is>
+      </c>
+      <c r="M6" s="41" t="inlineStr">
+        <is>
+          <t>30-35</t>
+        </is>
+      </c>
+      <c r="N6" s="41" t="inlineStr">
+        <is>
+          <t>For sixth grade, they are beginning to ask big questions about creation whereas seventh and eighth grade are definitely concerned with more societal problems like homosexuality, relationships, dating, and how they perceived the world around them based on what the media is telling them</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -3631,9 +3909,6 @@
           <t>Overall / key takeaways</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr"/>
-      <c r="C53" t="inlineStr"/>
-      <c r="D53" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4556,9 +4831,6 @@
           <t>Overall / key takeaways</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr"/>
-      <c r="C53" t="inlineStr"/>
-      <c r="D53" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5481,9 +5753,6 @@
           <t>Overall / key takeaways</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr"/>
-      <c r="C53" t="inlineStr"/>
-      <c r="D53" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6406,9 +6675,6 @@
           <t>Overall / key takeaways</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr"/>
-      <c r="C53" t="inlineStr"/>
-      <c r="D53" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7311,9 +7577,6 @@
           <t>Overall / key takeaways</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr"/>
-      <c r="C51" t="inlineStr"/>
-      <c r="D51" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7500,8 +7763,6 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr"/>
-      <c r="B15" t="inlineStr"/>
       <c r="C15" s="41" t="inlineStr">
         <is>
           <t>Strong, repeated demand for memory-verse SONGS with HAND MOTIONS (3rd, 4th; admin confirms value through HS).</t>
@@ -7509,8 +7770,6 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr"/>
-      <c r="B16" t="inlineStr"/>
       <c r="C16" s="41" t="inlineStr">
         <is>
           <t>Online auto-grading is wanted, but marking off for spelling is a dealbreaker — make spelling leniency configurable.</t>
@@ -7518,8 +7777,6 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr"/>
-      <c r="B17" t="inlineStr"/>
       <c r="C17" s="41" t="inlineStr">
         <is>
           <t>Content level/pacing runs high for younger grades ('Intro to Jesus', classical art) — add grade-appropriate scaffolding.</t>
@@ -7527,8 +7784,6 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr"/>
-      <c r="B18" t="inlineStr"/>
       <c r="C18" s="41" t="inlineStr">
         <is>
           <t>Role play is a hit in elementary (Good Samaritan) — opposite of the middle-school signal; keep it age-targeted.</t>
@@ -7536,8 +7791,6 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr"/>
-      <c r="B19" t="inlineStr"/>
       <c r="C19" s="41" t="inlineStr">
         <is>
           <t>Digital UX: reduce scrolling; the SW/TW toggle can confuse teachers.</t>
@@ -7545,8 +7798,6 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr"/>
-      <c r="B20" t="inlineStr"/>
       <c r="C20" s="41" t="inlineStr">
         <is>
           <t>Upper-elementary song style should avoid a juvenile tone; lean on recognizable artists.</t>
@@ -7554,8 +7805,6 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr"/>
-      <c r="B21" t="inlineStr"/>
       <c r="C21" s="41" t="inlineStr">
         <is>
           <t>Many unchurched students: don't assume base Bible knowledge (some don't know who Noah is).</t>
@@ -7696,8 +7945,6 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr"/>
-      <c r="B12" t="inlineStr"/>
       <c r="C12" s="41" t="inlineStr">
         <is>
           <t>Projecting the visuals is clunky across ALL grades — a slideshow version (let teachers show/hide slides) is the top ask.</t>
@@ -7705,8 +7952,6 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr"/>
-      <c r="B13" t="inlineStr"/>
       <c r="C13" s="41" t="inlineStr">
         <is>
           <t>Move to a SINGLE Bible translation (switching to all ESV) — multiple translations confuse students, especially the unchurched.</t>
@@ -7714,8 +7959,6 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr"/>
-      <c r="B14" t="inlineStr"/>
       <c r="C14" s="41" t="inlineStr">
         <is>
           <t>Memory verses: allow ONE per unit for lower grades (not two); ASL/hand motions are valued (a G1 teacher is improvising her own).</t>
@@ -7723,8 +7966,6 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr"/>
-      <c r="B15" t="inlineStr"/>
       <c r="C15" s="41" t="inlineStr">
         <is>
           <t>Assessments: test wording is too advanced/verbose for younger and unchurched students (prefer matching/fill-in-the-blank); provide PRINTABLE pre- and post-assessments for all grades (no student devices).</t>
@@ -7732,8 +7973,6 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr"/>
-      <c r="B16" t="inlineStr"/>
       <c r="C16" s="41" t="inlineStr">
         <is>
           <t>Differentiate the 'Intro to Jesus' unit (upper vs lower elementary) — it's the key unit for unchurched kids and shouldn't set the tone for all visuals.</t>
@@ -7741,8 +7980,6 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr"/>
-      <c r="B17" t="inlineStr"/>
       <c r="C17" s="41" t="inlineStr">
         <is>
           <t>Teaching Essentials: split by unit and surface key elements inline (Bible reading passage, memory verse) so teachers don't juggle multiple docs; printed TNs are too long.</t>
@@ -7750,8 +7987,6 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr"/>
-      <c r="B18" t="inlineStr"/>
       <c r="C18" s="41" t="inlineStr">
         <is>
           <t>Strengths: variety of activities (K), songs and discussions loved (K/G1); overall going well across grades.</t>

</xml_diff>

<commit_message>
Add Capistrano Valley (CA) feedback tab to interview Q&A mirror
Capture email feedback from Capistrano Valley Christian Schools (current
middle-school DeepRoots customer): Rosemarie Guzman (7th-grade Bible
teacher) on low curriculum usage, rigid/fast structure, and website
navigation (wants a physical book); and Marcus Choi (Head of School/CEO)
on how admins evaluate Bible curricula. Styled to match the Atlantic
Shores and Horizon feedback tabs, with an Observed Themes summary.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BUC7AKNsC5W1a963Yi5JKY
</commit_message>
<xml_diff>
--- a/outreach/DeepRoots_Interview_QA.xlsx
+++ b/outreach/DeepRoots_Interview_QA.xlsx
@@ -16,7 +16,8 @@
     <sheet name="Dayspring (Donna + Angela)" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Atlantic Shores (VA) Feedback" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="Horizon Christian (OR) Feedback" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Tradeshow Responses" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Capistrano Valley (CA) Feedback" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Tradeshow Responses" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -26,7 +27,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="18">
+  <fonts count="19">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -107,8 +108,13 @@
       <color rgb="00595959"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00C0392B"/>
+      <sz val="13"/>
+    </font>
   </fonts>
-  <fills count="19">
+  <fills count="20">
     <fill>
       <patternFill/>
     </fill>
@@ -201,6 +207,12 @@
         <bgColor rgb="00757575"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C0392B"/>
+        <bgColor rgb="00C0392B"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -228,7 +240,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -346,6 +358,11 @@
     <xf numFmtId="0" fontId="4" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -861,6 +878,126 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00C0392B"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="95" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="57" t="inlineStr">
+        <is>
+          <t>Capistrano Valley Christian Schools — California</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="55" t="inlineStr">
+        <is>
+          <t>Email feedback, Oct 2026  |  current DeepRoots customer (middle school)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="55" t="inlineStr">
+        <is>
+          <t>Contacts: Rosemarie Guzman — 7th Grade Bible Teacher (rguzman@cvcs.org)  |  Marcus Choi — Head of School / CEO (mchoi@cvcs.org)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="58" t="inlineStr">
+        <is>
+          <t>Grade / Role</t>
+        </is>
+      </c>
+      <c r="B5" s="58" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C5" s="58" t="inlineStr">
+        <is>
+          <t>Feedback</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="41" t="inlineStr">
+        <is>
+          <t>7th (Bible)</t>
+        </is>
+      </c>
+      <c r="B6" s="41" t="inlineStr">
+        <is>
+          <t>Rosemarie Guzman</t>
+        </is>
+      </c>
+      <c r="C6" s="41" t="inlineStr">
+        <is>
+          <t>Uses only about 15-20% of the curriculum. Feels it is a bit too structured and moves at a fast pace. Finds the lesson-plan layout rigid, though she appreciates the intent behind each lesson. Finds the website hard to navigate logistically (clicking back and forth) and said it would be easier as a physical book.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="41" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="B7" s="41" t="inlineStr">
+        <is>
+          <t>Marcus Choi (Head of School / CEO)</t>
+        </is>
+      </c>
+      <c r="C7" s="41" t="inlineStr">
+        <is>
+          <t>Shared detailed feedback on how administrators evaluate Bible curricula, suggesting we add information around: theological alignment, teacher readiness / prep time, online training videos, grade-level progression, evidence of student learning, and total cost.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="59" t="inlineStr">
+        <is>
+          <t>OBSERVED THEMES (from the notes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="C10" s="41" t="inlineStr">
+        <is>
+          <t>Low adoption: the 7th-grade teacher uses only 15-20% of the curriculum; structure and pace feel too rigid and fast, and the lesson-plan layout feels constraining despite good intent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="C11" s="41" t="inlineStr">
+        <is>
+          <t>Format / UX: the website is hard to navigate (clicking back and forth); a printed / physical book version is requested.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="C12" s="41" t="inlineStr">
+        <is>
+          <t>Admin buying criteria (Marcus Choi): theological alignment, teacher readiness and prep time, online training videos, clear grade-level progression, evidence of student learning, and total cost — a useful checklist for positioning and sales collateral.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="00757575"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>

</xml_diff>

<commit_message>
Add Josiah Gosyne (FL) call-notes tab to interview Q&A mirror
Capture the 10/22/2026 interview call with Josiah Gosyne (Pinewood
Christian Academy), who is building his own middle-school Bible
curriculum: 6th-grade adapted Sunday-school/systematic theology, 7th/8th
OT and NT surveys with Cornell notes and exegetical papers, strong
student engagement with advanced concepts, and next steps (sample lesson
+ follow-up). Indigo tab, grouped with the other research captures.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BUC7AKNsC5W1a963Yi5JKY
</commit_message>
<xml_diff>
--- a/outreach/DeepRoots_Interview_QA.xlsx
+++ b/outreach/DeepRoots_Interview_QA.xlsx
@@ -17,7 +17,8 @@
     <sheet name="Atlantic Shores (VA) Feedback" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="Horizon Christian (OR) Feedback" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="Capistrano Valley (CA) Feedback" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Tradeshow Responses" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Josiah Gosyne (FL) - Call Notes" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Tradeshow Responses" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -27,7 +28,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="19">
+  <fonts count="20">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -113,8 +114,13 @@
       <color rgb="00C0392B"/>
       <sz val="13"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="003B3B98"/>
+      <sz val="13"/>
+    </font>
   </fonts>
-  <fills count="20">
+  <fills count="21">
     <fill>
       <patternFill/>
     </fill>
@@ -213,6 +219,12 @@
         <bgColor rgb="00C0392B"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="003B3B98"/>
+        <bgColor rgb="003B3B98"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -240,7 +252,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -363,6 +375,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -998,6 +1016,193 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="003B3B98"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="115" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="60" t="inlineStr">
+        <is>
+          <t>Josiah Gosyne — Pinewood Christian Academy (Middleburg, FL)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="55" t="inlineStr">
+        <is>
+          <t>Interview call · 10/22/2026 · ~30 min · building his own middle-school Bible curriculum (market research)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="55" t="inlineStr">
+        <is>
+          <t>DeepRoots attendees: Troy Winkler, Lisa Van Vlear, Nancy Wood, Pat Williamson, Jacob Waller. (Josiah also completed our tradeshow survey — see Tradeshow Responses tab.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="41" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="61" t="inlineStr">
+        <is>
+          <t>6th grade curriculum structure</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="41" t="inlineStr">
+        <is>
+          <t>•  Adapted a Sunday-school program to fit a confessionally reformed covenant school.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="41" t="inlineStr">
+        <is>
+          <t>•  Blends systematic theology, exegetical Bible papers, and practical theology taught through stories.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="41" t="inlineStr">
+        <is>
+          <t>•  45-minute structured discussions with guided questions; deliberately low reliance on multimedia stimulation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="41" t="inlineStr">
+        <is>
+          <t>•  Class size: 16 students.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="41" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="61" t="inlineStr">
+        <is>
+          <t>7th &amp; 8th grade curriculum structure</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="41" t="inlineStr">
+        <is>
+          <t>•  7th grade is an Old Testament survey; 8th grade is a New Testament survey.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="41" t="inlineStr">
+        <is>
+          <t>•  Uses Cornell notes and student reference documents to reinforce processing during lectures.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="41" t="inlineStr">
+        <is>
+          <t>•  Exegetical Bible papers: students dissect scripture passages and write their own reflections.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="41" t="inlineStr">
+        <is>
+          <t>•  Class sizes: 26 in 7th grade (two sections) and 15 in 8th grade.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="41" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="61" t="inlineStr">
+        <is>
+          <t>Student engagement &amp; theological complexity</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="41" t="inlineStr">
+        <is>
+          <t>•  Students successfully work through advanced concepts such as the proto-gospel and the hypostatic union.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="41" t="inlineStr">
+        <is>
+          <t>•  Josiah and the head of school host open Q&amp;A sessions to address deep spiritual questions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="41" t="inlineStr">
+        <is>
+          <t>•  Student questions progress from creation (6th grade) to identity and ethics (7th-8th).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="41" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="61" t="inlineStr">
+        <is>
+          <t>Next steps</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="41" t="inlineStr">
+        <is>
+          <t>•  Josiah will send one sample lesson as an example of his current curriculum structure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="41" t="inlineStr">
+        <is>
+          <t>•  Troy to follow up with Josiah by email within the next couple of days (follow-up drafted).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="41" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="61" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="41" t="inlineStr">
+        <is>
+          <t>•  Gemini call notes — DeepRoots call, 10/22/2026 3:09 PM EDT.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="00757575"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>

</xml_diff>

<commit_message>
Add Oaks Christian (CA) feedback tab to interview Q&A mirror
First-quarter follow-up from Stephanie Niednagel (Director of Curriculum):
K-4 implementation going smoothly with a hired Bible Specialist; 4th grade
finds DR a lot of material for their schedule; reframing lessons as
instruction vs. devotion; eager for the TK program.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BUC7AKNsC5W1a963Yi5JKY
</commit_message>
<xml_diff>
--- a/outreach/DeepRoots_Interview_QA.xlsx
+++ b/outreach/DeepRoots_Interview_QA.xlsx
@@ -17,8 +17,9 @@
     <sheet name="Atlantic Shores (VA) Feedback" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="Horizon Christian (OR) Feedback" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="Capistrano Valley (CA) Feedback" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Josiah Gosyne (FL) - Call Notes" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Tradeshow Responses" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Oaks Christian (CA) Feedback" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Josiah Gosyne (FL) - Call Notes" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Tradeshow Responses" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -28,7 +29,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="20">
+  <fonts count="21">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -119,8 +120,13 @@
       <color rgb="003B3B98"/>
       <sz val="13"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00138D75"/>
+      <sz val="13"/>
+    </font>
   </fonts>
-  <fills count="21">
+  <fills count="22">
     <fill>
       <patternFill/>
     </fill>
@@ -225,6 +231,12 @@
         <bgColor rgb="003B3B98"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00138D75"/>
+        <bgColor rgb="00138D75"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -252,7 +264,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -379,6 +391,10 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="21" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1016,6 +1032,123 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00138D75"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="95" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="62" t="inlineStr">
+        <is>
+          <t>Oaks Christian School - California</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="55" t="inlineStr">
+        <is>
+          <t>Follow-up email feedback  |  10/23/2026  |  current DeepRoots customer (K-4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="55" t="inlineStr">
+        <is>
+          <t>Contact: Stephanie Niednagel - Director of Curriculum, Teacher Credentialing &amp; Induction Mentor  |  Oaks Christian School, 31749 La Tienda Drive, Westlake Village, CA 91362  |  818-824-9410</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="55" t="inlineStr">
+        <is>
+          <t>Context: Oaks adopted DeepRoots K-4 and hired a Bible Specialist (SarahBeth) who had taught DR at another school and supports the teachers. No teacher meeting was needed; Stephanie sent this on a DeepRoots check-in (from Erin).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="63" t="inlineStr">
+        <is>
+          <t>Grade / Role</t>
+        </is>
+      </c>
+      <c r="B6" s="63" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C6" s="63" t="inlineStr">
+        <is>
+          <t>Feedback</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="41" t="inlineStr">
+        <is>
+          <t>Admin / Curriculum</t>
+        </is>
+      </c>
+      <c r="B7" s="41" t="inlineStr">
+        <is>
+          <t>Stephanie Niednagel (Director of Curriculum)</t>
+        </is>
+      </c>
+      <c r="C7" s="41" t="inlineStr">
+        <is>
+          <t>Says implementation of Deep Roots is going smoothly and teachers feel well supported by the Bible Specialist ("take my silence as a good sign"). The 4th grade team is now rolling with Deep Roots but finds it to be "a lot of material for the time they have in their schedule"; the school is working with teachers on the essentials for each unit. Also guiding teachers toward a change of approach - treating the Bible lesson as actual "instruction" rather than simply devotion / heart-based discussion. Eager to see the forthcoming TK (transitional kindergarten) program. Will remind teachers about the upcoming Thanksgiving resources.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="59" t="inlineStr">
+        <is>
+          <t>OBSERVED THEMES (from the email)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="C10" s="41" t="inlineStr">
+        <is>
+          <t>Pacing / volume: the 4th grade team finds DR "a lot of material for the time they have" - supports a per-unit "essentials" guide or a lighter-time pathway.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="C11" s="41" t="inlineStr">
+        <is>
+          <t>Instructional positioning: the school is reframing DR from devotion / heart-based discussion toward actual instruction - signals demand for clearer instructional structure and learning outcomes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="C12" s="41" t="inlineStr">
+        <is>
+          <t>Support model that works: a dedicated Bible Specialist who already knew DR drove smooth adoption with no teacher meeting needed - a repeatable onboarding pattern.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="C13" s="41" t="inlineStr">
+        <is>
+          <t>Pipeline demand: already on K-4 and eager for the TK program - appetite for expanded grade-level coverage.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="003B3B98"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -1200,7 +1333,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00757575"/>

</xml_diff>

<commit_message>
Add Active Learning Referrals tracker tab to interview Q&A mirror
New tab logging Kim Van Vlear's teacher-scouting ask (standout, creative
Grades 1-8 Active Student Learning teachers for a future paid part-time
role). Pre-loaded with the 9 contacts emailed the follow-up question on
10/27: Jen Studt plus the 8 interviewees to date.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BUC7AKNsC5W1a963Yi5JKY
</commit_message>
<xml_diff>
--- a/outreach/DeepRoots_Interview_QA.xlsx
+++ b/outreach/DeepRoots_Interview_QA.xlsx
@@ -22,6 +22,7 @@
     <sheet name="Tradeshow Responses" sheetId="13" state="visible" r:id="rId13"/>
     <sheet name="Research 23-24 (7th)" sheetId="14" state="visible" r:id="rId14"/>
     <sheet name="Research 23-24 (8th)" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Active Learning Referrals" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -31,7 +32,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="25">
+  <fonts count="26">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -144,8 +145,13 @@
       <b val="1"/>
       <color rgb="00B9770E"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="007D3C98"/>
+      <sz val="13"/>
+    </font>
   </fonts>
-  <fills count="23">
+  <fills count="24">
     <fill>
       <patternFill/>
     </fill>
@@ -262,6 +268,12 @@
         <bgColor rgb="005D6D7E"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="007D3C98"/>
+        <bgColor rgb="007D3C98"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -289,7 +301,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -432,6 +444,10 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -58643,6 +58659,521 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="007D3C98"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="42" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="68" t="inlineStr">
+        <is>
+          <t>Active Learning Referrals - teacher scouting for Kim Van Vlear</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="55" t="inlineStr">
+        <is>
+          <t>Kim is looking for standout, incredibly creative Grades 1-8 teachers in Active Student Learning for a future paid, part-time role (likely under 6 months, a few hours/week) helping create Active Learning Engagements. For each referral, capture the teacher's name, grade, and email, plus the school, city, state, and the referring admin and their position - then send to Kim.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="69" t="inlineStr">
+        <is>
+          <t>Date Asked</t>
+        </is>
+      </c>
+      <c r="B4" s="69" t="inlineStr">
+        <is>
+          <t>Referring Contact (Admin)</t>
+        </is>
+      </c>
+      <c r="C4" s="69" t="inlineStr">
+        <is>
+          <t>Position</t>
+        </is>
+      </c>
+      <c r="D4" s="69" t="inlineStr">
+        <is>
+          <t>School</t>
+        </is>
+      </c>
+      <c r="E4" s="69" t="inlineStr">
+        <is>
+          <t>City</t>
+        </is>
+      </c>
+      <c r="F4" s="69" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="G4" s="69" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="H4" s="69" t="inlineStr">
+        <is>
+          <t>Referred Teacher</t>
+        </is>
+      </c>
+      <c r="I4" s="69" t="inlineStr">
+        <is>
+          <t>Grade</t>
+        </is>
+      </c>
+      <c r="J4" s="69" t="inlineStr">
+        <is>
+          <t>Teacher Email</t>
+        </is>
+      </c>
+      <c r="K4" s="69" t="inlineStr">
+        <is>
+          <t>Sent to Kim</t>
+        </is>
+      </c>
+      <c r="L4" s="69" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="41" t="inlineStr">
+        <is>
+          <t>10/27/2026</t>
+        </is>
+      </c>
+      <c r="B5" s="41" t="inlineStr">
+        <is>
+          <t>Jen Studt</t>
+        </is>
+      </c>
+      <c r="C5" s="41" t="inlineStr">
+        <is>
+          <t>(confirm title)</t>
+        </is>
+      </c>
+      <c r="D5" s="41" t="inlineStr">
+        <is>
+          <t>Concord Christian School</t>
+        </is>
+      </c>
+      <c r="E5" s="41" t="inlineStr"/>
+      <c r="F5" s="41" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="G5" s="41" t="inlineStr">
+        <is>
+          <t>Active Learning ask emailed 10/27</t>
+        </is>
+      </c>
+      <c r="H5" s="41" t="inlineStr"/>
+      <c r="I5" s="41" t="inlineStr"/>
+      <c r="J5" s="41" t="inlineStr"/>
+      <c r="K5" s="41" t="inlineStr"/>
+      <c r="L5" s="41" t="inlineStr">
+        <is>
+          <t>Big DeepRoots fan; earlier referred us to Steven/Danielle for middle school (they declined). Active Learning referral ask emailed 10/27.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="41" t="inlineStr">
+        <is>
+          <t>10/27/2026</t>
+        </is>
+      </c>
+      <c r="B6" s="41" t="inlineStr">
+        <is>
+          <t>Meredith Arldt</t>
+        </is>
+      </c>
+      <c r="C6" s="41" t="inlineStr">
+        <is>
+          <t>Assoc. Head of School</t>
+        </is>
+      </c>
+      <c r="D6" s="41" t="inlineStr">
+        <is>
+          <t>Aliso Viejo Christian School</t>
+        </is>
+      </c>
+      <c r="E6" s="41" t="inlineStr">
+        <is>
+          <t>Aliso Viejo</t>
+        </is>
+      </c>
+      <c r="F6" s="41" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="G6" s="41" t="inlineStr">
+        <is>
+          <t>Active Learning ask emailed 10/27</t>
+        </is>
+      </c>
+      <c r="H6" s="41" t="inlineStr"/>
+      <c r="I6" s="41" t="inlineStr"/>
+      <c r="J6" s="41" t="inlineStr"/>
+      <c r="K6" s="41" t="inlineStr"/>
+      <c r="L6" s="41" t="inlineStr">
+        <is>
+          <t>Interviewed 9/24. Active Learning referral ask emailed 10/27.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="41" t="inlineStr">
+        <is>
+          <t>10/27/2026</t>
+        </is>
+      </c>
+      <c r="B7" s="41" t="inlineStr">
+        <is>
+          <t>Will Weaver</t>
+        </is>
+      </c>
+      <c r="C7" s="41" t="inlineStr">
+        <is>
+          <t>Head of Spiritual Formation</t>
+        </is>
+      </c>
+      <c r="D7" s="41" t="inlineStr">
+        <is>
+          <t>Des Moines Christian School</t>
+        </is>
+      </c>
+      <c r="E7" s="41" t="inlineStr">
+        <is>
+          <t>Urbandale</t>
+        </is>
+      </c>
+      <c r="F7" s="41" t="inlineStr">
+        <is>
+          <t>IA</t>
+        </is>
+      </c>
+      <c r="G7" s="41" t="inlineStr">
+        <is>
+          <t>Active Learning ask emailed 10/27</t>
+        </is>
+      </c>
+      <c r="H7" s="41" t="inlineStr"/>
+      <c r="I7" s="41" t="inlineStr"/>
+      <c r="J7" s="41" t="inlineStr"/>
+      <c r="K7" s="41" t="inlineStr"/>
+      <c r="L7" s="41" t="inlineStr">
+        <is>
+          <t>Interviewed 9/30. Active Learning referral ask emailed 10/27.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="41" t="inlineStr">
+        <is>
+          <t>10/27/2026</t>
+        </is>
+      </c>
+      <c r="B8" s="41" t="inlineStr">
+        <is>
+          <t>Wendy Wagoner</t>
+        </is>
+      </c>
+      <c r="C8" s="41" t="inlineStr">
+        <is>
+          <t>Spiritual Life Coordinator (elementary)</t>
+        </is>
+      </c>
+      <c r="D8" s="41" t="inlineStr">
+        <is>
+          <t>Christian Academy of Indiana</t>
+        </is>
+      </c>
+      <c r="E8" s="41" t="inlineStr">
+        <is>
+          <t>New Albany</t>
+        </is>
+      </c>
+      <c r="F8" s="41" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="G8" s="41" t="inlineStr">
+        <is>
+          <t>Active Learning ask emailed 10/27</t>
+        </is>
+      </c>
+      <c r="H8" s="41" t="inlineStr"/>
+      <c r="I8" s="41" t="inlineStr"/>
+      <c r="J8" s="41" t="inlineStr"/>
+      <c r="K8" s="41" t="inlineStr"/>
+      <c r="L8" s="41" t="inlineStr">
+        <is>
+          <t>Interviewed 10/2. Active Learning referral ask emailed 10/27.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="41" t="inlineStr">
+        <is>
+          <t>10/27/2026</t>
+        </is>
+      </c>
+      <c r="B9" s="41" t="inlineStr">
+        <is>
+          <t>Nicole Burchett</t>
+        </is>
+      </c>
+      <c r="C9" s="41" t="inlineStr">
+        <is>
+          <t>Administrator / Director</t>
+        </is>
+      </c>
+      <c r="D9" s="41" t="inlineStr">
+        <is>
+          <t>Ironbridge Christian Academy</t>
+        </is>
+      </c>
+      <c r="E9" s="41" t="inlineStr">
+        <is>
+          <t>Chester</t>
+        </is>
+      </c>
+      <c r="F9" s="41" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="G9" s="41" t="inlineStr">
+        <is>
+          <t>Active Learning ask emailed 10/27</t>
+        </is>
+      </c>
+      <c r="H9" s="41" t="inlineStr"/>
+      <c r="I9" s="41" t="inlineStr"/>
+      <c r="J9" s="41" t="inlineStr"/>
+      <c r="K9" s="41" t="inlineStr"/>
+      <c r="L9" s="41" t="inlineStr">
+        <is>
+          <t>Interviewed 10/5. Active Learning referral ask emailed 10/27.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="41" t="inlineStr">
+        <is>
+          <t>10/27/2026</t>
+        </is>
+      </c>
+      <c r="B10" s="41" t="inlineStr">
+        <is>
+          <t>Crystal Thompson</t>
+        </is>
+      </c>
+      <c r="C10" s="41" t="inlineStr">
+        <is>
+          <t>5th/6th grade Bible teacher</t>
+        </is>
+      </c>
+      <c r="D10" s="41" t="inlineStr">
+        <is>
+          <t>Ironbridge Christian Academy</t>
+        </is>
+      </c>
+      <c r="E10" s="41" t="inlineStr">
+        <is>
+          <t>Chester</t>
+        </is>
+      </c>
+      <c r="F10" s="41" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="G10" s="41" t="inlineStr">
+        <is>
+          <t>Active Learning ask emailed 10/27</t>
+        </is>
+      </c>
+      <c r="H10" s="41" t="inlineStr"/>
+      <c r="I10" s="41" t="inlineStr"/>
+      <c r="J10" s="41" t="inlineStr"/>
+      <c r="K10" s="41" t="inlineStr"/>
+      <c r="L10" s="41" t="inlineStr">
+        <is>
+          <t>Interviewed 10/5. Active Learning referral ask emailed 10/27.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="41" t="inlineStr">
+        <is>
+          <t>10/27/2026</t>
+        </is>
+      </c>
+      <c r="B11" s="41" t="inlineStr">
+        <is>
+          <t>Donna Hurley</t>
+        </is>
+      </c>
+      <c r="C11" s="41" t="inlineStr">
+        <is>
+          <t>Director of Curriculum &amp; Instruction</t>
+        </is>
+      </c>
+      <c r="D11" s="41" t="inlineStr">
+        <is>
+          <t>Dayspring Christian Academy</t>
+        </is>
+      </c>
+      <c r="E11" s="41" t="inlineStr">
+        <is>
+          <t>Mountville</t>
+        </is>
+      </c>
+      <c r="F11" s="41" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="G11" s="41" t="inlineStr">
+        <is>
+          <t>Active Learning ask emailed 10/27</t>
+        </is>
+      </c>
+      <c r="H11" s="41" t="inlineStr"/>
+      <c r="I11" s="41" t="inlineStr"/>
+      <c r="J11" s="41" t="inlineStr"/>
+      <c r="K11" s="41" t="inlineStr"/>
+      <c r="L11" s="41" t="inlineStr">
+        <is>
+          <t>Interviewed 10/6. Active Learning referral ask emailed 10/27.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="41" t="inlineStr">
+        <is>
+          <t>10/27/2026</t>
+        </is>
+      </c>
+      <c r="B12" s="41" t="inlineStr">
+        <is>
+          <t>Angela Adams</t>
+        </is>
+      </c>
+      <c r="C12" s="41" t="inlineStr">
+        <is>
+          <t>Upper-school Bible department chair</t>
+        </is>
+      </c>
+      <c r="D12" s="41" t="inlineStr">
+        <is>
+          <t>Dayspring Christian Academy</t>
+        </is>
+      </c>
+      <c r="E12" s="41" t="inlineStr">
+        <is>
+          <t>Mountville</t>
+        </is>
+      </c>
+      <c r="F12" s="41" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="G12" s="41" t="inlineStr">
+        <is>
+          <t>Active Learning ask emailed 10/27</t>
+        </is>
+      </c>
+      <c r="H12" s="41" t="inlineStr"/>
+      <c r="I12" s="41" t="inlineStr"/>
+      <c r="J12" s="41" t="inlineStr"/>
+      <c r="K12" s="41" t="inlineStr"/>
+      <c r="L12" s="41" t="inlineStr">
+        <is>
+          <t>Interviewed 10/6. Active Learning referral ask emailed 10/27.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="41" t="inlineStr">
+        <is>
+          <t>10/27/2026</t>
+        </is>
+      </c>
+      <c r="B13" s="41" t="inlineStr">
+        <is>
+          <t>Josiah Gosyne</t>
+        </is>
+      </c>
+      <c r="C13" s="41" t="inlineStr">
+        <is>
+          <t>Middle-school Bible teacher / curriculum developer</t>
+        </is>
+      </c>
+      <c r="D13" s="41" t="inlineStr">
+        <is>
+          <t>Pinewood Christian Academy</t>
+        </is>
+      </c>
+      <c r="E13" s="41" t="inlineStr">
+        <is>
+          <t>Middleburg</t>
+        </is>
+      </c>
+      <c r="F13" s="41" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="G13" s="41" t="inlineStr">
+        <is>
+          <t>Active Learning ask emailed 10/27</t>
+        </is>
+      </c>
+      <c r="H13" s="41" t="inlineStr"/>
+      <c r="I13" s="41" t="inlineStr"/>
+      <c r="J13" s="41" t="inlineStr"/>
+      <c r="K13" s="41" t="inlineStr"/>
+      <c r="L13" s="41" t="inlineStr">
+        <is>
+          <t>Interviewed 10/22. Active Learning referral ask emailed 10/27.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add schedule (block vs. traditional) field to All Interviews tab
New 'Scheduling / S1' row capturing each school's class-schedule type
(block vs. traditional, period length, how often Bible meets), filled from
what interviews surfaced: Des Moines Christian, Ironbridge, and Dayspring
are block; Aliso Viejo and Christian Academy of Indiana appear traditional;
others not captured.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BUC7AKNsC5W1a963Yi5JKY
</commit_message>
<xml_diff>
--- a/outreach/DeepRoots_Interview_QA.xlsx
+++ b/outreach/DeepRoots_Interview_QA.xlsx
@@ -59181,7 +59181,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J43"/>
+  <dimension ref="A1:J44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -61026,6 +61026,58 @@
       <c r="J43" s="36" t="inlineStr">
         <is>
           <t>Something they currently build entirely themselves, made ready-made. Internally they teach New Testament survey (6th, starting with the 400-year intertestamental period), Old Testament survey (7th), and wisdom books (8th), and they want a curriculum that adds apologetics and archaeological evidence, world-history timelines, vocabulary, geography, and strong application and reflection, plus engagement 'learning supports' with student choice, object lessons, and resource pointers. It should suit 80-minute blocks with movement, favor printables with occasional digital, use videos of three-plus minutes, and be enjoyable and engaging rather than dull — and requests must be budgeted early, before December, since the state budget does not cover Christian materials like Bible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>Scheduling</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>Class schedule: block vs. traditional (period length &amp; how often Bible meets)</t>
+        </is>
+      </c>
+      <c r="D44" s="41" t="inlineStr">
+        <is>
+          <t>Appears traditional - team noted ~45-minute class periods (not explicitly asked).</t>
+        </is>
+      </c>
+      <c r="E44" s="41" t="inlineStr">
+        <is>
+          <t>Not captured (K-5 email feedback, not a full MS interview).</t>
+        </is>
+      </c>
+      <c r="F44" s="41" t="inlineStr">
+        <is>
+          <t>Block - 75-minute sessions every other day (~65-70 min effective after a 5-10 min reading period). Moving to a unified 5-8 MS next year.</t>
+        </is>
+      </c>
+      <c r="G44" s="41" t="inlineStr">
+        <is>
+          <t>Not captured (K-5 email feedback, not a full MS interview).</t>
+        </is>
+      </c>
+      <c r="H44" s="41" t="inlineStr">
+        <is>
+          <t>Appears traditional - ~30-40 minute periods (noted that help for schools with longer periods would be useful).</t>
+        </is>
+      </c>
+      <c r="I44" s="41" t="inlineStr">
+        <is>
+          <t>Block - 80-minute periods, every other day (cited as a constraint for getting through all units).</t>
+        </is>
+      </c>
+      <c r="J44" s="41" t="inlineStr">
+        <is>
+          <t>Block - 80-minute block; Bible meets within a 6-day rotation.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Log first Active Learning teacher referrals in tracker
Replies from Meredith Arldt (Mary-Margaret Fincher, 6-8 Science) and Nicole
Burchett (Valarie Walls, 2nd; Crystal Thompson, Bible) logged; Josiah Gosyne
reply received, names pending. Referral summary drafted to Kim.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BUC7AKNsC5W1a963Yi5JKY
</commit_message>
<xml_diff>
--- a/outreach/DeepRoots_Interview_QA.xlsx
+++ b/outreach/DeepRoots_Interview_QA.xlsx
@@ -59105,13 +59105,29 @@
       </c>
       <c r="G7" s="41" t="inlineStr">
         <is>
-          <t>Active Learning ask emailed 10/27</t>
-        </is>
-      </c>
-      <c r="H7" s="41" t="inlineStr"/>
-      <c r="I7" s="41" t="inlineStr"/>
-      <c r="J7" s="41" t="inlineStr"/>
-      <c r="K7" s="41" t="inlineStr"/>
+          <t>Referral received</t>
+        </is>
+      </c>
+      <c r="H7" s="41" t="inlineStr">
+        <is>
+          <t>Mary-Margaret Fincher</t>
+        </is>
+      </c>
+      <c r="I7" s="41" t="inlineStr">
+        <is>
+          <t>6-8 Science</t>
+        </is>
+      </c>
+      <c r="J7" s="41" t="inlineStr">
+        <is>
+          <t>mfincher@avchristianschool.org (cell 949-610-4586)</t>
+        </is>
+      </c>
+      <c r="K7" s="41" t="inlineStr">
+        <is>
+          <t>Drafted to Kim 10/29 (pending send)</t>
+        </is>
+      </c>
       <c r="L7" s="41" t="inlineStr">
         <is>
           <t>Interviewed 9/30. Active Learning referral ask emailed 10/27.</t>
@@ -59197,13 +59213,29 @@
       </c>
       <c r="G9" s="41" t="inlineStr">
         <is>
-          <t>Active Learning ask emailed 10/27</t>
-        </is>
-      </c>
-      <c r="H9" s="41" t="inlineStr"/>
-      <c r="I9" s="41" t="inlineStr"/>
-      <c r="J9" s="41" t="inlineStr"/>
-      <c r="K9" s="41" t="inlineStr"/>
+          <t>Referrals received (2)</t>
+        </is>
+      </c>
+      <c r="H9" s="41" t="inlineStr">
+        <is>
+          <t>Valarie Walls; Crystal Thompson</t>
+        </is>
+      </c>
+      <c r="I9" s="41" t="inlineStr">
+        <is>
+          <t>Valarie: 2nd grade (20 yrs K experience); Crystal: Bible, upper grades</t>
+        </is>
+      </c>
+      <c r="J9" s="41" t="inlineStr">
+        <is>
+          <t>vwalls@ironbridge.academy; cthompson@ironbridge.academy</t>
+        </is>
+      </c>
+      <c r="K9" s="41" t="inlineStr">
+        <is>
+          <t>Drafted to Kim 10/29 (pending send)</t>
+        </is>
+      </c>
       <c r="L9" s="41" t="inlineStr">
         <is>
           <t>Interviewed 10/5. Active Learning referral ask emailed 10/27.</t>
@@ -59381,7 +59413,7 @@
       </c>
       <c r="G13" s="41" t="inlineStr">
         <is>
-          <t>Active Learning ask emailed 10/27</t>
+          <t>Reply received - referral pending (has 1-2 in mind; will send names after asking them)</t>
         </is>
       </c>
       <c r="H13" s="41" t="inlineStr"/>

</xml_diff>

<commit_message>
Active Learning referrals: add Christine Valverde (via Angela Adams); fix Mary-Margaret row
Angela Adams referred Christine Valverde (7th-grade Bible, Dayspring).
First Kim email sent, so Mary-Margaret/Valarie/Crystal marked sent; Christine
is in a new hold-until-evening draft. Also corrected a row mix-up: Mary-Margaret
Fincher's referral was on Will Weaver's row and is now on Meredith Arldt's.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BUC7AKNsC5W1a963Yi5JKY
</commit_message>
<xml_diff>
--- a/outreach/DeepRoots_Interview_QA.xlsx
+++ b/outreach/DeepRoots_Interview_QA.xlsx
@@ -59059,13 +59059,29 @@
       </c>
       <c r="G6" s="41" t="inlineStr">
         <is>
-          <t>Active Learning ask emailed 10/27</t>
-        </is>
-      </c>
-      <c r="H6" s="41" t="inlineStr"/>
-      <c r="I6" s="41" t="inlineStr"/>
-      <c r="J6" s="41" t="inlineStr"/>
-      <c r="K6" s="41" t="inlineStr"/>
+          <t>Referral received</t>
+        </is>
+      </c>
+      <c r="H6" s="41" t="inlineStr">
+        <is>
+          <t>Mary-Margaret Fincher</t>
+        </is>
+      </c>
+      <c r="I6" s="41" t="inlineStr">
+        <is>
+          <t>6-8 Science</t>
+        </is>
+      </c>
+      <c r="J6" s="41" t="inlineStr">
+        <is>
+          <t>mfincher@avchristianschool.org (cell 949-610-4586)</t>
+        </is>
+      </c>
+      <c r="K6" s="41" t="inlineStr">
+        <is>
+          <t>Sent to Kim 10/29</t>
+        </is>
+      </c>
       <c r="L6" s="41" t="inlineStr">
         <is>
           <t>Interviewed 9/24. Active Learning referral ask emailed 10/27.</t>
@@ -59105,29 +59121,13 @@
       </c>
       <c r="G7" s="41" t="inlineStr">
         <is>
-          <t>Referral received</t>
-        </is>
-      </c>
-      <c r="H7" s="41" t="inlineStr">
-        <is>
-          <t>Mary-Margaret Fincher</t>
-        </is>
-      </c>
-      <c r="I7" s="41" t="inlineStr">
-        <is>
-          <t>6-8 Science</t>
-        </is>
-      </c>
-      <c r="J7" s="41" t="inlineStr">
-        <is>
-          <t>mfincher@avchristianschool.org (cell 949-610-4586)</t>
-        </is>
-      </c>
-      <c r="K7" s="41" t="inlineStr">
-        <is>
-          <t>Drafted to Kim 10/29 (pending send)</t>
-        </is>
-      </c>
+          <t>Active Learning ask emailed 10/27</t>
+        </is>
+      </c>
+      <c r="H7" s="41" t="inlineStr"/>
+      <c r="I7" s="41" t="inlineStr"/>
+      <c r="J7" s="41" t="inlineStr"/>
+      <c r="K7" s="41" t="inlineStr"/>
       <c r="L7" s="41" t="inlineStr">
         <is>
           <t>Interviewed 9/30. Active Learning referral ask emailed 10/27.</t>
@@ -59233,7 +59233,7 @@
       </c>
       <c r="K9" s="41" t="inlineStr">
         <is>
-          <t>Drafted to Kim 10/29 (pending send)</t>
+          <t>Sent to Kim 10/29</t>
         </is>
       </c>
       <c r="L9" s="41" t="inlineStr">
@@ -59367,13 +59367,29 @@
       </c>
       <c r="G12" s="41" t="inlineStr">
         <is>
-          <t>Active Learning ask emailed 10/27</t>
-        </is>
-      </c>
-      <c r="H12" s="41" t="inlineStr"/>
-      <c r="I12" s="41" t="inlineStr"/>
-      <c r="J12" s="41" t="inlineStr"/>
-      <c r="K12" s="41" t="inlineStr"/>
+          <t>Referral received</t>
+        </is>
+      </c>
+      <c r="H12" s="41" t="inlineStr">
+        <is>
+          <t>Christine Valverde</t>
+        </is>
+      </c>
+      <c r="I12" s="41" t="inlineStr">
+        <is>
+          <t>7th grade Bible</t>
+        </is>
+      </c>
+      <c r="J12" s="41" t="inlineStr">
+        <is>
+          <t>cvalverde@dayspringchristian.com</t>
+        </is>
+      </c>
+      <c r="K12" s="41" t="inlineStr">
+        <is>
+          <t>In new draft to Kim 10/29 (holding for evening)</t>
+        </is>
+      </c>
       <c r="L12" s="41" t="inlineStr">
         <is>
           <t>Interviewed 10/6. Active Learning referral ask emailed 10/27.</t>

</xml_diff>

<commit_message>
Active Learning: log Wendy Wagoner reply (self-candidate, no referral yet)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BUC7AKNsC5W1a963Yi5JKY
</commit_message>
<xml_diff>
--- a/outreach/DeepRoots_Interview_QA.xlsx
+++ b/outreach/DeepRoots_Interview_QA.xlsx
@@ -59167,7 +59167,7 @@
       </c>
       <c r="G8" s="41" t="inlineStr">
         <is>
-          <t>Active Learning ask emailed 10/27</t>
+          <t>Reply received - no name yet</t>
         </is>
       </c>
       <c r="H8" s="41" t="inlineStr"/>
@@ -59176,7 +59176,7 @@
       <c r="K8" s="41" t="inlineStr"/>
       <c r="L8" s="41" t="inlineStr">
         <is>
-          <t>Interviewed 10/2. Active Learning referral ask emailed 10/27.</t>
+          <t>Interviewed 10/2. Active Learning ask emailed 10/27. Reply 10/29: open to helping herself (prior curriculum work for Standard Publishing); wants a call to discuss scope/timeline; also offered to think of and ask other candidates.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Read Me: add orientation note for Nancy's team (live doc, how to contribute, current tab list)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BUC7AKNsC5W1a963Yi5JKY
</commit_message>
<xml_diff>
--- a/outreach/DeepRoots_Interview_QA.xlsx
+++ b/outreach/DeepRoots_Interview_QA.xlsx
@@ -832,7 +832,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A21"/>
+  <dimension ref="A1:A34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -970,6 +970,86 @@
       <c r="A21" s="10" t="inlineStr">
         <is>
           <t>Horizon Christian (OR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="59" t="inlineStr">
+        <is>
+          <t>Note for Nancy's team (added 10/30/2026):</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>This is a LIVE Google Sheet - it updates in real time, so anything you or we add shows up for everyone automatically. No need to re-share or send new versions. About 4 more interviews are scheduled next week; each will get its own tab here as it happens.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Adding your notes: open the tab for an interview you ran or sat in on and fill the Question -&gt; Answer column, then add your takeaway in the attendees/takeaways block at the bottom. The All Interviews tab shows every answer side by side for comparison.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="59" t="inlineStr">
+        <is>
+          <t>Current tabs:</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>- All Interviews - every question with each interviewee's answer side by side (color-coded by person).</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>- Individual interview tabs - Meredith Arldt, Will Weaver, Wendy Wagoner, Ironbridge (Nicole + Crystal), Dayspring (Donna + Angela).</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>- Feedback tabs (schools already using DeepRoots) - Atlantic Shores (VA), Horizon Christian (OR), Capistrano Valley (CA), Oaks Christian (CA), Genesis Prep (ID).</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>- Josiah Gosyne (FL) - Call Notes - single market-research call.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>- Tradeshow Responses - short survey answers mapped to our question numbers; grows as more come in.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>- Research 23-24 (7th) and (8th) - our Dec 2023 school research (~329 schools) with a 'Current Outreach?' flag linking to current interviewees / Round 3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>- Working/admin tabs - Consulting Gift List (interviewee thank-you shipping), Round 3 (non-responder outreach), Active Learning Referrals (teacher scouting for Kim). Questions? Ask Troy or Pat.</t>
         </is>
       </c>
     </row>

</xml_diff>